<commit_message>
Refresh registry review for August 25
</commit_message>
<xml_diff>
--- a/public-data/rwe-mcp-verified-capability-cards.xlsx
+++ b/public-data/rwe-mcp-verified-capability-cards.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verified RWE Capability Cards" sheetId="1" r:id="R1f3659dd7c794c95"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verified RWE Capability Cards" sheetId="1" r:id="R2034f56d8a934116"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -406,7 +406,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="5" t="str">
-        <x:v>Source-reviewed catalogue for RWE workflows · identity and static documentation review only · no installation, runtime, security, privacy, clinical, methodological, or regulatory validation · CC BY 4.0 · reviewed 2026-08-11</x:v>
+        <x:v>Source-reviewed catalogue for RWE workflows · identity and static documentation review only · no installation, runtime, security, privacy, clinical, methodological, or regulatory validation · CC BY 4.0 · reviewed 2026-08-25</x:v>
       </x:c>
       <x:c r="B2" s="5"/>
       <x:c r="C2" s="5"/>
@@ -539,7 +539,7 @@
         <x:v>Capabilities are attributed to the clinical-biostatistics component, not the entire collection. Generated code and method choices require independent review.</x:v>
       </x:c>
       <x:c r="J5" s="12" t="str">
-        <x:v>Static documentation reviewed.</x:v>
+        <x:v>Static documentation reviewed · repository archived.</x:v>
       </x:c>
       <x:c r="K5" s="12" t="str">
         <x:v>Canonical public source resolved: https://github.com/GPTomics/bioSkills</x:v>
@@ -569,13 +569,13 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T5" s="13" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U5" s="13" t="n">
-        <x:v>46228</x:v>
+        <x:v>46249</x:v>
       </x:c>
       <x:c r="V5" s="15" t="n">
-        <x:v>1157</x:v>
+        <x:v>1193</x:v>
       </x:c>
       <x:c r="W5" s="12" t="str">
         <x:v>https://github.com/GPTomics/bioSkills</x:v>
@@ -646,7 +646,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T6" s="14" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U6" s="14" t="n">
         <x:v>46200</x:v>
@@ -723,13 +723,13 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T7" s="13" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U7" s="13" t="n">
         <x:v>46227</x:v>
       </x:c>
       <x:c r="V7" s="15" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="W7" s="12" t="str">
         <x:v>https://github.com/MCPServings/paper-mcp</x:v>
@@ -800,7 +800,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T8" s="14" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U8" s="14" t="n">
         <x:v>45918</x:v>
@@ -877,7 +877,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T9" s="13" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U9" s="13" t="n">
         <x:v>45918</x:v>
@@ -954,7 +954,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T10" s="14" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U10" s="14" t="n">
         <x:v>46192</x:v>
@@ -1031,7 +1031,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T11" s="13" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U11" s="13" t="n">
         <x:v>46133</x:v>
@@ -1108,7 +1108,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T12" s="14" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U12" s="14" t="n">
         <x:v>46048</x:v>
@@ -1185,7 +1185,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T13" s="13" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U13" s="13" t="n">
         <x:v>46153</x:v>
@@ -1262,10 +1262,10 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T14" s="14" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U14" s="14" t="n">
-        <x:v>46244</x:v>
+        <x:v>46256</x:v>
       </x:c>
       <x:c r="V14" s="16" t="n">
         <x:v>6</x:v>
@@ -1339,13 +1339,13 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T15" s="13" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U15" s="13" t="n">
-        <x:v>46243</x:v>
+        <x:v>46251</x:v>
       </x:c>
       <x:c r="V15" s="15" t="n">
-        <x:v>65</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="W15" s="12" t="str">
         <x:v>https://github.com/dermatologist/pyomop</x:v>
@@ -1416,7 +1416,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T16" s="14" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U16" s="14" t="n">
         <x:v>46204</x:v>
@@ -1493,7 +1493,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T17" s="13" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U17" s="13" t="n">
         <x:v>46205</x:v>
@@ -1570,7 +1570,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T18" s="14" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U18" s="14" t="n">
         <x:v>46227</x:v>
@@ -1647,7 +1647,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T19" s="13" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U19" s="13" t="n">
         <x:v>46188</x:v>
@@ -1724,7 +1724,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T20" s="14" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U20" s="14" t="n">
         <x:v>46166</x:v>
@@ -1801,10 +1801,10 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T21" s="13" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U21" s="13" t="n">
-        <x:v>46231</x:v>
+        <x:v>46251</x:v>
       </x:c>
       <x:c r="V21" s="15" t="n">
         <x:v>5</x:v>
@@ -1878,7 +1878,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T22" s="14" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U22" s="14" t="n">
         <x:v>46081</x:v>
@@ -1955,7 +1955,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T23" s="13" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U23" s="13" t="n">
         <x:v>46223</x:v>
@@ -2032,10 +2032,10 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T24" s="14" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U24" s="14" t="n">
-        <x:v>46224</x:v>
+        <x:v>46257</x:v>
       </x:c>
       <x:c r="V24" s="16" t="n">
         <x:v>0</x:v>
@@ -2109,13 +2109,13 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T25" s="13" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U25" s="13" t="n">
-        <x:v>46245</x:v>
+        <x:v>46260</x:v>
       </x:c>
       <x:c r="V25" s="15" t="n">
-        <x:v>9585</x:v>
+        <x:v>9637</x:v>
       </x:c>
       <x:c r="W25" s="12" t="str">
         <x:v>https://github.com/awslabs/mcp/tree/main/src/healthlake-mcp-server</x:v>
@@ -2186,10 +2186,10 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T26" s="14" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U26" s="14" t="n">
-        <x:v>46240</x:v>
+        <x:v>46252</x:v>
       </x:c>
       <x:c r="V26" s="16" t="n">
         <x:v>10</x:v>
@@ -2263,13 +2263,13 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T27" s="13" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U27" s="13" t="n">
         <x:v>45884</x:v>
       </x:c>
       <x:c r="V27" s="15" t="n">
-        <x:v>84</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="W27" s="12" t="str">
         <x:v>https://github.com/jmandel/health-record-mcp</x:v>
@@ -2340,13 +2340,13 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T28" s="14" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U28" s="14" t="n">
-        <x:v>46244</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="V28" s="16" t="n">
-        <x:v>8</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="W28" s="11" t="str">
         <x:v>https://github.com/SidneyBissoli/medical-terminologies-mcp</x:v>
@@ -2417,7 +2417,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T29" s="13" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U29" s="13" t="n">
         <x:v>46237</x:v>
@@ -2494,7 +2494,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T30" s="14" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U30" s="14" t="n">
         <x:v>45854</x:v>
@@ -2571,13 +2571,13 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T31" s="13" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U31" s="13" t="n">
-        <x:v>46245</x:v>
+        <x:v>46258</x:v>
       </x:c>
       <x:c r="V31" s="15" t="n">
-        <x:v>297</x:v>
+        <x:v>300</x:v>
       </x:c>
       <x:c r="W31" s="12" t="str">
         <x:v>https://github.com/brycewang-stanford/StatsPAI</x:v>
@@ -2648,7 +2648,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T32" s="14" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U32" s="14" t="n">
         <x:v>45881</x:v>
@@ -2725,7 +2725,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T33" s="13" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U33" s="13" t="n">
         <x:v>46096</x:v>
@@ -2802,7 +2802,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T34" s="14" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U34" s="14" t="n">
         <x:v>45830</x:v>
@@ -2879,7 +2879,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T35" s="13" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U35" s="13" t="n">
         <x:v>46187</x:v>
@@ -2956,7 +2956,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T36" s="14" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U36" s="14" t="n">
         <x:v>46049</x:v>
@@ -3033,7 +3033,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T37" s="13" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U37" s="13" t="n">
         <x:v>46091</x:v>
@@ -3110,7 +3110,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T38" s="14" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U38" s="14" t="n">
         <x:v>46114</x:v>
@@ -3187,13 +3187,13 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T39" s="13" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U39" s="13" t="n">
         <x:v>46229</x:v>
       </x:c>
       <x:c r="V39" s="15" t="n">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="W39" s="12" t="str">
         <x:v>https://github.com/JeonKH81/MediStat-Table1</x:v>
@@ -3264,13 +3264,13 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T40" s="14" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U40" s="14" t="n">
-        <x:v>46229</x:v>
+        <x:v>46255</x:v>
       </x:c>
       <x:c r="V40" s="16" t="n">
-        <x:v>87</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="W40" s="11" t="str">
         <x:v>https://github.com/cyanheads/clinicaltrialsgov-mcp-server</x:v>
@@ -3341,13 +3341,13 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T41" s="13" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U41" s="13" t="n">
         <x:v>46217</x:v>
       </x:c>
       <x:c r="V41" s="15" t="n">
-        <x:v>129</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="W41" s="12" t="str">
         <x:v>https://github.com/wso2/fhir-mcp-server</x:v>
@@ -3418,7 +3418,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T42" s="14" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U42" s="14" t="n">
         <x:v>46238</x:v>
@@ -3495,13 +3495,13 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T43" s="13" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U43" s="13" t="n">
-        <x:v>46233</x:v>
+        <x:v>46255</x:v>
       </x:c>
       <x:c r="V43" s="15" t="n">
-        <x:v>134</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="W43" s="12" t="str">
         <x:v>https://github.com/cyanheads/pubmed-mcp-server</x:v>
@@ -3572,7 +3572,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T44" s="14" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U44" s="14" t="n">
         <x:v>46164</x:v>
@@ -3649,7 +3649,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T45" s="13" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U45" s="13" t="n">
         <x:v>46241</x:v>
@@ -3726,7 +3726,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T46" s="14" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U46" s="14" t="n">
         <x:v>46239</x:v>
@@ -3803,7 +3803,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T47" s="13" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U47" s="13" t="n">
         <x:v>46232</x:v>
@@ -3880,10 +3880,10 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T48" s="14" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U48" s="14" t="n">
-        <x:v>46174</x:v>
+        <x:v>46250</x:v>
       </x:c>
       <x:c r="V48" s="16" t="n">
         <x:v>0</x:v>
@@ -3957,7 +3957,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T49" s="13" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U49" s="13" t="n">
         <x:v>46217</x:v>
@@ -4034,13 +4034,13 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T50" s="14" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U50" s="14" t="n">
-        <x:v>46245</x:v>
+        <x:v>46254</x:v>
       </x:c>
       <x:c r="V50" s="16" t="n">
-        <x:v>29</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="W50" s="11" t="str">
         <x:v>https://github.com/aks129/HealthClawGuardrails</x:v>
@@ -4111,7 +4111,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T51" s="13" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U51" s="13" t="n">
         <x:v>46193</x:v>
@@ -4188,10 +4188,10 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T52" s="14" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U52" s="14" t="n">
-        <x:v>46242</x:v>
+        <x:v>46256</x:v>
       </x:c>
       <x:c r="V52" s="16" t="n">
         <x:v>0</x:v>
@@ -4265,13 +4265,13 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T53" s="13" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U53" s="13" t="n">
         <x:v>46126</x:v>
       </x:c>
       <x:c r="V53" s="15" t="n">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="W53" s="12" t="str">
         <x:v>https://github.com/langcare/langcare-mcp-fhir</x:v>
@@ -4342,7 +4342,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T54" s="14" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U54" s="14" t="n">
         <x:v>46244</x:v>
@@ -4419,10 +4419,10 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T55" s="13" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U55" s="13" t="n">
-        <x:v>46230</x:v>
+        <x:v>46257</x:v>
       </x:c>
       <x:c r="V55" s="15" t="n">
         <x:v>4</x:v>
@@ -4496,7 +4496,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T56" s="14" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U56" s="14" t="n">
         <x:v>46238</x:v>
@@ -4573,7 +4573,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T57" s="13" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U57" s="13" t="n">
         <x:v>46238</x:v>
@@ -4650,13 +4650,13 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T58" s="14" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U58" s="14" t="n">
-        <x:v>46243</x:v>
+        <x:v>46256</x:v>
       </x:c>
       <x:c r="V58" s="16" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="W58" s="11" t="str">
         <x:v>https://github.com/cyanheads/cdc-health-mcp-server</x:v>
@@ -4727,7 +4727,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T59" s="13" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U59" s="13" t="n">
         <x:v>46025</x:v>
@@ -4804,7 +4804,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T60" s="14" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U60" s="14" t="n">
         <x:v>46216</x:v>
@@ -4881,7 +4881,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T61" s="13" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U61" s="13" t="n">
         <x:v>46194</x:v>
@@ -4958,10 +4958,10 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T62" s="14" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U62" s="14" t="n">
-        <x:v>46241</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="V62" s="16" t="n">
         <x:v>4</x:v>
@@ -5035,7 +5035,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T63" s="13" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U63" s="13" t="n">
         <x:v>46174</x:v>
@@ -5112,7 +5112,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T64" s="14" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U64" s="14" t="n">
         <x:v>46238</x:v>
@@ -5189,7 +5189,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T65" s="13" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U65" s="13" t="n">
         <x:v>46238</x:v>
@@ -5266,7 +5266,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T66" s="14" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U66" s="14" t="n">
         <x:v>46151</x:v>
@@ -5343,7 +5343,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T67" s="13" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U67" s="13" t="n">
         <x:v>46238</x:v>
@@ -5420,7 +5420,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T68" s="14" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U68" s="14" t="n">
         <x:v>46118</x:v>
@@ -5497,7 +5497,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T69" s="13" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U69" s="13" t="n">
         <x:v>46245</x:v>
@@ -5574,7 +5574,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T70" s="14" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U70" s="14" t="n">
         <x:v>46234</x:v>
@@ -5651,7 +5651,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T71" s="13" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U71" s="13" t="n">
         <x:v>46243</x:v>
@@ -5728,7 +5728,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T72" s="14" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U72" s="14" t="n">
         <x:v>46238</x:v>
@@ -5805,7 +5805,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T73" s="13" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U73" s="13" t="n">
         <x:v>46245</x:v>
@@ -5882,7 +5882,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T74" s="14" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U74" s="14" t="n">
         <x:v>46244</x:v>
@@ -5959,7 +5959,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T75" s="13" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U75" s="13" t="n">
         <x:v>46243</x:v>
@@ -6036,7 +6036,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T76" s="14" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U76" s="14" t="n">
         <x:v>46245</x:v>
@@ -6113,7 +6113,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T77" s="13" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U77" s="13" t="n">
         <x:v>46238</x:v>
@@ -6190,7 +6190,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T78" s="14" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U78" s="14" t="n">
         <x:v>46245</x:v>
@@ -6267,7 +6267,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T79" s="13" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U79" s="13" t="n">
         <x:v>46240</x:v>
@@ -6344,7 +6344,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T80" s="14" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U80" s="14" t="n">
         <x:v>46145</x:v>
@@ -6421,7 +6421,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T81" s="13" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U81" s="13" t="n">
         <x:v>46078</x:v>
@@ -6498,7 +6498,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T82" s="14" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U82" s="14" t="n">
         <x:v>46238</x:v>
@@ -6575,7 +6575,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T83" s="13" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U83" s="13" t="n">
         <x:v>46175</x:v>
@@ -6652,7 +6652,7 @@
         <x:v>See project documentation; authentication was not independently tested</x:v>
       </x:c>
       <x:c r="T84" s="14" t="n">
-        <x:v>46245</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="U84" s="14" t="n">
         <x:v>46238</x:v>
@@ -6677,7 +6677,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R369167b6f7c74a36"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ff42825c9cf4779"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Publish audited 130-entry registry release
</commit_message>
<xml_diff>
--- a/public-data/rwe-mcp-verified-capability-cards.xlsx
+++ b/public-data/rwe-mcp-verified-capability-cards.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verified RWE Capability Cards" sheetId="1" r:id="R2034f56d8a934116"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verified RWE Capability Cards" sheetId="1" r:id="Rf41ef0355b9e4062"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -75,7 +75,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="17">
+  <x:cellXfs count="18">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -113,6 +113,7 @@
     <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -121,7 +122,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ReviewedCapabilityCards" displayName="ReviewedCapabilityCards" ref="A4:Y84" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ReviewedCapabilityCards" displayName="ReviewedCapabilityCards" ref="A4:Y134" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="25">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Name"/>
@@ -377,7 +378,7 @@
   <x:sheetData>
     <x:row r="1" ht="36" customHeight="1">
       <x:c r="A1" s="2" t="str">
-        <x:v>RWE MCP Registry — 80 Reviewed Capability Cards</x:v>
+        <x:v>RWE MCP Registry — 130 Reviewed Capability Cards</x:v>
       </x:c>
       <x:c r="B1" s="2"/>
       <x:c r="C1" s="2"/>
@@ -634,7 +635,7 @@
         <x:v>MIT</x:v>
       </x:c>
       <x:c r="P6" s="11" t="str">
-        <x:v>heor-agent-mcp 1.27.0</x:v>
+        <x:v>heor-agent-mcp 1.35.0</x:v>
       </x:c>
       <x:c r="Q6" s="11" t="str">
         <x:v>See project documentation; transport was not independently tested</x:v>
@@ -1250,7 +1251,7 @@
         <x:v>MIT</x:v>
       </x:c>
       <x:c r="P14" s="11" t="str">
-        <x:v>@omophub/omophub-mcp 1.5.3</x:v>
+        <x:v>@omophub/omophub-mcp 1.6.2</x:v>
       </x:c>
       <x:c r="Q14" s="11" t="str">
         <x:v>See project documentation; transport was not independently tested</x:v>
@@ -2020,7 +2021,7 @@
         <x:v>Apache-2.0</x:v>
       </x:c>
       <x:c r="P24" s="11" t="str">
-        <x:v>target-mcp 0.1.2</x:v>
+        <x:v>target-mcp 0.2.0</x:v>
       </x:c>
       <x:c r="Q24" s="11" t="str">
         <x:v>See project documentation; transport was not independently tested</x:v>
@@ -2328,7 +2329,7 @@
         <x:v>MIT</x:v>
       </x:c>
       <x:c r="P28" s="11" t="str">
-        <x:v>medical-terminologies-mcp 1.5.0</x:v>
+        <x:v>medical-terminologies-mcp 1.8.0</x:v>
       </x:c>
       <x:c r="Q28" s="11" t="str">
         <x:v>See project documentation; transport was not independently tested</x:v>
@@ -3252,7 +3253,7 @@
         <x:v>Apache-2.0</x:v>
       </x:c>
       <x:c r="P40" s="11" t="str">
-        <x:v>clinicaltrialsgov-mcp-server 2.8.2</x:v>
+        <x:v>clinicaltrialsgov-mcp-server 2.9.2</x:v>
       </x:c>
       <x:c r="Q40" s="11" t="str">
         <x:v>See project documentation; transport was not independently tested</x:v>
@@ -3483,7 +3484,7 @@
         <x:v>Apache-2.0</x:v>
       </x:c>
       <x:c r="P43" s="12" t="str">
-        <x:v>@cyanheads/pubmed-mcp-server 2.9.8</x:v>
+        <x:v>@cyanheads/pubmed-mcp-server 2.10.4</x:v>
       </x:c>
       <x:c r="Q43" s="12" t="str">
         <x:v>See project documentation; transport was not independently tested</x:v>
@@ -3868,7 +3869,7 @@
         <x:v>MIT</x:v>
       </x:c>
       <x:c r="P48" s="11" t="str">
-        <x:v>io.ausdata/aihw-mcp 0.4.18</x:v>
+        <x:v>io.ausdata/aihw-mcp 0.4.24</x:v>
       </x:c>
       <x:c r="Q48" s="11" t="str">
         <x:v>See project documentation; transport was not independently tested</x:v>
@@ -4638,7 +4639,7 @@
         <x:v>Apache-2.0</x:v>
       </x:c>
       <x:c r="P58" s="11" t="str">
-        <x:v>io.github.cyanheads/cdc-health-mcp-server 0.8.4</x:v>
+        <x:v>io.github.cyanheads/cdc-health-mcp-server 0.8.6</x:v>
       </x:c>
       <x:c r="Q58" s="11" t="str">
         <x:v>See project documentation; transport was not independently tested</x:v>
@@ -4946,7 +4947,7 @@
         <x:v>Apache-2.0</x:v>
       </x:c>
       <x:c r="P62" s="11" t="str">
-        <x:v>io.github.cyanheads/openfda-mcp-server 0.7.3</x:v>
+        <x:v>io.github.cyanheads/openfda-mcp-server 0.7.4</x:v>
       </x:c>
       <x:c r="Q62" s="11" t="str">
         <x:v>See project documentation; transport was not independently tested</x:v>
@@ -5947,7 +5948,7 @@
         <x:v>Apache-2.0</x:v>
       </x:c>
       <x:c r="P75" s="12" t="str">
-        <x:v>io.github.cyanheads/medical-codes-mcp-server 0.2.7</x:v>
+        <x:v>io.github.cyanheads/medical-codes-mcp-server 0.2.8</x:v>
       </x:c>
       <x:c r="Q75" s="12" t="str">
         <x:v>See project documentation; transport was not independently tested</x:v>
@@ -6024,7 +6025,7 @@
         <x:v>Apache-2.0</x:v>
       </x:c>
       <x:c r="P76" s="11" t="str">
-        <x:v>io.github.mims-harvard/tooluniverse 1.4.0</x:v>
+        <x:v>io.github.mims-harvard/tooluniverse 1.4.1</x:v>
       </x:c>
       <x:c r="Q76" s="11" t="str">
         <x:v>See project documentation; transport was not independently tested</x:v>
@@ -6178,7 +6179,7 @@
         <x:v>MIT</x:v>
       </x:c>
       <x:c r="P78" s="11" t="str">
-        <x:v>io.github.rubatoyd/scienceon-mcp 0.2.0</x:v>
+        <x:v>io.github.rubatoyd/scienceon-mcp 0.5.1</x:v>
       </x:c>
       <x:c r="Q78" s="11" t="str">
         <x:v>See project documentation; transport was not independently tested</x:v>
@@ -6668,6 +6669,3856 @@
       </x:c>
       <x:c r="Y84" s="11" t="str">
         <x:v>https://github.com/pipeworx-io/mcp-europepmc#readme</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85">
+      <x:c r="A85" t="str">
+        <x:v>RWE-0212</x:v>
+      </x:c>
+      <x:c r="B85" t="str">
+        <x:v>AEHRC FHIR Tools</x:v>
+      </x:c>
+      <x:c r="C85" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D85" t="str">
+        <x:v>Clinical Data &amp; Interoperability</x:v>
+      </x:c>
+      <x:c r="E85" t="str">
+        <x:v>FHIR tools by Australian e-Health Research Centre (CSIRO) for health data interoperability.</x:v>
+      </x:c>
+      <x:c r="F85" t="str">
+        <x:v>FHIR / clinical data | Interoperability | Governed access</x:v>
+      </x:c>
+      <x:c r="G85" t="str">
+        <x:v>Clinical-source inspection | Interoperability prototyping | Cohort and data-availability assessment</x:v>
+      </x:c>
+      <x:c r="H85" t="str">
+        <x:v>fhir-tools: General FHIR utilities including | au-fhir-tools: Australian-specific FHIR tools | tx-tools: Terminology services for code lookup and</x:v>
+      </x:c>
+      <x:c r="I85" t="str">
+        <x:v>Clinical systems can contain PHI and may expose write operations. Production use requires explicit authorization, least privilege, audit logging, retention controls, source-system validation, and organization-specific governance.</x:v>
+      </x:c>
+      <x:c r="J85" t="str">
+        <x:v>Static documentation and repository metadata reviewed.</x:v>
+      </x:c>
+      <x:c r="K85" t="str">
+        <x:v>Canonical public source resolved: https://github.com/aehrc/mcp-fhir-tools</x:v>
+      </x:c>
+      <x:c r="L85" t="str">
+        <x:v>Repository README and declared capability surface statically reviewed: https://github.com/aehrc/mcp-fhir-tools/blob/main/README.md</x:v>
+      </x:c>
+      <x:c r="M85" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N85" t="str">
+        <x:v>aehrc</x:v>
+      </x:c>
+      <x:c r="O85" t="str">
+        <x:v>Apache-2.0</x:v>
+      </x:c>
+      <x:c r="P85" t="str">
+        <x:v>Source repository</x:v>
+      </x:c>
+      <x:c r="Q85" t="str">
+        <x:v>See project documentation; transport was not independently tested</x:v>
+      </x:c>
+      <x:c r="R85" t="str">
+        <x:v>See project documentation; read/write scope was not independently tested</x:v>
+      </x:c>
+      <x:c r="S85" t="str">
+        <x:v>See project documentation; authentication was not independently tested</x:v>
+      </x:c>
+      <x:c r="T85" s="17" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="U85" s="17" t="n">
+        <x:v>45957</x:v>
+      </x:c>
+      <x:c r="V85" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="W85" t="str">
+        <x:v>https://github.com/aehrc/mcp-fhir-tools</x:v>
+      </x:c>
+      <x:c r="X85" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="Y85" t="str">
+        <x:v>https://github.com/aehrc/mcp-fhir-tools/blob/main/README.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86">
+      <x:c r="A86" t="str">
+        <x:v>RWE-0213</x:v>
+      </x:c>
+      <x:c r="B86" t="str">
+        <x:v>AgentCare MCP</x:v>
+      </x:c>
+      <x:c r="C86" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D86" t="str">
+        <x:v>Clinical Data &amp; Interoperability</x:v>
+      </x:c>
+      <x:c r="E86" t="str">
+        <x:v>Healthcare tools and prompts for interacting with FHIR data and medical resources on EMRs like Cerner and Epic.</x:v>
+      </x:c>
+      <x:c r="F86" t="str">
+        <x:v>FHIR / clinical data | Interoperability | Governed access</x:v>
+      </x:c>
+      <x:c r="G86" t="str">
+        <x:v>Clinical-source inspection | Interoperability prototyping | Cohort and data-availability assessment</x:v>
+      </x:c>
+      <x:c r="H86" t="str">
+        <x:v>Search or retrieve documented clinical-data resources | Return structured resources or metadata for downstream review | Support governed interoperability and data-availability workflows</x:v>
+      </x:c>
+      <x:c r="I86" t="str">
+        <x:v>Clinical systems can contain PHI and may expose write operations. Production use requires explicit authorization, least privilege, audit logging, retention controls, source-system validation, and organization-specific governance.</x:v>
+      </x:c>
+      <x:c r="J86" t="str">
+        <x:v>Static documentation and repository metadata reviewed.</x:v>
+      </x:c>
+      <x:c r="K86" t="str">
+        <x:v>Canonical public source resolved: https://github.com/Kartha-AI/agentcare-mcp</x:v>
+      </x:c>
+      <x:c r="L86" t="str">
+        <x:v>Repository README and declared capability surface statically reviewed: https://github.com/Kartha-AI/agentcare-mcp/blob/main/README.md</x:v>
+      </x:c>
+      <x:c r="M86" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N86" t="str">
+        <x:v>Kartha-AI</x:v>
+      </x:c>
+      <x:c r="O86" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P86" t="str">
+        <x:v>Source repository</x:v>
+      </x:c>
+      <x:c r="Q86" t="str">
+        <x:v>See project documentation; transport was not independently tested</x:v>
+      </x:c>
+      <x:c r="R86" t="str">
+        <x:v>See project documentation; read/write scope was not independently tested</x:v>
+      </x:c>
+      <x:c r="S86" t="str">
+        <x:v>See project documentation; authentication was not independently tested</x:v>
+      </x:c>
+      <x:c r="T86" s="17" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="U86" s="17" t="n">
+        <x:v>46076</x:v>
+      </x:c>
+      <x:c r="V86" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="W86" t="str">
+        <x:v>https://github.com/Kartha-AI/agentcare-mcp</x:v>
+      </x:c>
+      <x:c r="X86" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="Y86" t="str">
+        <x:v>https://github.com/Kartha-AI/agentcare-mcp/blob/main/README.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87">
+      <x:c r="A87" t="str">
+        <x:v>RWE-0248</x:v>
+      </x:c>
+      <x:c r="B87" t="str">
+        <x:v>Apple Health MCP</x:v>
+      </x:c>
+      <x:c r="C87" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D87" t="str">
+        <x:v>Public Health &amp; Epidemiology</x:v>
+      </x:c>
+      <x:c r="E87" t="str">
+        <x:v>Query Apple Health data with SQL and natural language via DuckDB for consumer and population health workflows.</x:v>
+      </x:c>
+      <x:c r="F87" t="str">
+        <x:v>Apple Health | Patient-generated data | DuckDB</x:v>
+      </x:c>
+      <x:c r="G87" t="str">
+        <x:v>Population-health surveillance | Burden and trend description | External context for RWE studies</x:v>
+      </x:c>
+      <x:c r="H87" t="str">
+        <x:v>An Apple Health CSV export created with | Only the Simple Health Export CSV layout is supported. | Search documented population-health indicators</x:v>
+      </x:c>
+      <x:c r="I87" t="str">
+        <x:v>Reporting delay, suppression, revisions, changing definitions, geographic comparability, and ecological inference can affect interpretation. Results require dataset-specific denominator and provenance checks.</x:v>
+      </x:c>
+      <x:c r="J87" t="str">
+        <x:v>Static documentation and repository metadata reviewed.</x:v>
+      </x:c>
+      <x:c r="K87" t="str">
+        <x:v>Canonical public source resolved: https://github.com/neiltron/apple-health-mcp</x:v>
+      </x:c>
+      <x:c r="L87" t="str">
+        <x:v>Repository README and declared capability surface statically reviewed: https://github.com/neiltron/apple-health-mcp/blob/main/README.md</x:v>
+      </x:c>
+      <x:c r="M87" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N87" t="str">
+        <x:v>neiltron</x:v>
+      </x:c>
+      <x:c r="O87" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P87" t="str">
+        <x:v>Source repository</x:v>
+      </x:c>
+      <x:c r="Q87" t="str">
+        <x:v>See project documentation; transport was not independently tested</x:v>
+      </x:c>
+      <x:c r="R87" t="str">
+        <x:v>See project documentation; read/write scope was not independently tested</x:v>
+      </x:c>
+      <x:c r="S87" t="str">
+        <x:v>See project documentation; authentication was not independently tested</x:v>
+      </x:c>
+      <x:c r="T87" s="17" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="U87" s="17" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="V87" t="n">
+        <x:v>563</x:v>
+      </x:c>
+      <x:c r="W87" t="str">
+        <x:v>https://github.com/neiltron/apple-health-mcp</x:v>
+      </x:c>
+      <x:c r="X87" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="Y87" t="str">
+        <x:v>https://github.com/neiltron/apple-health-mcp/blob/main/README.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88">
+      <x:c r="A88" t="str">
+        <x:v>RWE-0215</x:v>
+      </x:c>
+      <x:c r="B88" t="str">
+        <x:v>Azure FHIR MCP Server</x:v>
+      </x:c>
+      <x:c r="C88" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D88" t="str">
+        <x:v>Clinical Data &amp; Interoperability</x:v>
+      </x:c>
+      <x:c r="E88" t="str">
+        <x:v>Azure Health Data Services FHIR MCP server for cloud-native health data integration.</x:v>
+      </x:c>
+      <x:c r="F88" t="str">
+        <x:v>FHIR / clinical data | Interoperability | Governed access</x:v>
+      </x:c>
+      <x:c r="G88" t="str">
+        <x:v>Clinical-source inspection | Interoperability prototyping | Cohort and data-availability assessment</x:v>
+      </x:c>
+      <x:c r="H88" t="str">
+        <x:v>searchfhir - Search for FHIR resources based on a dictionary of search parameters | fhir://Patient/ - Access all Patient resources | fhir://Patient/{id} - Access a specific Patient resource</x:v>
+      </x:c>
+      <x:c r="I88" t="str">
+        <x:v>Clinical systems can contain PHI and may expose write operations. Production use requires explicit authorization, least privilege, audit logging, retention controls, source-system validation, and organization-specific governance.</x:v>
+      </x:c>
+      <x:c r="J88" t="str">
+        <x:v>Static documentation and repository metadata reviewed.</x:v>
+      </x:c>
+      <x:c r="K88" t="str">
+        <x:v>Canonical public source resolved: https://github.com/erikhoward/azure-fhir-mcp-server</x:v>
+      </x:c>
+      <x:c r="L88" t="str">
+        <x:v>Repository README and declared capability surface statically reviewed: https://github.com/erikhoward/azure-fhir-mcp-server/blob/main/README.md</x:v>
+      </x:c>
+      <x:c r="M88" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N88" t="str">
+        <x:v>erikhoward</x:v>
+      </x:c>
+      <x:c r="O88" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P88" t="str">
+        <x:v>Source repository</x:v>
+      </x:c>
+      <x:c r="Q88" t="str">
+        <x:v>See project documentation; transport was not independently tested</x:v>
+      </x:c>
+      <x:c r="R88" t="str">
+        <x:v>See project documentation; read/write scope was not independently tested</x:v>
+      </x:c>
+      <x:c r="S88" t="str">
+        <x:v>See project documentation; authentication was not independently tested</x:v>
+      </x:c>
+      <x:c r="T88" s="17" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="U88" s="17" t="n">
+        <x:v>45940</x:v>
+      </x:c>
+      <x:c r="V88" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="W88" t="str">
+        <x:v>https://github.com/erikhoward/azure-fhir-mcp-server</x:v>
+      </x:c>
+      <x:c r="X88" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="Y88" t="str">
+        <x:v>https://github.com/erikhoward/azure-fhir-mcp-server/blob/main/README.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89">
+      <x:c r="A89" t="str">
+        <x:v>RWE-0230</x:v>
+      </x:c>
+      <x:c r="B89" t="str">
+        <x:v>BioMCP</x:v>
+      </x:c>
+      <x:c r="C89" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D89" t="str">
+        <x:v>Literature &amp; Evidence Synthesis</x:v>
+      </x:c>
+      <x:c r="E89" t="str">
+        <x:v>Clinical trials, genomics, PubMed, and variant annotation in Rust for biomedical research workflows.</x:v>
+      </x:c>
+      <x:c r="F89" t="str">
+        <x:v>Evidence retrieval | Literature search | Source verification</x:v>
+      </x:c>
+      <x:c r="G89" t="str">
+        <x:v>Literature discovery | Evidence scoping | Citation and source retrieval</x:v>
+      </x:c>
+      <x:c r="H89" t="str">
+        <x:v>Search the literature: search article fans out across PubTator3 and | Pivot without rework: move from a gene, variant, drug, disease, pathway, | Analyze studies locally: study commands cover local query, cohort, survival,</x:v>
+      </x:c>
+      <x:c r="I89" t="str">
+        <x:v>Provider coverage, indexing delay, query translation, deduplication, full-text rights, and citation accuracy vary. Reproducible reviews still require logged searches, dates, screening decisions, evidence grading, and primary-source verification.</x:v>
+      </x:c>
+      <x:c r="J89" t="str">
+        <x:v>Static documentation and repository metadata reviewed.</x:v>
+      </x:c>
+      <x:c r="K89" t="str">
+        <x:v>Canonical public source resolved: https://github.com/genomoncology/biomcp</x:v>
+      </x:c>
+      <x:c r="L89" t="str">
+        <x:v>Repository README and declared capability surface statically reviewed: https://github.com/genomoncology/biomcp/blob/main/README.md</x:v>
+      </x:c>
+      <x:c r="M89" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N89" t="str">
+        <x:v>genomoncology</x:v>
+      </x:c>
+      <x:c r="O89" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P89" t="str">
+        <x:v>Source repository</x:v>
+      </x:c>
+      <x:c r="Q89" t="str">
+        <x:v>See project documentation; transport was not independently tested</x:v>
+      </x:c>
+      <x:c r="R89" t="str">
+        <x:v>See project documentation; read/write scope was not independently tested</x:v>
+      </x:c>
+      <x:c r="S89" t="str">
+        <x:v>See project documentation; authentication was not independently tested</x:v>
+      </x:c>
+      <x:c r="T89" s="17" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="U89" s="17" t="n">
+        <x:v>46260</x:v>
+      </x:c>
+      <x:c r="V89" t="n">
+        <x:v>607</x:v>
+      </x:c>
+      <x:c r="W89" t="str">
+        <x:v>https://github.com/genomoncology/biomcp</x:v>
+      </x:c>
+      <x:c r="X89" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="Y89" t="str">
+        <x:v>https://github.com/genomoncology/biomcp/blob/main/README.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90">
+      <x:c r="A90" t="str">
+        <x:v>RWE-0231</x:v>
+      </x:c>
+      <x:c r="B90" t="str">
+        <x:v>BioPortal MCP</x:v>
+      </x:c>
+      <x:c r="C90" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D90" t="str">
+        <x:v>OMOP &amp; terminology</x:v>
+      </x:c>
+      <x:c r="E90" t="str">
+        <x:v>Search and retrieve ontology terms across the NCBO BioPortal library of 1,000+ biomedical ontologies for terminology mapping and annotation.</x:v>
+      </x:c>
+      <x:c r="F90" t="str">
+        <x:v>Terminology | Code lookup | Normalization</x:v>
+      </x:c>
+      <x:c r="G90" t="str">
+        <x:v>Concept-set development | Code validation | Data harmonization</x:v>
+      </x:c>
+      <x:c r="H90" t="str">
+        <x:v>Search ontology terms: Search across BioPortal's extensive collection of biomedical ontologies | Search ontology properties: Find object properties, annotation properties, and datatype properties | Get ontology analytics: Access visitor statistics and usage analytics for ontologies</x:v>
+      </x:c>
+      <x:c r="I90" t="str">
+        <x:v>Automated code lookup or mapping can omit descendants, include inappropriate concepts, or obscure local meaning. Vocabulary versions, licensing, hierarchy behavior, and study-specific concept sets require expert adjudication.</x:v>
+      </x:c>
+      <x:c r="J90" t="str">
+        <x:v>Static documentation and repository metadata reviewed.</x:v>
+      </x:c>
+      <x:c r="K90" t="str">
+        <x:v>Canonical public source resolved: https://github.com/ncbo/bioportal-mcp</x:v>
+      </x:c>
+      <x:c r="L90" t="str">
+        <x:v>Repository README and declared capability surface statically reviewed: https://github.com/ncbo/bioportal-mcp/blob/main/README.md</x:v>
+      </x:c>
+      <x:c r="M90" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N90" t="str">
+        <x:v>ncbo</x:v>
+      </x:c>
+      <x:c r="O90" t="str">
+        <x:v>Not declared</x:v>
+      </x:c>
+      <x:c r="P90" t="str">
+        <x:v>Source repository</x:v>
+      </x:c>
+      <x:c r="Q90" t="str">
+        <x:v>See project documentation; transport was not independently tested</x:v>
+      </x:c>
+      <x:c r="R90" t="str">
+        <x:v>See project documentation; read/write scope was not independently tested</x:v>
+      </x:c>
+      <x:c r="S90" t="str">
+        <x:v>See project documentation; authentication was not independently tested</x:v>
+      </x:c>
+      <x:c r="T90" s="17" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="U90" s="17" t="n">
+        <x:v>45992</x:v>
+      </x:c>
+      <x:c r="V90" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="W90" t="str">
+        <x:v>https://github.com/ncbo/bioportal-mcp</x:v>
+      </x:c>
+      <x:c r="X90" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="Y90" t="str">
+        <x:v>https://github.com/ncbo/bioportal-mcp/blob/main/README.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91">
+      <x:c r="A91" t="str">
+        <x:v>RWE-0232</x:v>
+      </x:c>
+      <x:c r="B91" t="str">
+        <x:v>bioRxiv MCP</x:v>
+      </x:c>
+      <x:c r="C91" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D91" t="str">
+        <x:v>Literature &amp; Evidence Synthesis</x:v>
+      </x:c>
+      <x:c r="E91" t="str">
+        <x:v>bioRxiv and medRxiv preprint search, recent listings, and published-version crosswalks.</x:v>
+      </x:c>
+      <x:c r="F91" t="str">
+        <x:v>Evidence retrieval | Literature search | Source verification</x:v>
+      </x:c>
+      <x:c r="G91" t="str">
+        <x:v>Literature discovery | Evidence scoping | Citation and source retrieval</x:v>
+      </x:c>
+      <x:c r="H91" t="str">
+        <x:v>Optional author maps to an EuropePMC AUTH:"…" field query, ANDed with the keyword query — supply query, author, or both | Resolves the latest version via the details API first, for the URL version and clean not-found handling | No API call — hardcoded static list (~30 bioRxiv + ~50 medRxiv categories)</x:v>
+      </x:c>
+      <x:c r="I91" t="str">
+        <x:v>Provider coverage, indexing delay, query translation, deduplication, full-text rights, and citation accuracy vary. Reproducible reviews still require logged searches, dates, screening decisions, evidence grading, and primary-source verification.</x:v>
+      </x:c>
+      <x:c r="J91" t="str">
+        <x:v>Static documentation and repository metadata reviewed.</x:v>
+      </x:c>
+      <x:c r="K91" t="str">
+        <x:v>Canonical public source resolved: https://github.com/cyanheads/biorxiv-mcp-server</x:v>
+      </x:c>
+      <x:c r="L91" t="str">
+        <x:v>Repository README and declared capability surface statically reviewed: https://github.com/cyanheads/biorxiv-mcp-server/blob/main/README.md</x:v>
+      </x:c>
+      <x:c r="M91" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N91" t="str">
+        <x:v>cyanheads</x:v>
+      </x:c>
+      <x:c r="O91" t="str">
+        <x:v>Not declared</x:v>
+      </x:c>
+      <x:c r="P91" t="str">
+        <x:v>Source repository</x:v>
+      </x:c>
+      <x:c r="Q91" t="str">
+        <x:v>See project documentation; transport was not independently tested</x:v>
+      </x:c>
+      <x:c r="R91" t="str">
+        <x:v>See project documentation; read/write scope was not independently tested</x:v>
+      </x:c>
+      <x:c r="S91" t="str">
+        <x:v>See project documentation; authentication was not independently tested</x:v>
+      </x:c>
+      <x:c r="T91" s="17" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="U91" s="17" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="V91" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="W91" t="str">
+        <x:v>https://github.com/cyanheads/biorxiv-mcp-server</x:v>
+      </x:c>
+      <x:c r="X91" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="Y91" t="str">
+        <x:v>https://github.com/cyanheads/biorxiv-mcp-server/blob/main/README.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92">
+      <x:c r="A92" t="str">
+        <x:v>RWE-0189</x:v>
+      </x:c>
+      <x:c r="B92" t="str">
+        <x:v>BioThings MCP</x:v>
+      </x:c>
+      <x:c r="C92" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D92" t="str">
+        <x:v>Biomedical &amp; RWE Infrastructure</x:v>
+      </x:c>
+      <x:c r="E92" t="str">
+        <x:v>Query genes, genetic variants, drugs, and taxonomic information via the BioThings API.</x:v>
+      </x:c>
+      <x:c r="F92" t="str">
+        <x:v>Biomedical data | Research infrastructure | Identifier resolution</x:v>
+      </x:c>
+      <x:c r="G92" t="str">
+        <x:v>Biomedical evidence enrichment | Identifier and dataset discovery | Translational context for RWE</x:v>
+      </x:c>
+      <x:c r="H92" t="str">
+        <x:v>mygene.info — Gene annotation and query service | myvariant.info — Variant annotation and query service | mychem.info — Chemical compound annotation and query service</x:v>
+      </x:c>
+      <x:c r="I92" t="str">
+        <x:v>Biomedical, personal-health, or translational evidence does not by itself establish clinical effectiveness or causal validity. Source versions, identifiers, coverage, consent, licensing, and cross-database consistency require verification.</x:v>
+      </x:c>
+      <x:c r="J92" t="str">
+        <x:v>Static documentation and repository metadata reviewed.</x:v>
+      </x:c>
+      <x:c r="K92" t="str">
+        <x:v>Canonical public source resolved: https://github.com/longevity-genie/biothings-mcp</x:v>
+      </x:c>
+      <x:c r="L92" t="str">
+        <x:v>Repository README and declared capability surface statically reviewed: https://github.com/longevity-genie/biothings-mcp/blob/main/README.md</x:v>
+      </x:c>
+      <x:c r="M92" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N92" t="str">
+        <x:v>longevity-genie</x:v>
+      </x:c>
+      <x:c r="O92" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P92" t="str">
+        <x:v>Source repository</x:v>
+      </x:c>
+      <x:c r="Q92" t="str">
+        <x:v>See project documentation; transport was not independently tested</x:v>
+      </x:c>
+      <x:c r="R92" t="str">
+        <x:v>See project documentation; read/write scope was not independently tested</x:v>
+      </x:c>
+      <x:c r="S92" t="str">
+        <x:v>See project documentation; authentication was not independently tested</x:v>
+      </x:c>
+      <x:c r="T92" s="17" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="U92" s="17" t="n">
+        <x:v>45964</x:v>
+      </x:c>
+      <x:c r="V92" t="n">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="W92" t="str">
+        <x:v>https://github.com/longevity-genie/biothings-mcp</x:v>
+      </x:c>
+      <x:c r="X92" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="Y92" t="str">
+        <x:v>https://github.com/longevity-genie/biothings-mcp/blob/main/README.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93">
+      <x:c r="A93" t="str">
+        <x:v>RWE-0217</x:v>
+      </x:c>
+      <x:c r="B93" t="str">
+        <x:v>DICOM MCP Server</x:v>
+      </x:c>
+      <x:c r="C93" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D93" t="str">
+        <x:v>Clinical Data &amp; Interoperability</x:v>
+      </x:c>
+      <x:c r="E93" t="str">
+        <x:v>Query, read, and move medical images and reports from PACS and other DICOM-compliant systems.</x:v>
+      </x:c>
+      <x:c r="F93" t="str">
+        <x:v>FHIR / clinical data | Interoperability | Governed access</x:v>
+      </x:c>
+      <x:c r="G93" t="str">
+        <x:v>Clinical-source inspection | Interoperability prototyping | Cohort and data-availability assessment</x:v>
+      </x:c>
+      <x:c r="H93" t="str">
+        <x:v>🔍 Query Metadata: Search for patients, studies, series, and instances using various criteria. | 📄 Read DICOM Reports (PDF): Retrieve DICOM instances containing encapsulated PDFs (e.g., clinical reports) and extract the text content. | ⚙️ Utilities: Manage connections and understand query options.</x:v>
+      </x:c>
+      <x:c r="I93" t="str">
+        <x:v>Clinical systems can contain PHI and may expose write operations. Production use requires explicit authorization, least privilege, audit logging, retention controls, source-system validation, and organization-specific governance.</x:v>
+      </x:c>
+      <x:c r="J93" t="str">
+        <x:v>Static documentation and repository metadata reviewed.</x:v>
+      </x:c>
+      <x:c r="K93" t="str">
+        <x:v>Canonical public source resolved: https://github.com/ChristianHinge/dicom-mcp</x:v>
+      </x:c>
+      <x:c r="L93" t="str">
+        <x:v>Repository README and declared capability surface statically reviewed: https://github.com/ChristianHinge/dicom-mcp/blob/master/README.md</x:v>
+      </x:c>
+      <x:c r="M93" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N93" t="str">
+        <x:v>ChristianHinge</x:v>
+      </x:c>
+      <x:c r="O93" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P93" t="str">
+        <x:v>Source repository</x:v>
+      </x:c>
+      <x:c r="Q93" t="str">
+        <x:v>See project documentation; transport was not independently tested</x:v>
+      </x:c>
+      <x:c r="R93" t="str">
+        <x:v>See project documentation; read/write scope was not independently tested</x:v>
+      </x:c>
+      <x:c r="S93" t="str">
+        <x:v>See project documentation; authentication was not independently tested</x:v>
+      </x:c>
+      <x:c r="T93" s="17" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="U93" s="17" t="n">
+        <x:v>46185</x:v>
+      </x:c>
+      <x:c r="V93" t="n">
+        <x:v>99</x:v>
+      </x:c>
+      <x:c r="W93" t="str">
+        <x:v>https://github.com/ChristianHinge/dicom-mcp</x:v>
+      </x:c>
+      <x:c r="X93" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="Y93" t="str">
+        <x:v>https://github.com/ChristianHinge/dicom-mcp/blob/master/README.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94">
+      <x:c r="A94" t="str">
+        <x:v>RWE-0193</x:v>
+      </x:c>
+      <x:c r="B94" t="str">
+        <x:v>DrugBank MCP Server</x:v>
+      </x:c>
+      <x:c r="C94" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D94" t="str">
+        <x:v>Regulatory &amp; Product Data</x:v>
+      </x:c>
+      <x:c r="E94" t="str">
+        <x:v>Access 17,430+ drugs (13,166 small molecules, 4,264 biotech) with targets, enzymes, metabolic pathways, interactions, and regulatory data from the DrugBank Full Database.</x:v>
+      </x:c>
+      <x:c r="F94" t="str">
+        <x:v>Regulatory data | Product evidence | Source verification</x:v>
+      </x:c>
+      <x:c r="G94" t="str">
+        <x:v>Product and identifier resolution | Regulatory context | Evidence-source triangulation</x:v>
+      </x:c>
+      <x:c r="H94" t="str">
+        <x:v>Access to 17,430 drug records (13,166 small molecules + 4,264 biotech) | Drug names, descriptions, classifications | Drug interactions and contraindications</x:v>
+      </x:c>
+      <x:c r="I94" t="str">
+        <x:v>Regulatory and administrative records answer different questions from comparative-effectiveness studies and can change over time. Coverage, field semantics, refresh cadence, and every decision-relevant result must be checked against the authoritative source.</x:v>
+      </x:c>
+      <x:c r="J94" t="str">
+        <x:v>Static documentation and repository metadata reviewed.</x:v>
+      </x:c>
+      <x:c r="K94" t="str">
+        <x:v>Canonical public source resolved: https://github.com/openpharma-org/drugbank-mcp-server</x:v>
+      </x:c>
+      <x:c r="L94" t="str">
+        <x:v>Repository README and declared capability surface statically reviewed: https://github.com/openpharma-org/drugbank-mcp-server/blob/main/README.md</x:v>
+      </x:c>
+      <x:c r="M94" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N94" t="str">
+        <x:v>openpharma-org</x:v>
+      </x:c>
+      <x:c r="O94" t="str">
+        <x:v>Not declared</x:v>
+      </x:c>
+      <x:c r="P94" t="str">
+        <x:v>Source repository</x:v>
+      </x:c>
+      <x:c r="Q94" t="str">
+        <x:v>See project documentation; transport was not independently tested</x:v>
+      </x:c>
+      <x:c r="R94" t="str">
+        <x:v>See project documentation; read/write scope was not independently tested</x:v>
+      </x:c>
+      <x:c r="S94" t="str">
+        <x:v>See project documentation; authentication was not independently tested</x:v>
+      </x:c>
+      <x:c r="T94" s="17" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="U94" s="17" t="n">
+        <x:v>46149</x:v>
+      </x:c>
+      <x:c r="V94" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="W94" t="str">
+        <x:v>https://github.com/openpharma-org/drugbank-mcp-server</x:v>
+      </x:c>
+      <x:c r="X94" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="Y94" t="str">
+        <x:v>https://github.com/openpharma-org/drugbank-mcp-server/blob/main/README.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="95">
+      <x:c r="A95" t="str">
+        <x:v>RWE-0218</x:v>
+      </x:c>
+      <x:c r="B95" t="str">
+        <x:v>EHR-MCP</x:v>
+      </x:c>
+      <x:c r="C95" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D95" t="str">
+        <x:v>Clinical Data &amp; Interoperability</x:v>
+      </x:c>
+      <x:c r="E95" t="str">
+        <x:v>Framework-agnostic SMART-on-FHIR interoperability layer for multi-agent healthcare AI, returning typed `ClinicalContextBundle` from Epic, Cerner, and any FHIR R4 EHR.</x:v>
+      </x:c>
+      <x:c r="F95" t="str">
+        <x:v>FHIR / clinical data | Interoperability | Governed access</x:v>
+      </x:c>
+      <x:c r="G95" t="str">
+        <x:v>Clinical-source inspection | Interoperability prototyping | Cohort and data-availability assessment</x:v>
+      </x:c>
+      <x:c r="H95" t="str">
+        <x:v>Auth flow: RS384 JWT assertion → token exchange → Bearer token on all FHIR requests | Epic-compatible — aligns with Epic’s Non-Patient-Facing App registration requirements | [ ] Epic FHIR sandbox end-to-end integration test suite</x:v>
+      </x:c>
+      <x:c r="I95" t="str">
+        <x:v>Clinical systems can contain PHI and may expose write operations. Production use requires explicit authorization, least privilege, audit logging, retention controls, source-system validation, and organization-specific governance.</x:v>
+      </x:c>
+      <x:c r="J95" t="str">
+        <x:v>Static documentation and repository metadata reviewed.</x:v>
+      </x:c>
+      <x:c r="K95" t="str">
+        <x:v>Canonical public source resolved: https://github.com/jsfaulkner86/ehr-mcp</x:v>
+      </x:c>
+      <x:c r="L95" t="str">
+        <x:v>Repository README and declared capability surface statically reviewed: https://github.com/jsfaulkner86/ehr-mcp/blob/main/README.md</x:v>
+      </x:c>
+      <x:c r="M95" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N95" t="str">
+        <x:v>jsfaulkner86</x:v>
+      </x:c>
+      <x:c r="O95" t="str">
+        <x:v>Not declared</x:v>
+      </x:c>
+      <x:c r="P95" t="str">
+        <x:v>Source repository</x:v>
+      </x:c>
+      <x:c r="Q95" t="str">
+        <x:v>See project documentation; transport was not independently tested</x:v>
+      </x:c>
+      <x:c r="R95" t="str">
+        <x:v>See project documentation; read/write scope was not independently tested</x:v>
+      </x:c>
+      <x:c r="S95" t="str">
+        <x:v>See project documentation; authentication was not independently tested</x:v>
+      </x:c>
+      <x:c r="T95" s="17" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="U95" s="17" t="n">
+        <x:v>46163</x:v>
+      </x:c>
+      <x:c r="V95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="W95" t="str">
+        <x:v>https://github.com/jsfaulkner86/ehr-mcp</x:v>
+      </x:c>
+      <x:c r="X95" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="Y95" t="str">
+        <x:v>https://github.com/jsfaulkner86/ehr-mcp/blob/main/README.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="96">
+      <x:c r="A96" t="str">
+        <x:v>RWE-0233</x:v>
+      </x:c>
+      <x:c r="B96" t="str">
+        <x:v>GenePattern MCP</x:v>
+      </x:c>
+      <x:c r="C96" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D96" t="str">
+        <x:v>Biomedical &amp; RWE Infrastructure</x:v>
+      </x:c>
+      <x:c r="E96" t="str">
+        <x:v>Official GenePattern server bridging AI assistants to 200+ peer-reviewed bioinformatics modules for gene expression, single-cell, and genomic analysis.</x:v>
+      </x:c>
+      <x:c r="F96" t="str">
+        <x:v>Biomedical data | Research infrastructure | Identifier resolution</x:v>
+      </x:c>
+      <x:c r="G96" t="str">
+        <x:v>Biomedical evidence enrichment | Identifier and dataset discovery | Translational context for RWE</x:v>
+      </x:c>
+      <x:c r="H96" t="str">
+        <x:v>🧬 Search, inspect, and execute hundreds of peer-reviewed genomic analysis modules | 🔧 Want to contribute code? Fork the repo, make your changes, and open a PR. Please include tests. | Documented 2. run a bioinformatic analysis via your ai assistant capability</x:v>
+      </x:c>
+      <x:c r="I96" t="str">
+        <x:v>Biomedical, personal-health, or translational evidence does not by itself establish clinical effectiveness or causal validity. Source versions, identifiers, coverage, consent, licensing, and cross-database consistency require verification.</x:v>
+      </x:c>
+      <x:c r="J96" t="str">
+        <x:v>Static documentation and repository metadata reviewed.</x:v>
+      </x:c>
+      <x:c r="K96" t="str">
+        <x:v>Canonical public source resolved: https://github.com/genepattern/genepattern-mcp</x:v>
+      </x:c>
+      <x:c r="L96" t="str">
+        <x:v>Repository README and declared capability surface statically reviewed: https://github.com/genepattern/genepattern-mcp/blob/main/README.md</x:v>
+      </x:c>
+      <x:c r="M96" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N96" t="str">
+        <x:v>genepattern</x:v>
+      </x:c>
+      <x:c r="O96" t="str">
+        <x:v>BSD-3-Clause</x:v>
+      </x:c>
+      <x:c r="P96" t="str">
+        <x:v>Source repository</x:v>
+      </x:c>
+      <x:c r="Q96" t="str">
+        <x:v>See project documentation; transport was not independently tested</x:v>
+      </x:c>
+      <x:c r="R96" t="str">
+        <x:v>See project documentation; read/write scope was not independently tested</x:v>
+      </x:c>
+      <x:c r="S96" t="str">
+        <x:v>See project documentation; authentication was not independently tested</x:v>
+      </x:c>
+      <x:c r="T96" s="17" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="U96" s="17" t="n">
+        <x:v>46106</x:v>
+      </x:c>
+      <x:c r="V96" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="W96" t="str">
+        <x:v>https://github.com/genepattern/genepattern-mcp</x:v>
+      </x:c>
+      <x:c r="X96" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="Y96" t="str">
+        <x:v>https://github.com/genepattern/genepattern-mcp/blob/main/README.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97">
+      <x:c r="A97" t="str">
+        <x:v>RWE-0234</x:v>
+      </x:c>
+      <x:c r="B97" t="str">
+        <x:v>GenomeMCP</x:v>
+      </x:c>
+      <x:c r="C97" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D97" t="str">
+        <x:v>Biomedical &amp; RWE Infrastructure</x:v>
+      </x:c>
+      <x:c r="E97" t="str">
+        <x:v>Clinical genomics intelligence via ClinVar, gnomAD, Reactome, and NCBI-BLAST with variant interpretation and population genetics for precision medicine workflows.</x:v>
+      </x:c>
+      <x:c r="F97" t="str">
+        <x:v>Biomedical data | Research infrastructure | Identifier resolution</x:v>
+      </x:c>
+      <x:c r="G97" t="str">
+        <x:v>Biomedical evidence enrichment | Identifier and dataset discovery | Translational context for RWE</x:v>
+      </x:c>
+      <x:c r="H97" t="str">
+        <x:v>searchclinvar(term) — Query ClinVar for genes, variants, or diseases | getsupportingliterature(id) — PubMed articles linked to a variant | getpathwayinfo(gene) — Reactome biological pathways for a gene</x:v>
+      </x:c>
+      <x:c r="I97" t="str">
+        <x:v>Biomedical, personal-health, or translational evidence does not by itself establish clinical effectiveness or causal validity. Source versions, identifiers, coverage, consent, licensing, and cross-database consistency require verification.</x:v>
+      </x:c>
+      <x:c r="J97" t="str">
+        <x:v>Static documentation and repository metadata reviewed.</x:v>
+      </x:c>
+      <x:c r="K97" t="str">
+        <x:v>Canonical public source resolved: https://github.com/Eldergenix/GenomeMCP</x:v>
+      </x:c>
+      <x:c r="L97" t="str">
+        <x:v>Repository README and declared capability surface statically reviewed: https://github.com/Eldergenix/GenomeMCP/blob/main/README.md</x:v>
+      </x:c>
+      <x:c r="M97" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N97" t="str">
+        <x:v>Eldergenix</x:v>
+      </x:c>
+      <x:c r="O97" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P97" t="str">
+        <x:v>Source repository</x:v>
+      </x:c>
+      <x:c r="Q97" t="str">
+        <x:v>See project documentation; transport was not independently tested</x:v>
+      </x:c>
+      <x:c r="R97" t="str">
+        <x:v>See project documentation; read/write scope was not independently tested</x:v>
+      </x:c>
+      <x:c r="S97" t="str">
+        <x:v>See project documentation; authentication was not independently tested</x:v>
+      </x:c>
+      <x:c r="T97" s="17" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="U97" s="17" t="n">
+        <x:v>46146</x:v>
+      </x:c>
+      <x:c r="V97" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="W97" t="str">
+        <x:v>https://github.com/Eldergenix/GenomeMCP</x:v>
+      </x:c>
+      <x:c r="X97" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="Y97" t="str">
+        <x:v>https://github.com/Eldergenix/GenomeMCP/blob/main/README.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="98">
+      <x:c r="A98" t="str">
+        <x:v>RWE-0194</x:v>
+      </x:c>
+      <x:c r="B98" t="str">
+        <x:v>Health Canada DPD MCP</x:v>
+      </x:c>
+      <x:c r="C98" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D98" t="str">
+        <x:v>Regulatory &amp; Product Data</x:v>
+      </x:c>
+      <x:c r="E98" t="str">
+        <x:v>Exposes Health Canada's Drug Product Database (~47,000 approved drugs spanning human pharmaceuticals, biologics, veterinary drugs, radiopharmaceuticals, and disinfectants) as MCP tools for Canadian drug lookup.</x:v>
+      </x:c>
+      <x:c r="F98" t="str">
+        <x:v>Regulatory data | Product evidence | Source verification</x:v>
+      </x:c>
+      <x:c r="G98" t="str">
+        <x:v>Product and identifier resolution | Regulatory context | Evidence-source triangulation</x:v>
+      </x:c>
+      <x:c r="H98" t="str">
+        <x:v>Comprehensive drug product queries | "Search for drugs with the brand name Tylenol" | "What are the active ingredients in drug code 48905?"</x:v>
+      </x:c>
+      <x:c r="I98" t="str">
+        <x:v>Regulatory and administrative records answer different questions from comparative-effectiveness studies and can change over time. Coverage, field semantics, refresh cadence, and every decision-relevant result must be checked against the authoritative source.</x:v>
+      </x:c>
+      <x:c r="J98" t="str">
+        <x:v>Static documentation and repository metadata reviewed.</x:v>
+      </x:c>
+      <x:c r="K98" t="str">
+        <x:v>Canonical public source resolved: https://github.com/wkurzatz/PharmacyMCP</x:v>
+      </x:c>
+      <x:c r="L98" t="str">
+        <x:v>Repository README and declared capability surface statically reviewed: https://github.com/wkurzatz/PharmacyMCP/blob/main/README.md</x:v>
+      </x:c>
+      <x:c r="M98" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N98" t="str">
+        <x:v>wkurzatz</x:v>
+      </x:c>
+      <x:c r="O98" t="str">
+        <x:v>Not declared</x:v>
+      </x:c>
+      <x:c r="P98" t="str">
+        <x:v>Source repository</x:v>
+      </x:c>
+      <x:c r="Q98" t="str">
+        <x:v>See project documentation; transport was not independently tested</x:v>
+      </x:c>
+      <x:c r="R98" t="str">
+        <x:v>See project documentation; read/write scope was not independently tested</x:v>
+      </x:c>
+      <x:c r="S98" t="str">
+        <x:v>See project documentation; authentication was not independently tested</x:v>
+      </x:c>
+      <x:c r="T98" s="17" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="U98" s="17" t="n">
+        <x:v>46086</x:v>
+      </x:c>
+      <x:c r="V98" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="W98" t="str">
+        <x:v>https://github.com/wkurzatz/PharmacyMCP</x:v>
+      </x:c>
+      <x:c r="X98" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="Y98" t="str">
+        <x:v>https://github.com/wkurzatz/PharmacyMCP/blob/main/README.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99">
+      <x:c r="A99" t="str">
+        <x:v>RWE-0252</x:v>
+      </x:c>
+      <x:c r="B99" t="str">
+        <x:v>Health Export MCP</x:v>
+      </x:c>
+      <x:c r="C99" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D99" t="str">
+        <x:v>Biomedical &amp; RWE Infrastructure</x:v>
+      </x:c>
+      <x:c r="E99" t="str">
+        <x:v>Zero-dependency Apple Health MCP server exposing 190 HealthKit metrics as JSON to any MCP client, local-first and read-only with no developer server in the path.</x:v>
+      </x:c>
+      <x:c r="F99" t="str">
+        <x:v>HealthKit | Patient-generated data | Local-first</x:v>
+      </x:c>
+      <x:c r="G99" t="str">
+        <x:v>Biomedical evidence enrichment | Identifier and dataset discovery | Translational context for RWE</x:v>
+      </x:c>
+      <x:c r="H99" t="str">
+        <x:v>Setup: point the server at your exported data and add it to your AI client. | Read-only. The server only reads your exported data, it never touches HealthKit and never writes back. | Optional pairing. Set PAIRINGSECRET to the code the iOS app shows (Settings → Agent pairing) to gate access.</x:v>
+      </x:c>
+      <x:c r="I99" t="str">
+        <x:v>Biomedical, personal-health, or translational evidence does not by itself establish clinical effectiveness or causal validity. Source versions, identifiers, coverage, consent, licensing, and cross-database consistency require verification.</x:v>
+      </x:c>
+      <x:c r="J99" t="str">
+        <x:v>Static documentation and repository metadata reviewed.</x:v>
+      </x:c>
+      <x:c r="K99" t="str">
+        <x:v>Canonical public source resolved: https://github.com/PhilipAD/health-export-mcp</x:v>
+      </x:c>
+      <x:c r="L99" t="str">
+        <x:v>Repository README and declared capability surface statically reviewed: https://github.com/PhilipAD/health-export-mcp/blob/main/README.md</x:v>
+      </x:c>
+      <x:c r="M99" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N99" t="str">
+        <x:v>PhilipAD</x:v>
+      </x:c>
+      <x:c r="O99" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P99" t="str">
+        <x:v>Source repository</x:v>
+      </x:c>
+      <x:c r="Q99" t="str">
+        <x:v>See project documentation; transport was not independently tested</x:v>
+      </x:c>
+      <x:c r="R99" t="str">
+        <x:v>See project documentation; read/write scope was not independently tested</x:v>
+      </x:c>
+      <x:c r="S99" t="str">
+        <x:v>See project documentation; authentication was not independently tested</x:v>
+      </x:c>
+      <x:c r="T99" s="17" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="U99" s="17" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="V99" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="W99" t="str">
+        <x:v>https://github.com/PhilipAD/health-export-mcp</x:v>
+      </x:c>
+      <x:c r="X99" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="Y99" t="str">
+        <x:v>https://github.com/PhilipAD/health-export-mcp/blob/main/README.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="100">
+      <x:c r="A100" t="str">
+        <x:v>RWE-0184</x:v>
+      </x:c>
+      <x:c r="B100" t="str">
+        <x:v>Healthcare Billing Codes</x:v>
+      </x:c>
+      <x:c r="C100" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D100" t="str">
+        <x:v>OMOP &amp; terminology</x:v>
+      </x:c>
+      <x:c r="E100" t="str">
+        <x:v>CPT, ICD-10, and HCPCS billing code lookup and search for revenue cycle workflows.</x:v>
+      </x:c>
+      <x:c r="F100" t="str">
+        <x:v>Terminology | Code lookup | Normalization</x:v>
+      </x:c>
+      <x:c r="G100" t="str">
+        <x:v>Concept-set development | Code validation | Data harmonization</x:v>
+      </x:c>
+      <x:c r="H100" t="str">
+        <x:v>Lookup billing codes: Get detailed information about specific CPT, ICD-10, or HCPCS codes | Search by description: Find codes by searching keywords in descriptions | Category information: View code categories and typical reimbursement rates (where applicable)</x:v>
+      </x:c>
+      <x:c r="I100" t="str">
+        <x:v>Automated code lookup or mapping can omit descendants, include inappropriate concepts, or obscure local meaning. Vocabulary versions, licensing, hierarchy behavior, and study-specific concept sets require expert adjudication.</x:v>
+      </x:c>
+      <x:c r="J100" t="str">
+        <x:v>Static documentation and repository metadata reviewed.</x:v>
+      </x:c>
+      <x:c r="K100" t="str">
+        <x:v>Canonical public source resolved: https://github.com/contextkits/healthcare-billing-codes</x:v>
+      </x:c>
+      <x:c r="L100" t="str">
+        <x:v>Repository README and declared capability surface statically reviewed: https://github.com/contextkits/healthcare-billing-codes/blob/main/README.md</x:v>
+      </x:c>
+      <x:c r="M100" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N100" t="str">
+        <x:v>contextkits</x:v>
+      </x:c>
+      <x:c r="O100" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P100" t="str">
+        <x:v>Source repository</x:v>
+      </x:c>
+      <x:c r="Q100" t="str">
+        <x:v>See project documentation; transport was not independently tested</x:v>
+      </x:c>
+      <x:c r="R100" t="str">
+        <x:v>See project documentation; read/write scope was not independently tested</x:v>
+      </x:c>
+      <x:c r="S100" t="str">
+        <x:v>See project documentation; authentication was not independently tested</x:v>
+      </x:c>
+      <x:c r="T100" s="17" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="U100" s="17" t="n">
+        <x:v>46063</x:v>
+      </x:c>
+      <x:c r="V100" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="W100" t="str">
+        <x:v>https://github.com/contextkits/healthcare-billing-codes</x:v>
+      </x:c>
+      <x:c r="X100" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="Y100" t="str">
+        <x:v>https://github.com/contextkits/healthcare-billing-codes/blob/main/README.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="101">
+      <x:c r="A101" t="str">
+        <x:v>RWE-0195</x:v>
+      </x:c>
+      <x:c r="B101" t="str">
+        <x:v>Healthcare Data Hub</x:v>
+      </x:c>
+      <x:c r="C101" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D101" t="str">
+        <x:v>Literature &amp; Evidence Synthesis</x:v>
+      </x:c>
+      <x:c r="E101" t="str">
+        <x:v>All-in-one server for FDA drug info, PubMed, medRxiv, NCBI Bookshelf, clinical trials, ICD-10, DICOM metadata, and medical calculator.</x:v>
+      </x:c>
+      <x:c r="F101" t="str">
+        <x:v>Evidence retrieval | Literature search | Source verification</x:v>
+      </x:c>
+      <x:c r="G101" t="str">
+        <x:v>Literature discovery | Evidence scoping | Citation and source retrieval</x:v>
+      </x:c>
+      <x:c r="H101" t="str">
+        <x:v>FDA Drug Information: Search and retrieve comprehensive drug information from the FDA database (improved response parsing) | PubMed Research: Search medical literature from PubMed's database of scientific articles | Health Topics: Access evidence-based health information from Health.gov (updated to API v4)</x:v>
+      </x:c>
+      <x:c r="I101" t="str">
+        <x:v>Provider coverage, indexing delay, query translation, deduplication, full-text rights, and citation accuracy vary. Reproducible reviews still require logged searches, dates, screening decisions, evidence grading, and primary-source verification.</x:v>
+      </x:c>
+      <x:c r="J101" t="str">
+        <x:v>Static documentation and repository metadata reviewed.</x:v>
+      </x:c>
+      <x:c r="K101" t="str">
+        <x:v>Canonical public source resolved: https://github.com/Cicatriiz/healthcare-mcp-public</x:v>
+      </x:c>
+      <x:c r="L101" t="str">
+        <x:v>Repository README and declared capability surface statically reviewed: https://github.com/Cicatriiz/healthcare-mcp-public/blob/main/README.md</x:v>
+      </x:c>
+      <x:c r="M101" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N101" t="str">
+        <x:v>Cicatriiz</x:v>
+      </x:c>
+      <x:c r="O101" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P101" t="str">
+        <x:v>Source repository</x:v>
+      </x:c>
+      <x:c r="Q101" t="str">
+        <x:v>See project documentation; transport was not independently tested</x:v>
+      </x:c>
+      <x:c r="R101" t="str">
+        <x:v>See project documentation; read/write scope was not independently tested</x:v>
+      </x:c>
+      <x:c r="S101" t="str">
+        <x:v>See project documentation; authentication was not independently tested</x:v>
+      </x:c>
+      <x:c r="T101" s="17" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="U101" s="17" t="n">
+        <x:v>45885</x:v>
+      </x:c>
+      <x:c r="V101" t="n">
+        <x:v>127</x:v>
+      </x:c>
+      <x:c r="W101" t="str">
+        <x:v>https://github.com/Cicatriiz/healthcare-mcp-public</x:v>
+      </x:c>
+      <x:c r="X101" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="Y101" t="str">
+        <x:v>https://github.com/Cicatriiz/healthcare-mcp-public/blob/main/README.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="102">
+      <x:c r="A102" t="str">
+        <x:v>RWE-0253</x:v>
+      </x:c>
+      <x:c r="B102" t="str">
+        <x:v>Healthcare Data MCP</x:v>
+      </x:c>
+      <x:c r="C102" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D102" t="str">
+        <x:v>Public Health &amp; Epidemiology</x:v>
+      </x:c>
+      <x:c r="E102" t="str">
+        <x:v>Eighteen local MCP servers for US public healthcare market intelligence spanning facilities, ownership, quality metrics, claims, workforce, research, and compliance screening.</x:v>
+      </x:c>
+      <x:c r="F102" t="str">
+        <x:v>Public health | Population data | Surveillance</x:v>
+      </x:c>
+      <x:c r="G102" t="str">
+        <x:v>Population-health surveillance | Burden and trend description | External context for RWE studies</x:v>
+      </x:c>
+      <x:c r="H102" t="str">
+        <x:v>Some source APIs require keys for reliable or full access. | The MCPB Desktop Extension skeleton should be validated in Claude Desktop before broad distribution. | Search documented population-health indicators</x:v>
+      </x:c>
+      <x:c r="I102" t="str">
+        <x:v>Reporting delay, suppression, revisions, changing definitions, geographic comparability, and ecological inference can affect interpretation. Results require dataset-specific denominator and provenance checks.</x:v>
+      </x:c>
+      <x:c r="J102" t="str">
+        <x:v>Static documentation and repository metadata reviewed.</x:v>
+      </x:c>
+      <x:c r="K102" t="str">
+        <x:v>Canonical public source resolved: https://github.com/ajhcs/healthcare-data-mcp</x:v>
+      </x:c>
+      <x:c r="L102" t="str">
+        <x:v>Repository README and declared capability surface statically reviewed: https://github.com/ajhcs/healthcare-data-mcp/blob/main/README.md</x:v>
+      </x:c>
+      <x:c r="M102" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N102" t="str">
+        <x:v>ajhcs</x:v>
+      </x:c>
+      <x:c r="O102" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P102" t="str">
+        <x:v>Source repository</x:v>
+      </x:c>
+      <x:c r="Q102" t="str">
+        <x:v>See project documentation; transport was not independently tested</x:v>
+      </x:c>
+      <x:c r="R102" t="str">
+        <x:v>See project documentation; read/write scope was not independently tested</x:v>
+      </x:c>
+      <x:c r="S102" t="str">
+        <x:v>See project documentation; authentication was not independently tested</x:v>
+      </x:c>
+      <x:c r="T102" s="17" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="U102" s="17" t="n">
+        <x:v>46240</x:v>
+      </x:c>
+      <x:c r="V102" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="W102" t="str">
+        <x:v>https://github.com/ajhcs/healthcare-data-mcp</x:v>
+      </x:c>
+      <x:c r="X102" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="Y102" t="str">
+        <x:v>https://github.com/ajhcs/healthcare-data-mcp/blob/main/README.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="103">
+      <x:c r="A103" t="str">
+        <x:v>RWE-0196</x:v>
+      </x:c>
+      <x:c r="B103" t="str">
+        <x:v>ICD-10 MCP</x:v>
+      </x:c>
+      <x:c r="C103" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D103" t="str">
+        <x:v>OMOP &amp; terminology</x:v>
+      </x:c>
+      <x:c r="E103" t="str">
+        <x:v>Offline ICD-10-CM FY2026, ICD-9-CM, and ICD-10 WHO 2019 lookup with 124K codes and 102K bidirectional GEMs crosswalk mappings; FTS5 full-text search in an embedded SQLite DB with zero network calls.</x:v>
+      </x:c>
+      <x:c r="F103" t="str">
+        <x:v>Terminology | Code lookup | Normalization</x:v>
+      </x:c>
+      <x:c r="G103" t="str">
+        <x:v>Concept-set development | Code validation | Data harmonization</x:v>
+      </x:c>
+      <x:c r="H103" t="str">
+        <x:v>CROSS JOIN in FTS queries forces SQLite's query planner to use the FTS index first, avoiding full table scans on broad search terms | Bitmask flags on crosswalk entries pack approximate/no-map/combination into a single integer | WITHOUT ROWID on the crosswalk table for clustered primary key access</x:v>
+      </x:c>
+      <x:c r="I103" t="str">
+        <x:v>Automated code lookup or mapping can omit descendants, include inappropriate concepts, or obscure local meaning. Vocabulary versions, licensing, hierarchy behavior, and study-specific concept sets require expert adjudication.</x:v>
+      </x:c>
+      <x:c r="J103" t="str">
+        <x:v>Static documentation and repository metadata reviewed.</x:v>
+      </x:c>
+      <x:c r="K103" t="str">
+        <x:v>Canonical public source resolved: https://github.com/stabgan/mcp-icd10</x:v>
+      </x:c>
+      <x:c r="L103" t="str">
+        <x:v>Repository README and declared capability surface statically reviewed: https://github.com/stabgan/mcp-icd10/blob/main/README.md</x:v>
+      </x:c>
+      <x:c r="M103" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N103" t="str">
+        <x:v>stabgan</x:v>
+      </x:c>
+      <x:c r="O103" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P103" t="str">
+        <x:v>Source repository</x:v>
+      </x:c>
+      <x:c r="Q103" t="str">
+        <x:v>See project documentation; transport was not independently tested</x:v>
+      </x:c>
+      <x:c r="R103" t="str">
+        <x:v>See project documentation; read/write scope was not independently tested</x:v>
+      </x:c>
+      <x:c r="S103" t="str">
+        <x:v>See project documentation; authentication was not independently tested</x:v>
+      </x:c>
+      <x:c r="T103" s="17" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="U103" s="17" t="n">
+        <x:v>46095</x:v>
+      </x:c>
+      <x:c r="V103" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="W103" t="str">
+        <x:v>https://github.com/stabgan/mcp-icd10</x:v>
+      </x:c>
+      <x:c r="X103" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="Y103" t="str">
+        <x:v>https://github.com/stabgan/mcp-icd10/blob/main/README.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="104">
+      <x:c r="A104" t="str">
+        <x:v>RWE-0235</x:v>
+      </x:c>
+      <x:c r="B104" t="str">
+        <x:v>M3 MIMIC MCP</x:v>
+      </x:c>
+      <x:c r="C104" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D104" t="str">
+        <x:v>RWE Data &amp; Analytics</x:v>
+      </x:c>
+      <x:c r="E104" t="str">
+        <x:v>Query MIMIC-IV medical data via natural language for clinical research.</x:v>
+      </x:c>
+      <x:c r="F104" t="str">
+        <x:v>MIMIC-IV | Clinical data | Natural-language query</x:v>
+      </x:c>
+      <x:c r="G104" t="str">
+        <x:v>Clinical-data exploration | Cohort feasibility | Research query prototyping</x:v>
+      </x:c>
+      <x:c r="H104" t="str">
+        <x:v>☁️ BigQuery Support: Access full MIMIC-IV dataset on Google Cloud | "Show me patient demographics from the ICU" | m3 config claude --backend bigquery --project-id YOURPROJECTID - Quick BigQuery setup</x:v>
+      </x:c>
+      <x:c r="I104" t="str">
+        <x:v>Biomedical, personal-health, or translational evidence does not by itself establish clinical effectiveness or causal validity. Source versions, identifiers, coverage, consent, licensing, and cross-database consistency require verification.</x:v>
+      </x:c>
+      <x:c r="J104" t="str">
+        <x:v>Static documentation and repository metadata reviewed.</x:v>
+      </x:c>
+      <x:c r="K104" t="str">
+        <x:v>Canonical public source resolved: https://github.com/rafiattrach/m3</x:v>
+      </x:c>
+      <x:c r="L104" t="str">
+        <x:v>Repository README and declared capability surface statically reviewed: https://github.com/rafiattrach/m3/blob/main/README.md</x:v>
+      </x:c>
+      <x:c r="M104" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N104" t="str">
+        <x:v>rafiattrach</x:v>
+      </x:c>
+      <x:c r="O104" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P104" t="str">
+        <x:v>Source repository</x:v>
+      </x:c>
+      <x:c r="Q104" t="str">
+        <x:v>See project documentation; transport was not independently tested</x:v>
+      </x:c>
+      <x:c r="R104" t="str">
+        <x:v>See project documentation; read/write scope was not independently tested</x:v>
+      </x:c>
+      <x:c r="S104" t="str">
+        <x:v>See project documentation; authentication was not independently tested</x:v>
+      </x:c>
+      <x:c r="T104" s="17" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="U104" s="17" t="n">
+        <x:v>46134</x:v>
+      </x:c>
+      <x:c r="V104" t="n">
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="W104" t="str">
+        <x:v>https://github.com/rafiattrach/m3</x:v>
+      </x:c>
+      <x:c r="X104" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="Y104" t="str">
+        <x:v>https://github.com/rafiattrach/m3/blob/main/README.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="105">
+      <x:c r="A105" t="str">
+        <x:v>RWE-0221</x:v>
+      </x:c>
+      <x:c r="B105" t="str">
+        <x:v>MCP FHIR Patient Index</x:v>
+      </x:c>
+      <x:c r="C105" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D105" t="str">
+        <x:v>Clinical Data &amp; Interoperability</x:v>
+      </x:c>
+      <x:c r="E105" t="str">
+        <x:v>Master patient index (MPI) on Rails 8 with conformant FHIR R4 API, MCP server, and admin web UI for patient CRUD; English/US-only and dev-stage with explicit security caveats requiring credential regeneration and SOC 2 hardening before production deployment.</x:v>
+      </x:c>
+      <x:c r="F105" t="str">
+        <x:v>FHIR / clinical data | Interoperability | Governed access</x:v>
+      </x:c>
+      <x:c r="G105" t="str">
+        <x:v>Clinical-source inspection | Interoperability prototyping | Cohort and data-availability assessment</x:v>
+      </x:c>
+      <x:c r="H105" t="str">
+        <x:v>Built-in minimalistic FHIR server | Create, read, update, and destroy patients | Supports US (en-speaking) patients only (no I18n)</x:v>
+      </x:c>
+      <x:c r="I105" t="str">
+        <x:v>Clinical systems can contain PHI and may expose write operations. Production use requires explicit authorization, least privilege, audit logging, retention controls, source-system validation, and organization-specific governance.</x:v>
+      </x:c>
+      <x:c r="J105" t="str">
+        <x:v>Static documentation and repository metadata reviewed.</x:v>
+      </x:c>
+      <x:c r="K105" t="str">
+        <x:v>Canonical public source resolved: https://github.com/Shaumik-Ashraf/mcp-fhir-patient-index</x:v>
+      </x:c>
+      <x:c r="L105" t="str">
+        <x:v>Repository README and declared capability surface statically reviewed: https://github.com/Shaumik-Ashraf/mcp-fhir-patient-index/blob/main/README.md</x:v>
+      </x:c>
+      <x:c r="M105" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N105" t="str">
+        <x:v>Shaumik-Ashraf</x:v>
+      </x:c>
+      <x:c r="O105" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P105" t="str">
+        <x:v>Source repository</x:v>
+      </x:c>
+      <x:c r="Q105" t="str">
+        <x:v>See project documentation; transport was not independently tested</x:v>
+      </x:c>
+      <x:c r="R105" t="str">
+        <x:v>See project documentation; read/write scope was not independently tested</x:v>
+      </x:c>
+      <x:c r="S105" t="str">
+        <x:v>See project documentation; authentication was not independently tested</x:v>
+      </x:c>
+      <x:c r="T105" s="17" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="U105" s="17" t="n">
+        <x:v>46163</x:v>
+      </x:c>
+      <x:c r="V105" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="W105" t="str">
+        <x:v>https://github.com/Shaumik-Ashraf/mcp-fhir-patient-index</x:v>
+      </x:c>
+      <x:c r="X105" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="Y105" t="str">
+        <x:v>https://github.com/Shaumik-Ashraf/mcp-fhir-patient-index/blob/main/README.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="106">
+      <x:c r="A106" t="str">
+        <x:v>RWE-0236</x:v>
+      </x:c>
+      <x:c r="B106" t="str">
+        <x:v>MCP Simple PubMed</x:v>
+      </x:c>
+      <x:c r="C106" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D106" t="str">
+        <x:v>Literature &amp; Evidence Synthesis</x:v>
+      </x:c>
+      <x:c r="E106" t="str">
+        <x:v>Popular standalone PubMed MCP server for biomedical literature search.</x:v>
+      </x:c>
+      <x:c r="F106" t="str">
+        <x:v>Evidence retrieval | Literature search | Source verification</x:v>
+      </x:c>
+      <x:c r="G106" t="str">
+        <x:v>Literature discovery | Evidence scoping | Citation and source retrieval</x:v>
+      </x:c>
+      <x:c r="H106" t="str">
+        <x:v>Search PubMed - Search the database using keywords, MeSH terms, author names, date ranges, and Boolean operators | Get Full Text - Download full text when available (for open access articles in PubMed Central) | Access Abstracts - Retrieve article abstracts and metadata via resource URIs</x:v>
+      </x:c>
+      <x:c r="I106" t="str">
+        <x:v>Provider coverage, indexing delay, query translation, deduplication, full-text rights, and citation accuracy vary. Reproducible reviews still require logged searches, dates, screening decisions, evidence grading, and primary-source verification.</x:v>
+      </x:c>
+      <x:c r="J106" t="str">
+        <x:v>Static documentation and repository metadata reviewed.</x:v>
+      </x:c>
+      <x:c r="K106" t="str">
+        <x:v>Canonical public source resolved: https://github.com/andybrandt/mcp-simple-pubmed</x:v>
+      </x:c>
+      <x:c r="L106" t="str">
+        <x:v>Repository README and declared capability surface statically reviewed: https://github.com/andybrandt/mcp-simple-pubmed/blob/master/README.md</x:v>
+      </x:c>
+      <x:c r="M106" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N106" t="str">
+        <x:v>andybrandt</x:v>
+      </x:c>
+      <x:c r="O106" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P106" t="str">
+        <x:v>Source repository</x:v>
+      </x:c>
+      <x:c r="Q106" t="str">
+        <x:v>See project documentation; transport was not independently tested</x:v>
+      </x:c>
+      <x:c r="R106" t="str">
+        <x:v>See project documentation; read/write scope was not independently tested</x:v>
+      </x:c>
+      <x:c r="S106" t="str">
+        <x:v>See project documentation; authentication was not independently tested</x:v>
+      </x:c>
+      <x:c r="T106" s="17" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="U106" s="17" t="n">
+        <x:v>46100</x:v>
+      </x:c>
+      <x:c r="V106" t="n">
+        <x:v>171</x:v>
+      </x:c>
+      <x:c r="W106" t="str">
+        <x:v>https://github.com/andybrandt/mcp-simple-pubmed</x:v>
+      </x:c>
+      <x:c r="X106" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="Y106" t="str">
+        <x:v>https://github.com/andybrandt/mcp-simple-pubmed/blob/master/README.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="107">
+      <x:c r="A107" t="str">
+        <x:v>RWE-0199</x:v>
+      </x:c>
+      <x:c r="B107" t="str">
+        <x:v>MCP-LOINC</x:v>
+      </x:c>
+      <x:c r="C107" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D107" t="str">
+        <x:v>OMOP &amp; terminology</x:v>
+      </x:c>
+      <x:c r="E107" t="str">
+        <x:v>LOINC API wrapper for medical terminology standardization and lab code lookup.</x:v>
+      </x:c>
+      <x:c r="F107" t="str">
+        <x:v>Terminology | Code lookup | Normalization</x:v>
+      </x:c>
+      <x:c r="G107" t="str">
+        <x:v>Concept-set development | Code validation | Data harmonization</x:v>
+      </x:c>
+      <x:c r="H107" t="str">
+        <x:v>Getting LOINC API Access | LOINC Code Search | Search for LOINC codes by various terms and filters</x:v>
+      </x:c>
+      <x:c r="I107" t="str">
+        <x:v>Automated code lookup or mapping can omit descendants, include inappropriate concepts, or obscure local meaning. Vocabulary versions, licensing, hierarchy behavior, and study-specific concept sets require expert adjudication.</x:v>
+      </x:c>
+      <x:c r="J107" t="str">
+        <x:v>Static documentation and repository metadata reviewed.</x:v>
+      </x:c>
+      <x:c r="K107" t="str">
+        <x:v>Canonical public source resolved: https://github.com/Kryzo/mcp-Loinc</x:v>
+      </x:c>
+      <x:c r="L107" t="str">
+        <x:v>Repository README and declared capability surface statically reviewed: https://github.com/Kryzo/mcp-Loinc/blob/main/README.md</x:v>
+      </x:c>
+      <x:c r="M107" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N107" t="str">
+        <x:v>Kryzo</x:v>
+      </x:c>
+      <x:c r="O107" t="str">
+        <x:v>Not declared</x:v>
+      </x:c>
+      <x:c r="P107" t="str">
+        <x:v>Source repository</x:v>
+      </x:c>
+      <x:c r="Q107" t="str">
+        <x:v>See project documentation; transport was not independently tested</x:v>
+      </x:c>
+      <x:c r="R107" t="str">
+        <x:v>See project documentation; read/write scope was not independently tested</x:v>
+      </x:c>
+      <x:c r="S107" t="str">
+        <x:v>See project documentation; authentication was not independently tested</x:v>
+      </x:c>
+      <x:c r="T107" s="17" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="U107" s="17" t="n">
+        <x:v>45743</x:v>
+      </x:c>
+      <x:c r="V107" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="W107" t="str">
+        <x:v>https://github.com/Kryzo/mcp-Loinc</x:v>
+      </x:c>
+      <x:c r="X107" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="Y107" t="str">
+        <x:v>https://github.com/Kryzo/mcp-Loinc/blob/main/README.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="108">
+      <x:c r="A108" t="str">
+        <x:v>RWE-0185</x:v>
+      </x:c>
+      <x:c r="B108" t="str">
+        <x:v>Medicaid MCP Server</x:v>
+      </x:c>
+      <x:c r="C108" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D108" t="str">
+        <x:v>OMOP &amp; terminology</x:v>
+      </x:c>
+      <x:c r="E108" t="str">
+        <x:v>Medicaid public data access including NADAC drug pricing (1.5M NDCs), Federal Upper Limits, state formularies, and drug rebate program data via data.medicaid.gov.</x:v>
+      </x:c>
+      <x:c r="F108" t="str">
+        <x:v>Terminology | Code lookup | Normalization</x:v>
+      </x:c>
+      <x:c r="G108" t="str">
+        <x:v>Concept-set development | Code validation | Data harmonization</x:v>
+      </x:c>
+      <x:c r="H108" t="str">
+        <x:v>California - 40K drugs with NDC codes, prior authorization requirements, tier-based pricing | New York - 37K drugs with MRA pricing, daily updates, preferred drug lists | Ohio - 76K drugs with comprehensive step therapy and quantity limit data</x:v>
+      </x:c>
+      <x:c r="I108" t="str">
+        <x:v>Automated code lookup or mapping can omit descendants, include inappropriate concepts, or obscure local meaning. Vocabulary versions, licensing, hierarchy behavior, and study-specific concept sets require expert adjudication.</x:v>
+      </x:c>
+      <x:c r="J108" t="str">
+        <x:v>Static documentation and repository metadata reviewed.</x:v>
+      </x:c>
+      <x:c r="K108" t="str">
+        <x:v>Canonical public source resolved: https://github.com/openpharma-org/medicaid-mcp-server</x:v>
+      </x:c>
+      <x:c r="L108" t="str">
+        <x:v>Repository README and declared capability surface statically reviewed: https://github.com/openpharma-org/medicaid-mcp-server/blob/main/README.md</x:v>
+      </x:c>
+      <x:c r="M108" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N108" t="str">
+        <x:v>openpharma-org</x:v>
+      </x:c>
+      <x:c r="O108" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P108" t="str">
+        <x:v>Source repository</x:v>
+      </x:c>
+      <x:c r="Q108" t="str">
+        <x:v>See project documentation; transport was not independently tested</x:v>
+      </x:c>
+      <x:c r="R108" t="str">
+        <x:v>See project documentation; read/write scope was not independently tested</x:v>
+      </x:c>
+      <x:c r="S108" t="str">
+        <x:v>See project documentation; authentication was not independently tested</x:v>
+      </x:c>
+      <x:c r="T108" s="17" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="U108" s="17" t="n">
+        <x:v>46070</x:v>
+      </x:c>
+      <x:c r="V108" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="W108" t="str">
+        <x:v>https://github.com/openpharma-org/medicaid-mcp-server</x:v>
+      </x:c>
+      <x:c r="X108" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="Y108" t="str">
+        <x:v>https://github.com/openpharma-org/medicaid-mcp-server/blob/main/README.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="109">
+      <x:c r="A109" t="str">
+        <x:v>RWE-0202</x:v>
+      </x:c>
+      <x:c r="B109" t="str">
+        <x:v>Medical Calculator MCP</x:v>
+      </x:c>
+      <x:c r="C109" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D109" t="str">
+        <x:v>Biomedical &amp; RWE Infrastructure</x:v>
+      </x:c>
+      <x:c r="E109" t="str">
+        <x:v>121 validated clinical calculators across anesthesiology, critical care, pediatrics, nephrology, pulmonology, cardiology, hematology, emergency medicine, hepatology, and acid-base/metabolic medicine; DDD-onion architecture with 2,073 tests and 244 PMID + 205 DOI citations baked into the formula references.</x:v>
+      </x:c>
+      <x:c r="F109" t="str">
+        <x:v>Biomedical data | Research infrastructure | Identifier resolution</x:v>
+      </x:c>
+      <x:c r="G109" t="str">
+        <x:v>Biomedical evidence enrichment | Identifier and dataset discovery | Translational context for RWE</x:v>
+      </x:c>
+      <x:c r="H109" t="str">
+        <x:v>Research Framework | Roadmap | ⚠️ Boundary Validation: Literature-backed clinical range checking with automatic warnings</x:v>
+      </x:c>
+      <x:c r="I109" t="str">
+        <x:v>Biomedical, personal-health, or translational evidence does not by itself establish clinical effectiveness or causal validity. Source versions, identifiers, coverage, consent, licensing, and cross-database consistency require verification.</x:v>
+      </x:c>
+      <x:c r="J109" t="str">
+        <x:v>Static documentation and repository metadata reviewed.</x:v>
+      </x:c>
+      <x:c r="K109" t="str">
+        <x:v>Canonical public source resolved: https://github.com/u9401066/medical-calc-mcp</x:v>
+      </x:c>
+      <x:c r="L109" t="str">
+        <x:v>Repository README and declared capability surface statically reviewed: https://github.com/u9401066/medical-calc-mcp/blob/main/README.md</x:v>
+      </x:c>
+      <x:c r="M109" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N109" t="str">
+        <x:v>u9401066</x:v>
+      </x:c>
+      <x:c r="O109" t="str">
+        <x:v>Apache-2.0</x:v>
+      </x:c>
+      <x:c r="P109" t="str">
+        <x:v>Source repository</x:v>
+      </x:c>
+      <x:c r="Q109" t="str">
+        <x:v>See project documentation; transport was not independently tested</x:v>
+      </x:c>
+      <x:c r="R109" t="str">
+        <x:v>See project documentation; read/write scope was not independently tested</x:v>
+      </x:c>
+      <x:c r="S109" t="str">
+        <x:v>See project documentation; authentication was not independently tested</x:v>
+      </x:c>
+      <x:c r="T109" s="17" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="U109" s="17" t="n">
+        <x:v>46156</x:v>
+      </x:c>
+      <x:c r="V109" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="W109" t="str">
+        <x:v>https://github.com/u9401066/medical-calc-mcp</x:v>
+      </x:c>
+      <x:c r="X109" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="Y109" t="str">
+        <x:v>https://github.com/u9401066/medical-calc-mcp/blob/main/README.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="110">
+      <x:c r="A110" t="str">
+        <x:v>RWE-0237</x:v>
+      </x:c>
+      <x:c r="B110" t="str">
+        <x:v>Medical MCPs</x:v>
+      </x:c>
+      <x:c r="C110" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D110" t="str">
+        <x:v>Regulatory &amp; Product Data</x:v>
+      </x:c>
+      <x:c r="E110" t="str">
+        <x:v>100+ unified tools across 14 biomedical APIs including Reactome, KEGG, UniProt, OMIM, ChEMBL, and OpenFDA.</x:v>
+      </x:c>
+      <x:c r="F110" t="str">
+        <x:v>Regulatory data | Product evidence | Source verification</x:v>
+      </x:c>
+      <x:c r="G110" t="str">
+        <x:v>Product and identifier resolution | Regulatory context | Evidence-source triangulation</x:v>
+      </x:c>
+      <x:c r="H110" t="str">
+        <x:v>Pathways: Reactome, KEGG, Pathway Commons | Drugs: ChEMBL, MyChem.info, OpenFDA | Literature: PubMed/PubTator3</x:v>
+      </x:c>
+      <x:c r="I110" t="str">
+        <x:v>Regulatory and administrative records answer different questions from comparative-effectiveness studies and can change over time. Coverage, field semantics, refresh cadence, and every decision-relevant result must be checked against the authoritative source.</x:v>
+      </x:c>
+      <x:c r="J110" t="str">
+        <x:v>Static documentation and repository metadata reviewed.</x:v>
+      </x:c>
+      <x:c r="K110" t="str">
+        <x:v>Canonical public source resolved: https://github.com/pascalwhoop/medical-mcps</x:v>
+      </x:c>
+      <x:c r="L110" t="str">
+        <x:v>Repository README and declared capability surface statically reviewed: https://github.com/pascalwhoop/medical-mcps/blob/main/README.md</x:v>
+      </x:c>
+      <x:c r="M110" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N110" t="str">
+        <x:v>pascalwhoop</x:v>
+      </x:c>
+      <x:c r="O110" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P110" t="str">
+        <x:v>Source repository</x:v>
+      </x:c>
+      <x:c r="Q110" t="str">
+        <x:v>See project documentation; transport was not independently tested</x:v>
+      </x:c>
+      <x:c r="R110" t="str">
+        <x:v>See project documentation; read/write scope was not independently tested</x:v>
+      </x:c>
+      <x:c r="S110" t="str">
+        <x:v>See project documentation; authentication was not independently tested</x:v>
+      </x:c>
+      <x:c r="T110" s="17" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="U110" s="17" t="n">
+        <x:v>46137</x:v>
+      </x:c>
+      <x:c r="V110" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="W110" t="str">
+        <x:v>https://github.com/pascalwhoop/medical-mcps</x:v>
+      </x:c>
+      <x:c r="X110" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="Y110" t="str">
+        <x:v>https://github.com/pascalwhoop/medical-mcps/blob/main/README.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="111">
+      <x:c r="A111" t="str">
+        <x:v>RWE-0238</x:v>
+      </x:c>
+      <x:c r="B111" t="str">
+        <x:v>Medical Research MCP Suite</x:v>
+      </x:c>
+      <x:c r="C111" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D111" t="str">
+        <x:v>Literature &amp; Evidence Synthesis</x:v>
+      </x:c>
+      <x:c r="E111" t="str">
+        <x:v>Cross-database medical research intelligence unifying ClinicalTrials.gov, PubMed, and FDA with AI analysis.</x:v>
+      </x:c>
+      <x:c r="F111" t="str">
+        <x:v>Evidence retrieval | Literature search | Source verification</x:v>
+      </x:c>
+      <x:c r="G111" t="str">
+        <x:v>Literature discovery | Evidence scoping | Citation and source retrieval</x:v>
+      </x:c>
+      <x:c r="H111" t="str">
+        <x:v>🔬 ClinicalTrials.gov - 400,000+ clinical studies with real-time data | 📚 PubMed - 35M+ research papers and literature analysis | 💊 FDA Database - 80,000+ drug products and safety data</x:v>
+      </x:c>
+      <x:c r="I111" t="str">
+        <x:v>Provider coverage, indexing delay, query translation, deduplication, full-text rights, and citation accuracy vary. Reproducible reviews still require logged searches, dates, screening decisions, evidence grading, and primary-source verification.</x:v>
+      </x:c>
+      <x:c r="J111" t="str">
+        <x:v>Static documentation and repository metadata reviewed.</x:v>
+      </x:c>
+      <x:c r="K111" t="str">
+        <x:v>Canonical public source resolved: https://github.com/ezhou89/medical-research-mcp-suite</x:v>
+      </x:c>
+      <x:c r="L111" t="str">
+        <x:v>Repository README and declared capability surface statically reviewed: https://github.com/ezhou89/medical-research-mcp-suite/blob/master/README.md</x:v>
+      </x:c>
+      <x:c r="M111" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N111" t="str">
+        <x:v>ezhou89</x:v>
+      </x:c>
+      <x:c r="O111" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P111" t="str">
+        <x:v>Source repository</x:v>
+      </x:c>
+      <x:c r="Q111" t="str">
+        <x:v>See project documentation; transport was not independently tested</x:v>
+      </x:c>
+      <x:c r="R111" t="str">
+        <x:v>See project documentation; read/write scope was not independently tested</x:v>
+      </x:c>
+      <x:c r="S111" t="str">
+        <x:v>See project documentation; authentication was not independently tested</x:v>
+      </x:c>
+      <x:c r="T111" s="17" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="U111" s="17" t="n">
+        <x:v>46041</x:v>
+      </x:c>
+      <x:c r="V111" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="W111" t="str">
+        <x:v>https://github.com/ezhou89/medical-research-mcp-suite</x:v>
+      </x:c>
+      <x:c r="X111" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="Y111" t="str">
+        <x:v>https://github.com/ezhou89/medical-research-mcp-suite/blob/master/README.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="112">
+      <x:c r="A112" t="str">
+        <x:v>RWE-0203</x:v>
+      </x:c>
+      <x:c r="B112" t="str">
+        <x:v>Medical-MCP</x:v>
+      </x:c>
+      <x:c r="C112" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D112" t="str">
+        <x:v>Literature &amp; Evidence Synthesis</x:v>
+      </x:c>
+      <x:c r="E112" t="str">
+        <x:v>Comprehensive medical information from FDA, WHO, PubMed, RxNorm, and Google Scholar.</x:v>
+      </x:c>
+      <x:c r="F112" t="str">
+        <x:v>Evidence retrieval | Literature search | Source verification</x:v>
+      </x:c>
+      <x:c r="G112" t="str">
+        <x:v>Literature discovery | Evidence scoping | Citation and source retrieval</x:v>
+      </x:c>
+      <x:c r="H112" t="str">
+        <x:v>🔬 Comprehensive – Drug info, health stats, medical literature, clinical guidelines, pediatric sources | search-drugs – Search FDA database by brand or generic name | get-drug-details – Get comprehensive drug info by NDC code</x:v>
+      </x:c>
+      <x:c r="I112" t="str">
+        <x:v>Provider coverage, indexing delay, query translation, deduplication, full-text rights, and citation accuracy vary. Reproducible reviews still require logged searches, dates, screening decisions, evidence grading, and primary-source verification.</x:v>
+      </x:c>
+      <x:c r="J112" t="str">
+        <x:v>Static documentation and repository metadata reviewed.</x:v>
+      </x:c>
+      <x:c r="K112" t="str">
+        <x:v>Canonical public source resolved: https://github.com/JamesANZ/medical-mcp</x:v>
+      </x:c>
+      <x:c r="L112" t="str">
+        <x:v>Repository README and declared capability surface statically reviewed: https://github.com/JamesANZ/medical-mcp/blob/main/README.md</x:v>
+      </x:c>
+      <x:c r="M112" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N112" t="str">
+        <x:v>JamesANZ</x:v>
+      </x:c>
+      <x:c r="O112" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P112" t="str">
+        <x:v>Source repository</x:v>
+      </x:c>
+      <x:c r="Q112" t="str">
+        <x:v>See project documentation; transport was not independently tested</x:v>
+      </x:c>
+      <x:c r="R112" t="str">
+        <x:v>See project documentation; read/write scope was not independently tested</x:v>
+      </x:c>
+      <x:c r="S112" t="str">
+        <x:v>See project documentation; authentication was not independently tested</x:v>
+      </x:c>
+      <x:c r="T112" s="17" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="U112" s="17" t="n">
+        <x:v>46177</x:v>
+      </x:c>
+      <x:c r="V112" t="n">
+        <x:v>109</x:v>
+      </x:c>
+      <x:c r="W112" t="str">
+        <x:v>https://github.com/JamesANZ/medical-mcp</x:v>
+      </x:c>
+      <x:c r="X112" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="Y112" t="str">
+        <x:v>https://github.com/JamesANZ/medical-mcp/blob/main/README.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="113">
+      <x:c r="A113" t="str">
+        <x:v>RWE-0186</x:v>
+      </x:c>
+      <x:c r="B113" t="str">
+        <x:v>Medicare MCP</x:v>
+      </x:c>
+      <x:c r="C113" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D113" t="str">
+        <x:v>Regulatory &amp; Product Data</x:v>
+      </x:c>
+      <x:c r="E113" t="str">
+        <x:v>CMS Medicare provider services, prescriber data, hospital utilization, drug spending, and Part B ASP pricing via the Socrata API with quarterly automated updates.</x:v>
+      </x:c>
+      <x:c r="F113" t="str">
+        <x:v>Regulatory data | Product evidence | Source verification</x:v>
+      </x:c>
+      <x:c r="G113" t="str">
+        <x:v>Product and identifier resolution | Regulatory context | Evidence-source triangulation</x:v>
+      </x:c>
+      <x:c r="H113" t="str">
+        <x:v>Prescriber Data: Medicare Part D prescriber information by drug, provider, and geography | Hospital Data: Medicare inpatient hospital utilization and payment data | Drug Spending: Medicare Part D and Part B drug spending trends</x:v>
+      </x:c>
+      <x:c r="I113" t="str">
+        <x:v>Regulatory and administrative records answer different questions from comparative-effectiveness studies and can change over time. Coverage, field semantics, refresh cadence, and every decision-relevant result must be checked against the authoritative source.</x:v>
+      </x:c>
+      <x:c r="J113" t="str">
+        <x:v>Static documentation and repository metadata reviewed.</x:v>
+      </x:c>
+      <x:c r="K113" t="str">
+        <x:v>Canonical public source resolved: https://github.com/openpharma-org/medicare-mcp</x:v>
+      </x:c>
+      <x:c r="L113" t="str">
+        <x:v>Repository README and declared capability surface statically reviewed: https://github.com/openpharma-org/medicare-mcp/blob/main/README.md</x:v>
+      </x:c>
+      <x:c r="M113" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N113" t="str">
+        <x:v>openpharma-org</x:v>
+      </x:c>
+      <x:c r="O113" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P113" t="str">
+        <x:v>Source repository</x:v>
+      </x:c>
+      <x:c r="Q113" t="str">
+        <x:v>See project documentation; transport was not independently tested</x:v>
+      </x:c>
+      <x:c r="R113" t="str">
+        <x:v>See project documentation; read/write scope was not independently tested</x:v>
+      </x:c>
+      <x:c r="S113" t="str">
+        <x:v>See project documentation; authentication was not independently tested</x:v>
+      </x:c>
+      <x:c r="T113" s="17" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="U113" s="17" t="n">
+        <x:v>46249</x:v>
+      </x:c>
+      <x:c r="V113" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="W113" t="str">
+        <x:v>https://github.com/openpharma-org/medicare-mcp</x:v>
+      </x:c>
+      <x:c r="X113" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="Y113" t="str">
+        <x:v>https://github.com/openpharma-org/medicare-mcp/blob/main/README.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="114">
+      <x:c r="A114" t="str">
+        <x:v>RWE-0223</x:v>
+      </x:c>
+      <x:c r="B114" t="str">
+        <x:v>Momentum FHIR MCP Server</x:v>
+      </x:c>
+      <x:c r="C114" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D114" t="str">
+        <x:v>Clinical Data &amp; Interoperability</x:v>
+      </x:c>
+      <x:c r="E114" t="str">
+        <x:v>Natural language interface for healthcare data that eliminates weeks of FHIR learning and prevents LLM hallucination of medical codes.</x:v>
+      </x:c>
+      <x:c r="F114" t="str">
+        <x:v>FHIR / clinical data | Interoperability | Governed access</x:v>
+      </x:c>
+      <x:c r="G114" t="str">
+        <x:v>Clinical-source inspection | Interoperability prototyping | Cohort and data-availability assessment</x:v>
+      </x:c>
+      <x:c r="H114" t="str">
+        <x:v>🗺️ Roadmap | 🏥 FHIR Resource Management: Full CRUD operations for all major FHIR resources | 🔍 Semantic Search: Advanced document search using vector embeddings (via Pinecone)</x:v>
+      </x:c>
+      <x:c r="I114" t="str">
+        <x:v>Clinical systems can contain PHI and may expose write operations. Production use requires explicit authorization, least privilege, audit logging, retention controls, source-system validation, and organization-specific governance.</x:v>
+      </x:c>
+      <x:c r="J114" t="str">
+        <x:v>Static documentation and repository metadata reviewed.</x:v>
+      </x:c>
+      <x:c r="K114" t="str">
+        <x:v>Canonical public source resolved: https://github.com/the-momentum/fhir-mcp-server</x:v>
+      </x:c>
+      <x:c r="L114" t="str">
+        <x:v>Repository README and declared capability surface statically reviewed: https://github.com/the-momentum/fhir-mcp-server/blob/main/README.md</x:v>
+      </x:c>
+      <x:c r="M114" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N114" t="str">
+        <x:v>the-momentum</x:v>
+      </x:c>
+      <x:c r="O114" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P114" t="str">
+        <x:v>Source repository</x:v>
+      </x:c>
+      <x:c r="Q114" t="str">
+        <x:v>See project documentation; transport was not independently tested</x:v>
+      </x:c>
+      <x:c r="R114" t="str">
+        <x:v>See project documentation; read/write scope was not independently tested</x:v>
+      </x:c>
+      <x:c r="S114" t="str">
+        <x:v>See project documentation; authentication was not independently tested</x:v>
+      </x:c>
+      <x:c r="T114" s="17" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="U114" s="17" t="n">
+        <x:v>45953</x:v>
+      </x:c>
+      <x:c r="V114" t="n">
+        <x:v>97</x:v>
+      </x:c>
+      <x:c r="W114" t="str">
+        <x:v>https://github.com/the-momentum/fhir-mcp-server</x:v>
+      </x:c>
+      <x:c r="X114" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="Y114" t="str">
+        <x:v>https://github.com/the-momentum/fhir-mcp-server/blob/main/README.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="115">
+      <x:c r="A115" t="str">
+        <x:v>RWE-0187</x:v>
+      </x:c>
+      <x:c r="B115" t="str">
+        <x:v>NPI Providers MCP</x:v>
+      </x:c>
+      <x:c r="C115" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D115" t="str">
+        <x:v>OMOP &amp; terminology</x:v>
+      </x:c>
+      <x:c r="E115" t="str">
+        <x:v>US provider lookup through the NPPES NPI Registry with NUCC taxonomy resolution.</x:v>
+      </x:c>
+      <x:c r="F115" t="str">
+        <x:v>Terminology | Code lookup | Normalization</x:v>
+      </x:c>
+      <x:c r="G115" t="str">
+        <x:v>Concept-set development | Code validation | Data harmonization</x:v>
+      </x:c>
+      <x:c r="H115" t="str">
+        <x:v>Batch fetch up to 10 NPIs per call; the 10-digit format is validated before any API call | get — return the full entry for an exact taxonomy code | Detects the registry's quirk of returning HTTP 200 with an Errors[] body on validation failure and maps it to typed, recoverable error reasons</x:v>
+      </x:c>
+      <x:c r="I115" t="str">
+        <x:v>Automated code lookup or mapping can omit descendants, include inappropriate concepts, or obscure local meaning. Vocabulary versions, licensing, hierarchy behavior, and study-specific concept sets require expert adjudication.</x:v>
+      </x:c>
+      <x:c r="J115" t="str">
+        <x:v>Static documentation and repository metadata reviewed.</x:v>
+      </x:c>
+      <x:c r="K115" t="str">
+        <x:v>Canonical public source resolved: https://github.com/cyanheads/npi-providers-mcp-server</x:v>
+      </x:c>
+      <x:c r="L115" t="str">
+        <x:v>Repository README and declared capability surface statically reviewed: https://github.com/cyanheads/npi-providers-mcp-server/blob/main/README.md</x:v>
+      </x:c>
+      <x:c r="M115" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N115" t="str">
+        <x:v>cyanheads</x:v>
+      </x:c>
+      <x:c r="O115" t="str">
+        <x:v>Apache-2.0</x:v>
+      </x:c>
+      <x:c r="P115" t="str">
+        <x:v>Source repository</x:v>
+      </x:c>
+      <x:c r="Q115" t="str">
+        <x:v>See project documentation; transport was not independently tested</x:v>
+      </x:c>
+      <x:c r="R115" t="str">
+        <x:v>See project documentation; read/write scope was not independently tested</x:v>
+      </x:c>
+      <x:c r="S115" t="str">
+        <x:v>See project documentation; authentication was not independently tested</x:v>
+      </x:c>
+      <x:c r="T115" s="17" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="U115" s="17" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="V115" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="W115" t="str">
+        <x:v>https://github.com/cyanheads/npi-providers-mcp-server</x:v>
+      </x:c>
+      <x:c r="X115" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="Y115" t="str">
+        <x:v>https://github.com/cyanheads/npi-providers-mcp-server/blob/main/README.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="116">
+      <x:c r="A116" t="str">
+        <x:v>RWE-0239</x:v>
+      </x:c>
+      <x:c r="B116" t="str">
+        <x:v>Open Targets Platform MCP</x:v>
+      </x:c>
+      <x:c r="C116" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D116" t="str">
+        <x:v>Literature &amp; Evidence Synthesis</x:v>
+      </x:c>
+      <x:c r="E116" t="str">
+        <x:v>Official Open Targets server exposing the Platform GraphQL API for target-disease associations, drug-target evidence, and genetic associations to support drug discovery and target identification.</x:v>
+      </x:c>
+      <x:c r="F116" t="str">
+        <x:v>Evidence retrieval | Literature search | Source verification</x:v>
+      </x:c>
+      <x:c r="G116" t="str">
+        <x:v>Literature discovery | Evidence scoping | Citation and source retrieval</x:v>
+      </x:c>
+      <x:c r="H116" t="str">
+        <x:v>🔍 Category-Based Schema Access: Fetch and explore focused subsets of the Open Targets Platform GraphQL schema using category-based subschemas | 📊 Query Execution: Execute custom GraphQL queries against the Open Targets Platform API | ⚡ Batch Query Processing: Execute the same query multiple times with different parameters efficiently</x:v>
+      </x:c>
+      <x:c r="I116" t="str">
+        <x:v>Provider coverage, indexing delay, query translation, deduplication, full-text rights, and citation accuracy vary. Reproducible reviews still require logged searches, dates, screening decisions, evidence grading, and primary-source verification.</x:v>
+      </x:c>
+      <x:c r="J116" t="str">
+        <x:v>Static documentation and repository metadata reviewed.</x:v>
+      </x:c>
+      <x:c r="K116" t="str">
+        <x:v>Canonical public source resolved: https://github.com/opentargets/platform-mcp</x:v>
+      </x:c>
+      <x:c r="L116" t="str">
+        <x:v>Repository README and declared capability surface statically reviewed: https://github.com/opentargets/platform-mcp/blob/main/README.md</x:v>
+      </x:c>
+      <x:c r="M116" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N116" t="str">
+        <x:v>opentargets</x:v>
+      </x:c>
+      <x:c r="O116" t="str">
+        <x:v>Apache-2.0</x:v>
+      </x:c>
+      <x:c r="P116" t="str">
+        <x:v>Source repository</x:v>
+      </x:c>
+      <x:c r="Q116" t="str">
+        <x:v>See project documentation; transport was not independently tested</x:v>
+      </x:c>
+      <x:c r="R116" t="str">
+        <x:v>See project documentation; read/write scope was not independently tested</x:v>
+      </x:c>
+      <x:c r="S116" t="str">
+        <x:v>See project documentation; authentication was not independently tested</x:v>
+      </x:c>
+      <x:c r="T116" s="17" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="U116" s="17" t="n">
+        <x:v>46204</x:v>
+      </x:c>
+      <x:c r="V116" t="n">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="W116" t="str">
+        <x:v>https://github.com/opentargets/platform-mcp</x:v>
+      </x:c>
+      <x:c r="X116" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="Y116" t="str">
+        <x:v>https://github.com/opentargets/platform-mcp/blob/main/README.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="117">
+      <x:c r="A117" t="str">
+        <x:v>RWE-0225</x:v>
+      </x:c>
+      <x:c r="B117" t="str">
+        <x:v>Orthanc DICOM MCP</x:v>
+      </x:c>
+      <x:c r="C117" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D117" t="str">
+        <x:v>Clinical Data &amp; Interoperability</x:v>
+      </x:c>
+      <x:c r="E117" t="str">
+        <x:v>DICOM MCP with Orthanc PACS integration, radiology report generation, FHIR ImagingStudy, and mini-RIS.</x:v>
+      </x:c>
+      <x:c r="F117" t="str">
+        <x:v>FHIR / clinical data | Interoperability | Governed access</x:v>
+      </x:c>
+      <x:c r="G117" t="str">
+        <x:v>Clinical-source inspection | Interoperability prototyping | Cohort and data-availability assessment</x:v>
+      </x:c>
+      <x:c r="H117" t="str">
+        <x:v>🔍 Query DICOM: Search for patients, studies, series, and instances using various criteria | 📄 Read DICOM Reports (PDF): Retrieve DICOM instances containing encapsulated PDFs (e.g., clinical reports) and extract the text content | ⚙️ FHIR Integration: Query and manage FHIR resources (Patient, ImagingStudy, ServiceRequest, etc.)</x:v>
+      </x:c>
+      <x:c r="I117" t="str">
+        <x:v>Clinical systems can contain PHI and may expose write operations. Production use requires explicit authorization, least privilege, audit logging, retention controls, source-system validation, and organization-specific governance.</x:v>
+      </x:c>
+      <x:c r="J117" t="str">
+        <x:v>Static documentation and repository metadata reviewed.</x:v>
+      </x:c>
+      <x:c r="K117" t="str">
+        <x:v>Canonical public source resolved: https://github.com/sscotti/dicom-mcp</x:v>
+      </x:c>
+      <x:c r="L117" t="str">
+        <x:v>Repository README and declared capability surface statically reviewed: https://github.com/sscotti/dicom-mcp/blob/master/README.md</x:v>
+      </x:c>
+      <x:c r="M117" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N117" t="str">
+        <x:v>sscotti</x:v>
+      </x:c>
+      <x:c r="O117" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P117" t="str">
+        <x:v>Source repository</x:v>
+      </x:c>
+      <x:c r="Q117" t="str">
+        <x:v>See project documentation; transport was not independently tested</x:v>
+      </x:c>
+      <x:c r="R117" t="str">
+        <x:v>See project documentation; read/write scope was not independently tested</x:v>
+      </x:c>
+      <x:c r="S117" t="str">
+        <x:v>See project documentation; authentication was not independently tested</x:v>
+      </x:c>
+      <x:c r="T117" s="17" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="U117" s="17" t="n">
+        <x:v>46074</x:v>
+      </x:c>
+      <x:c r="V117" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="W117" t="str">
+        <x:v>https://github.com/sscotti/dicom-mcp</x:v>
+      </x:c>
+      <x:c r="X117" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="Y117" t="str">
+        <x:v>https://github.com/sscotti/dicom-mcp/blob/master/README.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="118">
+      <x:c r="A118" t="str">
+        <x:v>RWE-0208</x:v>
+      </x:c>
+      <x:c r="B118" t="str">
+        <x:v>Pharmacogenomics MCP</x:v>
+      </x:c>
+      <x:c r="C118" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D118" t="str">
+        <x:v>Literature &amp; Evidence Synthesis</x:v>
+      </x:c>
+      <x:c r="E118" t="str">
+        <x:v>Real-time pharmacogenomics across ClinVar variant pathogenicity, PharmGKB drug-gene interactions with CPIC/DPWG dosing guidelines, gnomAD population frequencies, Open Targets drug-target-disease associations, and ClinicalTrials.gov.</x:v>
+      </x:c>
+      <x:c r="F118" t="str">
+        <x:v>Evidence retrieval | Literature search | Source verification</x:v>
+      </x:c>
+      <x:c r="G118" t="str">
+        <x:v>Literature discovery | Evidence scoping | Citation and source retrieval</x:v>
+      </x:c>
+      <x:c r="H118" t="str">
+        <x:v>PharmGKB: Drug-gene interactions, clinical annotations, CPIC/DPWG dosing guidelines | Open Targets: Drug-target-disease associations, pharmacogenomics evidence | ClinicalTrials.gov: Clinical trial search (US and international)</x:v>
+      </x:c>
+      <x:c r="I118" t="str">
+        <x:v>Provider coverage, indexing delay, query translation, deduplication, full-text rights, and citation accuracy vary. Reproducible reviews still require logged searches, dates, screening decisions, evidence grading, and primary-source verification.</x:v>
+      </x:c>
+      <x:c r="J118" t="str">
+        <x:v>Static documentation and repository metadata reviewed.</x:v>
+      </x:c>
+      <x:c r="K118" t="str">
+        <x:v>Canonical public source resolved: https://github.com/Julius-Schmidt/mcp-pharmacogenomics</x:v>
+      </x:c>
+      <x:c r="L118" t="str">
+        <x:v>Repository README and declared capability surface statically reviewed: https://github.com/Julius-Schmidt/mcp-pharmacogenomics/blob/main/README.md</x:v>
+      </x:c>
+      <x:c r="M118" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N118" t="str">
+        <x:v>Julius-Schmidt</x:v>
+      </x:c>
+      <x:c r="O118" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P118" t="str">
+        <x:v>Source repository</x:v>
+      </x:c>
+      <x:c r="Q118" t="str">
+        <x:v>See project documentation; transport was not independently tested</x:v>
+      </x:c>
+      <x:c r="R118" t="str">
+        <x:v>See project documentation; read/write scope was not independently tested</x:v>
+      </x:c>
+      <x:c r="S118" t="str">
+        <x:v>See project documentation; authentication was not independently tested</x:v>
+      </x:c>
+      <x:c r="T118" s="17" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="U118" s="17" t="n">
+        <x:v>46080</x:v>
+      </x:c>
+      <x:c r="V118" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="W118" t="str">
+        <x:v>https://github.com/Julius-Schmidt/mcp-pharmacogenomics</x:v>
+      </x:c>
+      <x:c r="X118" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="Y118" t="str">
+        <x:v>https://github.com/Julius-Schmidt/mcp-pharmacogenomics/blob/main/README.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="119">
+      <x:c r="A119" t="str">
+        <x:v>RWE-0255</x:v>
+      </x:c>
+      <x:c r="B119" t="str">
+        <x:v>PopHIVE MCP Server</x:v>
+      </x:c>
+      <x:c r="C119" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D119" t="str">
+        <x:v>Public Health &amp; Epidemiology</x:v>
+      </x:c>
+      <x:c r="E119" t="str">
+        <x:v>Yale PopHIVE population health data for community health analysis and value-based care.</x:v>
+      </x:c>
+      <x:c r="F119" t="str">
+        <x:v>Public health | Population data | Surveillance</x:v>
+      </x:c>
+      <x:c r="G119" t="str">
+        <x:v>Population-health surveillance | Burden and trend description | External context for RWE studies</x:v>
+      </x:c>
+      <x:c r="H119" t="str">
+        <x:v>Google Health Trends: Population behavior and symptom search patterns | comparestates: Compare health metrics across multiple states with statistical analysis | timeseriesanalysis: Analyze trends over time with aggregation options</x:v>
+      </x:c>
+      <x:c r="I119" t="str">
+        <x:v>Reporting delay, suppression, revisions, changing definitions, geographic comparability, and ecological inference can affect interpretation. Results require dataset-specific denominator and provenance checks.</x:v>
+      </x:c>
+      <x:c r="J119" t="str">
+        <x:v>Static documentation and repository metadata reviewed.</x:v>
+      </x:c>
+      <x:c r="K119" t="str">
+        <x:v>Canonical public source resolved: https://github.com/Cicatriiz/pophive-mcp-server</x:v>
+      </x:c>
+      <x:c r="L119" t="str">
+        <x:v>Repository README and declared capability surface statically reviewed: https://github.com/Cicatriiz/pophive-mcp-server/blob/main/README.md</x:v>
+      </x:c>
+      <x:c r="M119" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N119" t="str">
+        <x:v>Cicatriiz</x:v>
+      </x:c>
+      <x:c r="O119" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P119" t="str">
+        <x:v>Source repository</x:v>
+      </x:c>
+      <x:c r="Q119" t="str">
+        <x:v>See project documentation; transport was not independently tested</x:v>
+      </x:c>
+      <x:c r="R119" t="str">
+        <x:v>See project documentation; read/write scope was not independently tested</x:v>
+      </x:c>
+      <x:c r="S119" t="str">
+        <x:v>See project documentation; authentication was not independently tested</x:v>
+      </x:c>
+      <x:c r="T119" s="17" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="U119" s="17" t="n">
+        <x:v>45867</x:v>
+      </x:c>
+      <x:c r="V119" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="W119" t="str">
+        <x:v>https://github.com/Cicatriiz/pophive-mcp-server</x:v>
+      </x:c>
+      <x:c r="X119" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="Y119" t="str">
+        <x:v>https://github.com/Cicatriiz/pophive-mcp-server/blob/main/README.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="120">
+      <x:c r="A120" t="str">
+        <x:v>RWE-0240</x:v>
+      </x:c>
+      <x:c r="B120" t="str">
+        <x:v>Precision Medicine MCP</x:v>
+      </x:c>
+      <x:c r="C120" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D120" t="str">
+        <x:v>Biomedical &amp; RWE Infrastructure</x:v>
+      </x:c>
+      <x:c r="E120" t="str">
+        <x:v>Multi-omics precision medicine platform with genomics, spatial transcriptomics, imaging, and clinician-in-the-loop workflows.</x:v>
+      </x:c>
+      <x:c r="F120" t="str">
+        <x:v>Biomedical data | Research infrastructure | Identifier resolution</x:v>
+      </x:c>
+      <x:c r="G120" t="str">
+        <x:v>Biomedical evidence enrichment | Identifier and dataset discovery | Translational context for RWE</x:v>
+      </x:c>
+      <x:c r="H120" t="str">
+        <x:v>Search documented biomedical or research-data sources | Retrieve structured identifiers and evidence records | Support cross-source evidence enrichment</x:v>
+      </x:c>
+      <x:c r="I120" t="str">
+        <x:v>Biomedical, personal-health, or translational evidence does not by itself establish clinical effectiveness or causal validity. Source versions, identifiers, coverage, consent, licensing, and cross-database consistency require verification.</x:v>
+      </x:c>
+      <x:c r="J120" t="str">
+        <x:v>Static documentation and repository metadata reviewed.</x:v>
+      </x:c>
+      <x:c r="K120" t="str">
+        <x:v>Canonical public source resolved: https://github.com/lynnlangit/precision-medicine-mcp</x:v>
+      </x:c>
+      <x:c r="L120" t="str">
+        <x:v>Repository README and declared capability surface statically reviewed: https://github.com/lynnlangit/precision-medicine-mcp/blob/main/README.md</x:v>
+      </x:c>
+      <x:c r="M120" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N120" t="str">
+        <x:v>lynnlangit</x:v>
+      </x:c>
+      <x:c r="O120" t="str">
+        <x:v>Apache-2.0</x:v>
+      </x:c>
+      <x:c r="P120" t="str">
+        <x:v>Source repository</x:v>
+      </x:c>
+      <x:c r="Q120" t="str">
+        <x:v>See project documentation; transport was not independently tested</x:v>
+      </x:c>
+      <x:c r="R120" t="str">
+        <x:v>See project documentation; read/write scope was not independently tested</x:v>
+      </x:c>
+      <x:c r="S120" t="str">
+        <x:v>See project documentation; authentication was not independently tested</x:v>
+      </x:c>
+      <x:c r="T120" s="17" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="U120" s="17" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="V120" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="W120" t="str">
+        <x:v>https://github.com/lynnlangit/precision-medicine-mcp</x:v>
+      </x:c>
+      <x:c r="X120" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="Y120" t="str">
+        <x:v>https://github.com/lynnlangit/precision-medicine-mcp/blob/main/README.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="121">
+      <x:c r="A121" t="str">
+        <x:v>RWE-0241</x:v>
+      </x:c>
+      <x:c r="B121" t="str">
+        <x:v>Protein Structure Analyzer</x:v>
+      </x:c>
+      <x:c r="C121" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D121" t="str">
+        <x:v>Biomedical &amp; RWE Infrastructure</x:v>
+      </x:c>
+      <x:c r="E121" t="str">
+        <x:v>Protein structure analysis via MCP for research and drug discovery workflows.</x:v>
+      </x:c>
+      <x:c r="F121" t="str">
+        <x:v>Biomedical data | Research infrastructure | Identifier resolution</x:v>
+      </x:c>
+      <x:c r="G121" t="str">
+        <x:v>Biomedical evidence enrichment | Identifier and dataset discovery | Translational context for RWE</x:v>
+      </x:c>
+      <x:c r="H121" t="str">
+        <x:v>Structure Search: Find proteins by name, gene, or organism | Region Analysis: Identify high/low confidence structural regions | Parallel Analysis: Confidence analysis for protein sets</x:v>
+      </x:c>
+      <x:c r="I121" t="str">
+        <x:v>Biomedical, personal-health, or translational evidence does not by itself establish clinical effectiveness or causal validity. Source versions, identifiers, coverage, consent, licensing, and cross-database consistency require verification.</x:v>
+      </x:c>
+      <x:c r="J121" t="str">
+        <x:v>Static documentation and repository metadata reviewed.</x:v>
+      </x:c>
+      <x:c r="K121" t="str">
+        <x:v>Canonical public source resolved: https://github.com/Augmented-Nature/AlphaFold-MCP-Server</x:v>
+      </x:c>
+      <x:c r="L121" t="str">
+        <x:v>Repository README and declared capability surface statically reviewed: https://github.com/Augmented-Nature/AlphaFold-MCP-Server/blob/main/README.md</x:v>
+      </x:c>
+      <x:c r="M121" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N121" t="str">
+        <x:v>Augmented-Nature</x:v>
+      </x:c>
+      <x:c r="O121" t="str">
+        <x:v>Not declared</x:v>
+      </x:c>
+      <x:c r="P121" t="str">
+        <x:v>Source repository</x:v>
+      </x:c>
+      <x:c r="Q121" t="str">
+        <x:v>See project documentation; transport was not independently tested</x:v>
+      </x:c>
+      <x:c r="R121" t="str">
+        <x:v>See project documentation; read/write scope was not independently tested</x:v>
+      </x:c>
+      <x:c r="S121" t="str">
+        <x:v>See project documentation; authentication was not independently tested</x:v>
+      </x:c>
+      <x:c r="T121" s="17" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="U121" s="17" t="n">
+        <x:v>46012</x:v>
+      </x:c>
+      <x:c r="V121" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="W121" t="str">
+        <x:v>https://github.com/Augmented-Nature/AlphaFold-MCP-Server</x:v>
+      </x:c>
+      <x:c r="X121" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="Y121" t="str">
+        <x:v>https://github.com/Augmented-Nature/AlphaFold-MCP-Server/blob/main/README.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="122">
+      <x:c r="A122" t="str">
+        <x:v>RWE-0242</x:v>
+      </x:c>
+      <x:c r="B122" t="str">
+        <x:v>PubMed MCP</x:v>
+      </x:c>
+      <x:c r="C122" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D122" t="str">
+        <x:v>Literature &amp; Evidence Synthesis</x:v>
+      </x:c>
+      <x:c r="E122" t="str">
+        <x:v>Advanced PubMed search with citation export (BibTeX, APA, MLA), author search, journal analysis, and article comparison.</x:v>
+      </x:c>
+      <x:c r="F122" t="str">
+        <x:v>Evidence retrieval | Literature search | Source verification</x:v>
+      </x:c>
+      <x:c r="G122" t="str">
+        <x:v>Literature discovery | Evidence scoping | Citation and source retrieval</x:v>
+      </x:c>
+      <x:c r="H122" t="str">
+        <x:v>Advanced PubMed Search: Search with complex filters including date ranges, article types, authors, journals, and MeSH terms | Article Details: Retrieve detailed information for specific PMIDs including abstracts, authors, and metadata | Citation Export: Export citations in multiple formats (BibTeX, APA, MLA, Chicago, Vancouver, EndNote, RIS)</x:v>
+      </x:c>
+      <x:c r="I122" t="str">
+        <x:v>Provider coverage, indexing delay, query translation, deduplication, full-text rights, and citation accuracy vary. Reproducible reviews still require logged searches, dates, screening decisions, evidence grading, and primary-source verification.</x:v>
+      </x:c>
+      <x:c r="J122" t="str">
+        <x:v>Static documentation and repository metadata reviewed.</x:v>
+      </x:c>
+      <x:c r="K122" t="str">
+        <x:v>Canonical public source resolved: https://github.com/chrismannina/pubmed-mcp</x:v>
+      </x:c>
+      <x:c r="L122" t="str">
+        <x:v>Repository README and declared capability surface statically reviewed: https://github.com/chrismannina/pubmed-mcp/blob/main/README.md</x:v>
+      </x:c>
+      <x:c r="M122" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N122" t="str">
+        <x:v>chrismannina</x:v>
+      </x:c>
+      <x:c r="O122" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P122" t="str">
+        <x:v>Source repository</x:v>
+      </x:c>
+      <x:c r="Q122" t="str">
+        <x:v>See project documentation; transport was not independently tested</x:v>
+      </x:c>
+      <x:c r="R122" t="str">
+        <x:v>See project documentation; read/write scope was not independently tested</x:v>
+      </x:c>
+      <x:c r="S122" t="str">
+        <x:v>See project documentation; authentication was not independently tested</x:v>
+      </x:c>
+      <x:c r="T122" s="17" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="U122" s="17" t="n">
+        <x:v>45826</x:v>
+      </x:c>
+      <x:c r="V122" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="W122" t="str">
+        <x:v>https://github.com/chrismannina/pubmed-mcp</x:v>
+      </x:c>
+      <x:c r="X122" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="Y122" t="str">
+        <x:v>https://github.com/chrismannina/pubmed-mcp/blob/main/README.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="123">
+      <x:c r="A123" t="str">
+        <x:v>RWE-0226</x:v>
+      </x:c>
+      <x:c r="B123" t="str">
+        <x:v>Quiquemz FHIR MCP</x:v>
+      </x:c>
+      <x:c r="C123" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D123" t="str">
+        <x:v>Clinical Data &amp; Interoperability</x:v>
+      </x:c>
+      <x:c r="E123" t="str">
+        <x:v>C# FHIR R4 MCP server with CRUD, search, transactions, and Azure FHIR Server support.</x:v>
+      </x:c>
+      <x:c r="F123" t="str">
+        <x:v>FHIR / clinical data | Interoperability | Governed access</x:v>
+      </x:c>
+      <x:c r="G123" t="str">
+        <x:v>Clinical-source inspection | Interoperability prototyping | Cohort and data-availability assessment</x:v>
+      </x:c>
+      <x:c r="H123" t="str">
+        <x:v>ReadResource: Retrieve a resource by its ID. | SearchResources: Search for resources based on specific criteria. | FindNumberOfResources: Count the number of resources that match a search criteria.</x:v>
+      </x:c>
+      <x:c r="I123" t="str">
+        <x:v>Clinical systems can contain PHI and may expose write operations. Production use requires explicit authorization, least privilege, audit logging, retention controls, source-system validation, and organization-specific governance.</x:v>
+      </x:c>
+      <x:c r="J123" t="str">
+        <x:v>Static documentation and repository metadata reviewed.</x:v>
+      </x:c>
+      <x:c r="K123" t="str">
+        <x:v>Canonical public source resolved: https://github.com/quiquemz/fhir-mcp-server</x:v>
+      </x:c>
+      <x:c r="L123" t="str">
+        <x:v>Repository README and declared capability surface statically reviewed: https://github.com/quiquemz/fhir-mcp-server/blob/main/README.md</x:v>
+      </x:c>
+      <x:c r="M123" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N123" t="str">
+        <x:v>quiquemz</x:v>
+      </x:c>
+      <x:c r="O123" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P123" t="str">
+        <x:v>Source repository</x:v>
+      </x:c>
+      <x:c r="Q123" t="str">
+        <x:v>See project documentation; transport was not independently tested</x:v>
+      </x:c>
+      <x:c r="R123" t="str">
+        <x:v>See project documentation; read/write scope was not independently tested</x:v>
+      </x:c>
+      <x:c r="S123" t="str">
+        <x:v>See project documentation; authentication was not independently tested</x:v>
+      </x:c>
+      <x:c r="T123" s="17" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="U123" s="17" t="n">
+        <x:v>45779</x:v>
+      </x:c>
+      <x:c r="V123" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="W123" t="str">
+        <x:v>https://github.com/quiquemz/fhir-mcp-server</x:v>
+      </x:c>
+      <x:c r="X123" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="Y123" t="str">
+        <x:v>https://github.com/quiquemz/fhir-mcp-server/blob/main/README.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="124">
+      <x:c r="A124" t="str">
+        <x:v>RWE-0243</x:v>
+      </x:c>
+      <x:c r="B124" t="str">
+        <x:v>Reactome MCP</x:v>
+      </x:c>
+      <x:c r="C124" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D124" t="str">
+        <x:v>Biomedical &amp; RWE Infrastructure</x:v>
+      </x:c>
+      <x:c r="E124" t="str">
+        <x:v>Official Reactome MCP server exposing 40+ tools for pathway search, enrichment analysis, ID mapping, species/disease annotation, and biological pathway data export.</x:v>
+      </x:c>
+      <x:c r="F124" t="str">
+        <x:v>Biomedical data | Research infrastructure | Identifier resolution</x:v>
+      </x:c>
+      <x:c r="G124" t="str">
+        <x:v>Biomedical evidence enrichment | Identifier and dataset discovery | Translational context for RWE</x:v>
+      </x:c>
+      <x:c r="H124" t="str">
+        <x:v>Pathway enrichment analysis — submit gene/protein lists and retrieve over-representation results, including p-values, FDR, and found/not-found identifiers | Search — full-text search across pathways, reactions, proteins, genes, and compounds with faceting, pagination, autocomplete, and spellcheck | Pathway browsing — navigate the pathway hierarchy, retrieve event details, ancestors, contained events, and participants</x:v>
+      </x:c>
+      <x:c r="I124" t="str">
+        <x:v>Biomedical, personal-health, or translational evidence does not by itself establish clinical effectiveness or causal validity. Source versions, identifiers, coverage, consent, licensing, and cross-database consistency require verification.</x:v>
+      </x:c>
+      <x:c r="J124" t="str">
+        <x:v>Static documentation and repository metadata reviewed.</x:v>
+      </x:c>
+      <x:c r="K124" t="str">
+        <x:v>Canonical public source resolved: https://github.com/reactome/reactome-mcp</x:v>
+      </x:c>
+      <x:c r="L124" t="str">
+        <x:v>Repository README and declared capability surface statically reviewed: https://github.com/reactome/reactome-mcp/blob/main/README.md</x:v>
+      </x:c>
+      <x:c r="M124" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N124" t="str">
+        <x:v>reactome</x:v>
+      </x:c>
+      <x:c r="O124" t="str">
+        <x:v>Apache-2.0</x:v>
+      </x:c>
+      <x:c r="P124" t="str">
+        <x:v>Source repository</x:v>
+      </x:c>
+      <x:c r="Q124" t="str">
+        <x:v>See project documentation; transport was not independently tested</x:v>
+      </x:c>
+      <x:c r="R124" t="str">
+        <x:v>See project documentation; read/write scope was not independently tested</x:v>
+      </x:c>
+      <x:c r="S124" t="str">
+        <x:v>See project documentation; authentication was not independently tested</x:v>
+      </x:c>
+      <x:c r="T124" s="17" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="U124" s="17" t="n">
+        <x:v>46204</x:v>
+      </x:c>
+      <x:c r="V124" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="W124" t="str">
+        <x:v>https://github.com/reactome/reactome-mcp</x:v>
+      </x:c>
+      <x:c r="X124" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="Y124" t="str">
+        <x:v>https://github.com/reactome/reactome-mcp/blob/main/README.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="125">
+      <x:c r="A125" t="str">
+        <x:v>RWE-0211</x:v>
+      </x:c>
+      <x:c r="B125" t="str">
+        <x:v>SNOMED CT MCP</x:v>
+      </x:c>
+      <x:c r="C125" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D125" t="str">
+        <x:v>Clinical Data &amp; Interoperability</x:v>
+      </x:c>
+      <x:c r="E125" t="str">
+        <x:v>SNOMED CT concept lookup via FHIR R4 terminology server for clinical coding.</x:v>
+      </x:c>
+      <x:c r="F125" t="str">
+        <x:v>FHIR / clinical data | Interoperability | Governed access</x:v>
+      </x:c>
+      <x:c r="G125" t="str">
+        <x:v>Clinical-source inspection | Interoperability prototyping | Cohort and data-availability assessment</x:v>
+      </x:c>
+      <x:c r="H125" t="str">
+        <x:v>term (string, required) — Clinical term to search, e.g. "exercise therapy", "diabetes", "appendectomy" | domain (string, optional, default "all") — Scope the search to a SNOMED CT top-level hierarchy: | "pharmaceuticalproduct" — medications, vaccines, clinical drugs</x:v>
+      </x:c>
+      <x:c r="I125" t="str">
+        <x:v>Clinical systems can contain PHI and may expose write operations. Production use requires explicit authorization, least privilege, audit logging, retention controls, source-system validation, and organization-specific governance.</x:v>
+      </x:c>
+      <x:c r="J125" t="str">
+        <x:v>Static documentation and repository metadata reviewed.</x:v>
+      </x:c>
+      <x:c r="K125" t="str">
+        <x:v>Canonical public source resolved: https://github.com/eigenbau/mcp-snomed-ct</x:v>
+      </x:c>
+      <x:c r="L125" t="str">
+        <x:v>Repository README and declared capability surface statically reviewed: https://github.com/eigenbau/mcp-snomed-ct/blob/main/README.md</x:v>
+      </x:c>
+      <x:c r="M125" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N125" t="str">
+        <x:v>eigenbau</x:v>
+      </x:c>
+      <x:c r="O125" t="str">
+        <x:v>Apache-2.0</x:v>
+      </x:c>
+      <x:c r="P125" t="str">
+        <x:v>Source repository</x:v>
+      </x:c>
+      <x:c r="Q125" t="str">
+        <x:v>See project documentation; transport was not independently tested</x:v>
+      </x:c>
+      <x:c r="R125" t="str">
+        <x:v>See project documentation; read/write scope was not independently tested</x:v>
+      </x:c>
+      <x:c r="S125" t="str">
+        <x:v>See project documentation; authentication was not independently tested</x:v>
+      </x:c>
+      <x:c r="T125" s="17" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="U125" s="17" t="n">
+        <x:v>46085</x:v>
+      </x:c>
+      <x:c r="V125" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="W125" t="str">
+        <x:v>https://github.com/eigenbau/mcp-snomed-ct</x:v>
+      </x:c>
+      <x:c r="X125" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="Y125" t="str">
+        <x:v>https://github.com/eigenbau/mcp-snomed-ct/blob/main/README.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="126">
+      <x:c r="A126" t="str">
+        <x:v>RWE-0245</x:v>
+      </x:c>
+      <x:c r="B126" t="str">
+        <x:v>TealFlow MCP</x:v>
+      </x:c>
+      <x:c r="C126" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D126" t="str">
+        <x:v>Trials &amp; Study Design</x:v>
+      </x:c>
+      <x:c r="E126" t="str">
+        <x:v>Build Teal R Shiny clinical trial analysis apps with AI assistance.</x:v>
+      </x:c>
+      <x:c r="F126" t="str">
+        <x:v>Clinical trials | R / Shiny | Teal</x:v>
+      </x:c>
+      <x:c r="G126" t="str">
+        <x:v>Trial-analysis prototyping | Interactive results review | Reproducible app development</x:v>
+      </x:c>
+      <x:c r="H126" t="str">
+        <x:v>teal.modules.general - General-purpose analysis modules | teal.modules.clinical - Clinical trial-specific modules | Quickstart Guide - Get started with VSCode and GitHub Copilot</x:v>
+      </x:c>
+      <x:c r="I126" t="str">
+        <x:v>Provider coverage, indexing delay, query translation, deduplication, full-text rights, and citation accuracy vary. Reproducible reviews still require logged searches, dates, screening decisions, evidence grading, and primary-source verification.</x:v>
+      </x:c>
+      <x:c r="J126" t="str">
+        <x:v>Static documentation and repository metadata reviewed.</x:v>
+      </x:c>
+      <x:c r="K126" t="str">
+        <x:v>Canonical public source resolved: https://github.com/Appsilon/TealFlowMCP</x:v>
+      </x:c>
+      <x:c r="L126" t="str">
+        <x:v>Repository README and declared capability surface statically reviewed: https://github.com/Appsilon/TealFlowMCP/blob/develop/README.md</x:v>
+      </x:c>
+      <x:c r="M126" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N126" t="str">
+        <x:v>Appsilon</x:v>
+      </x:c>
+      <x:c r="O126" t="str">
+        <x:v>Not declared</x:v>
+      </x:c>
+      <x:c r="P126" t="str">
+        <x:v>Source repository</x:v>
+      </x:c>
+      <x:c r="Q126" t="str">
+        <x:v>See project documentation; transport was not independently tested</x:v>
+      </x:c>
+      <x:c r="R126" t="str">
+        <x:v>See project documentation; read/write scope was not independently tested</x:v>
+      </x:c>
+      <x:c r="S126" t="str">
+        <x:v>See project documentation; authentication was not independently tested</x:v>
+      </x:c>
+      <x:c r="T126" s="17" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="U126" s="17" t="n">
+        <x:v>46082</x:v>
+      </x:c>
+      <x:c r="V126" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="W126" t="str">
+        <x:v>https://github.com/Appsilon/TealFlowMCP</x:v>
+      </x:c>
+      <x:c r="X126" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="Y126" t="str">
+        <x:v>https://github.com/Appsilon/TealFlowMCP/blob/develop/README.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="127">
+      <x:c r="A127" t="str">
+        <x:v>RWE-0256</x:v>
+      </x:c>
+      <x:c r="B127" t="str">
+        <x:v>WHO GHO MCP</x:v>
+      </x:c>
+      <x:c r="C127" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D127" t="str">
+        <x:v>Public Health &amp; Epidemiology</x:v>
+      </x:c>
+      <x:c r="E127" t="str">
+        <x:v>WHO Global Health Observatory indicators by country, region, year, and demographic.</x:v>
+      </x:c>
+      <x:c r="F127" t="str">
+        <x:v>Public health | Population data | Surveillance</x:v>
+      </x:c>
+      <x:c r="G127" t="str">
+        <x:v>Population-health surveillance | Burden and trend description | External context for RWE studies</x:v>
+      </x:c>
+      <x:c r="H127" t="str">
+        <x:v>Returns indicator codes and display names for use with whoqueryindicatordata | Call before whoqueryindicatordata to confirm which filter dimensions are valid | Codes absent from the catalog are reported in notFound rather than raising an error</x:v>
+      </x:c>
+      <x:c r="I127" t="str">
+        <x:v>Reporting delay, suppression, revisions, changing definitions, geographic comparability, and ecological inference can affect interpretation. Results require dataset-specific denominator and provenance checks.</x:v>
+      </x:c>
+      <x:c r="J127" t="str">
+        <x:v>Static documentation and repository metadata reviewed.</x:v>
+      </x:c>
+      <x:c r="K127" t="str">
+        <x:v>Canonical public source resolved: https://github.com/cyanheads/who-gho-mcp-server</x:v>
+      </x:c>
+      <x:c r="L127" t="str">
+        <x:v>Repository README and declared capability surface statically reviewed: https://github.com/cyanheads/who-gho-mcp-server/blob/main/README.md</x:v>
+      </x:c>
+      <x:c r="M127" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N127" t="str">
+        <x:v>cyanheads</x:v>
+      </x:c>
+      <x:c r="O127" t="str">
+        <x:v>Apache-2.0</x:v>
+      </x:c>
+      <x:c r="P127" t="str">
+        <x:v>Source repository</x:v>
+      </x:c>
+      <x:c r="Q127" t="str">
+        <x:v>See project documentation; transport was not independently tested</x:v>
+      </x:c>
+      <x:c r="R127" t="str">
+        <x:v>See project documentation; read/write scope was not independently tested</x:v>
+      </x:c>
+      <x:c r="S127" t="str">
+        <x:v>See project documentation; authentication was not independently tested</x:v>
+      </x:c>
+      <x:c r="T127" s="17" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="U127" s="17" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="V127" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="W127" t="str">
+        <x:v>https://github.com/cyanheads/who-gho-mcp-server</x:v>
+      </x:c>
+      <x:c r="X127" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="Y127" t="str">
+        <x:v>https://github.com/cyanheads/who-gho-mcp-server/blob/main/README.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="128">
+      <x:c r="A128" t="str">
+        <x:v>RWE-0216</x:v>
+      </x:c>
+      <x:c r="B128" t="str">
+        <x:v>CDS Hooks FHIR MCP</x:v>
+      </x:c>
+      <x:c r="C128" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D128" t="str">
+        <x:v>Clinical Data &amp; Interoperability</x:v>
+      </x:c>
+      <x:c r="E128" t="str">
+        <x:v>FHIR R4 MCP with 17 tools including CDS Hooks integration (patient-view, order-select/sign, encounter-start/discharge), FHIR Consent checking, AuditEvent logging, RBAC, and multi-persona output for clinician/patient/admin contexts.</x:v>
+      </x:c>
+      <x:c r="F128" t="str">
+        <x:v>FHIR / clinical data | Interoperability | Governed access</x:v>
+      </x:c>
+      <x:c r="G128" t="str">
+        <x:v>Clinical-source inspection | Interoperability prototyping | Cohort and data-availability assessment</x:v>
+      </x:c>
+      <x:c r="H128" t="str">
+        <x:v>Governance layer — consent checking, FHIR AuditEvent logging, RBAC | Multi-persona output — same data formatted for clinician, patient, or admin | 17 MCP tools — CRUD, search, bulk import/export, CDS Hooks, consent, audit</x:v>
+      </x:c>
+      <x:c r="I128" t="str">
+        <x:v>Clinical systems can contain PHI and may expose write operations. Production use requires explicit authorization, least privilege, audit logging, retention controls, source-system validation, and organization-specific governance.</x:v>
+      </x:c>
+      <x:c r="J128" t="str">
+        <x:v>Static documentation and repository metadata reviewed.</x:v>
+      </x:c>
+      <x:c r="K128" t="str">
+        <x:v>Canonical public source resolved: https://github.com/mj991218/mcp-fhir</x:v>
+      </x:c>
+      <x:c r="L128" t="str">
+        <x:v>Repository README and declared capability surface statically reviewed: https://github.com/mj991218/mcp-fhir/blob/master/README.md</x:v>
+      </x:c>
+      <x:c r="M128" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N128" t="str">
+        <x:v>mj991218</x:v>
+      </x:c>
+      <x:c r="O128" t="str">
+        <x:v>Not declared</x:v>
+      </x:c>
+      <x:c r="P128" t="str">
+        <x:v>Source repository</x:v>
+      </x:c>
+      <x:c r="Q128" t="str">
+        <x:v>See project documentation; transport was not independently tested</x:v>
+      </x:c>
+      <x:c r="R128" t="str">
+        <x:v>See project documentation; read/write scope was not independently tested</x:v>
+      </x:c>
+      <x:c r="S128" t="str">
+        <x:v>See project documentation; authentication was not independently tested</x:v>
+      </x:c>
+      <x:c r="T128" s="17" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="U128" s="17" t="n">
+        <x:v>46093</x:v>
+      </x:c>
+      <x:c r="V128" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W128" t="str">
+        <x:v>https://github.com/mj991218/mcp-fhir</x:v>
+      </x:c>
+      <x:c r="X128" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="Y128" t="str">
+        <x:v>https://github.com/mj991218/mcp-fhir/blob/master/README.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="129">
+      <x:c r="A129" t="str">
+        <x:v>RWE-0219</x:v>
+      </x:c>
+      <x:c r="B129" t="str">
+        <x:v>Epic FHIR MCP Server</x:v>
+      </x:c>
+      <x:c r="C129" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D129" t="str">
+        <x:v>Clinical Data &amp; Interoperability</x:v>
+      </x:c>
+      <x:c r="E129" t="str">
+        <x:v>Production-ready Epic FHIR R4 connector with OAuth2 Backend Systems Flow + JWT authentication, supporting both stdio (Claude Desktop) and Streamable HTTP transports for web clients.</x:v>
+      </x:c>
+      <x:c r="F129" t="str">
+        <x:v>FHIR / clinical data | Interoperability | Governed access</x:v>
+      </x:c>
+      <x:c r="G129" t="str">
+        <x:v>Clinical-source inspection | Interoperability prototyping | Cohort and data-availability assessment</x:v>
+      </x:c>
+      <x:c r="H129" t="str">
+        <x:v>Epic FHIR R4 API - Access patient data, medications, observations, and more | Epic FHIR Sandbox account (Sign up) | Patient.Read</x:v>
+      </x:c>
+      <x:c r="I129" t="str">
+        <x:v>Clinical systems can contain PHI and may expose write operations. Production use requires explicit authorization, least privilege, audit logging, retention controls, source-system validation, and organization-specific governance.</x:v>
+      </x:c>
+      <x:c r="J129" t="str">
+        <x:v>Static documentation and repository metadata reviewed.</x:v>
+      </x:c>
+      <x:c r="K129" t="str">
+        <x:v>Canonical public source resolved: https://github.com/albertorb/mcp-server-fhir</x:v>
+      </x:c>
+      <x:c r="L129" t="str">
+        <x:v>Repository README and declared capability surface statically reviewed: https://github.com/albertorb/mcp-server-fhir/blob/main/README.md</x:v>
+      </x:c>
+      <x:c r="M129" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N129" t="str">
+        <x:v>albertorb</x:v>
+      </x:c>
+      <x:c r="O129" t="str">
+        <x:v>Apache-2.0</x:v>
+      </x:c>
+      <x:c r="P129" t="str">
+        <x:v>Source repository</x:v>
+      </x:c>
+      <x:c r="Q129" t="str">
+        <x:v>See project documentation; transport was not independently tested</x:v>
+      </x:c>
+      <x:c r="R129" t="str">
+        <x:v>See project documentation; read/write scope was not independently tested</x:v>
+      </x:c>
+      <x:c r="S129" t="str">
+        <x:v>See project documentation; authentication was not independently tested</x:v>
+      </x:c>
+      <x:c r="T129" s="17" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="U129" s="17" t="n">
+        <x:v>46038</x:v>
+      </x:c>
+      <x:c r="V129" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W129" t="str">
+        <x:v>https://github.com/albertorb/mcp-server-fhir</x:v>
+      </x:c>
+      <x:c r="X129" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="Y129" t="str">
+        <x:v>https://github.com/albertorb/mcp-server-fhir/blob/main/README.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="130">
+      <x:c r="A130" t="str">
+        <x:v>RWE-0197</x:v>
+      </x:c>
+      <x:c r="B130" t="str">
+        <x:v>Japan Healthcare MCP</x:v>
+      </x:c>
+      <x:c r="C130" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D130" t="str">
+        <x:v>Regulatory &amp; Product Data</x:v>
+      </x:c>
+      <x:c r="E130" t="str">
+        <x:v>Local-first TypeScript monorepo and MCP server for Japanese healthcare reference data (drug master, reimbursement and medical fee codes, PMDA) with SQLite storage, source attribution, synthetic sample data, and CLI/REST companions.</x:v>
+      </x:c>
+      <x:c r="F130" t="str">
+        <x:v>Regulatory data | Product evidence | Source verification</x:v>
+      </x:c>
+      <x:c r="G130" t="str">
+        <x:v>Product and identifier resolution | Regulatory context | Evidence-source triangulation</x:v>
+      </x:c>
+      <x:c r="H130" t="str">
+        <x:v>Keep source attribution and data provenance visible in search results. | packages/core — core data models, importers, search, source attribution, and safety response modules. | packages/cli — jhc command line interface for local database initialization, imports, searches, diffs, and MCP startup.</x:v>
+      </x:c>
+      <x:c r="I130" t="str">
+        <x:v>Regulatory and administrative records answer different questions from comparative-effectiveness studies and can change over time. Coverage, field semantics, refresh cadence, and every decision-relevant result must be checked against the authoritative source.</x:v>
+      </x:c>
+      <x:c r="J130" t="str">
+        <x:v>Static documentation and repository metadata reviewed.</x:v>
+      </x:c>
+      <x:c r="K130" t="str">
+        <x:v>Canonical public source resolved: https://github.com/chinahamu/japan-healthcare-mcp</x:v>
+      </x:c>
+      <x:c r="L130" t="str">
+        <x:v>Repository README and declared capability surface statically reviewed: https://github.com/chinahamu/japan-healthcare-mcp/blob/main/README.md</x:v>
+      </x:c>
+      <x:c r="M130" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N130" t="str">
+        <x:v>chinahamu</x:v>
+      </x:c>
+      <x:c r="O130" t="str">
+        <x:v>Apache-2.0</x:v>
+      </x:c>
+      <x:c r="P130" t="str">
+        <x:v>Source repository</x:v>
+      </x:c>
+      <x:c r="Q130" t="str">
+        <x:v>See project documentation; transport was not independently tested</x:v>
+      </x:c>
+      <x:c r="R130" t="str">
+        <x:v>See project documentation; read/write scope was not independently tested</x:v>
+      </x:c>
+      <x:c r="S130" t="str">
+        <x:v>See project documentation; authentication was not independently tested</x:v>
+      </x:c>
+      <x:c r="T130" s="17" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="U130" s="17" t="n">
+        <x:v>46199</x:v>
+      </x:c>
+      <x:c r="V130" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W130" t="str">
+        <x:v>https://github.com/chinahamu/japan-healthcare-mcp</x:v>
+      </x:c>
+      <x:c r="X130" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="Y130" t="str">
+        <x:v>https://github.com/chinahamu/japan-healthcare-mcp/blob/main/README.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="131">
+      <x:c r="A131" t="str">
+        <x:v>RWE-0198</x:v>
+      </x:c>
+      <x:c r="B131" t="str">
+        <x:v>Lab Results Analyzer MCP</x:v>
+      </x:c>
+      <x:c r="C131" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D131" t="str">
+        <x:v>Clinical Data &amp; Interoperability</x:v>
+      </x:c>
+      <x:c r="E131" t="str">
+        <x:v>FHIR-based lab-results retrieval, trend analysis, abnormal flagging, and patient-friendly summary generation across 20+ reference-range-backed common lab tests; built on Prompt Opinion's scoped-token FHIR context.</x:v>
+      </x:c>
+      <x:c r="F131" t="str">
+        <x:v>FHIR / clinical data | Interoperability | Governed access</x:v>
+      </x:c>
+      <x:c r="G131" t="str">
+        <x:v>Clinical-source inspection | Interoperability prototyping | Cohort and data-availability assessment</x:v>
+      </x:c>
+      <x:c r="H131" t="str">
+        <x:v>Retrieve lab results from a FHIR server for the current patient | Analyze trends in specific lab values over time (e.g., "Is glucose trending up?") | Generate patient-friendly summaries of recent lab work in plain language</x:v>
+      </x:c>
+      <x:c r="I131" t="str">
+        <x:v>Clinical systems can contain PHI and may expose write operations. Production use requires explicit authorization, least privilege, audit logging, retention controls, source-system validation, and organization-specific governance.</x:v>
+      </x:c>
+      <x:c r="J131" t="str">
+        <x:v>Static documentation and repository metadata reviewed.</x:v>
+      </x:c>
+      <x:c r="K131" t="str">
+        <x:v>Canonical public source resolved: https://github.com/JuanM94/mcp-lab-analyzer</x:v>
+      </x:c>
+      <x:c r="L131" t="str">
+        <x:v>Repository README and declared capability surface statically reviewed: https://github.com/JuanM94/mcp-lab-analyzer/blob/main/README.md</x:v>
+      </x:c>
+      <x:c r="M131" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N131" t="str">
+        <x:v>JuanM94</x:v>
+      </x:c>
+      <x:c r="O131" t="str">
+        <x:v>Not declared</x:v>
+      </x:c>
+      <x:c r="P131" t="str">
+        <x:v>Source repository</x:v>
+      </x:c>
+      <x:c r="Q131" t="str">
+        <x:v>See project documentation; transport was not independently tested</x:v>
+      </x:c>
+      <x:c r="R131" t="str">
+        <x:v>See project documentation; read/write scope was not independently tested</x:v>
+      </x:c>
+      <x:c r="S131" t="str">
+        <x:v>See project documentation; authentication was not independently tested</x:v>
+      </x:c>
+      <x:c r="T131" s="17" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="U131" s="17" t="n">
+        <x:v>46115</x:v>
+      </x:c>
+      <x:c r="V131" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W131" t="str">
+        <x:v>https://github.com/JuanM94/mcp-lab-analyzer</x:v>
+      </x:c>
+      <x:c r="X131" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="Y131" t="str">
+        <x:v>https://github.com/JuanM94/mcp-lab-analyzer/blob/main/README.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="132">
+      <x:c r="A132" t="str">
+        <x:v>RWE-0209</x:v>
+      </x:c>
+      <x:c r="B132" t="str">
+        <x:v>Pipeworx Medical Codes MCP</x:v>
+      </x:c>
+      <x:c r="C132" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D132" t="str">
+        <x:v>OMOP &amp; terminology</x:v>
+      </x:c>
+      <x:c r="E132" t="str">
+        <x:v>Keyless ICD-10, LOINC, and RxTerms clinical-term search via the Pipeworx hosted gateway or self-hosted; distinct from the offline cyanheads Medical Codes MCP under Revenue Cycle Management.</x:v>
+      </x:c>
+      <x:c r="F132" t="str">
+        <x:v>Terminology | Code lookup | Normalization</x:v>
+      </x:c>
+      <x:c r="G132" t="str">
+        <x:v>Concept-set development | Code validation | Data harmonization</x:v>
+      </x:c>
+      <x:c r="H132" t="str">
+        <x:v>Search documented codes or terminology sources | Retrieve concept metadata and identifiers | Support code validation or normalization workflows</x:v>
+      </x:c>
+      <x:c r="I132" t="str">
+        <x:v>Automated code lookup or mapping can omit descendants, include inappropriate concepts, or obscure local meaning. Vocabulary versions, licensing, hierarchy behavior, and study-specific concept sets require expert adjudication.</x:v>
+      </x:c>
+      <x:c r="J132" t="str">
+        <x:v>Static documentation and repository metadata reviewed.</x:v>
+      </x:c>
+      <x:c r="K132" t="str">
+        <x:v>Canonical public source resolved: https://github.com/pipeworx-io/mcp-medical-codes</x:v>
+      </x:c>
+      <x:c r="L132" t="str">
+        <x:v>Repository README and declared capability surface statically reviewed: https://github.com/pipeworx-io/mcp-medical-codes/blob/main/README.md</x:v>
+      </x:c>
+      <x:c r="M132" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N132" t="str">
+        <x:v>pipeworx-io</x:v>
+      </x:c>
+      <x:c r="O132" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P132" t="str">
+        <x:v>Source repository</x:v>
+      </x:c>
+      <x:c r="Q132" t="str">
+        <x:v>See project documentation; transport was not independently tested</x:v>
+      </x:c>
+      <x:c r="R132" t="str">
+        <x:v>See project documentation; read/write scope was not independently tested</x:v>
+      </x:c>
+      <x:c r="S132" t="str">
+        <x:v>See project documentation; authentication was not independently tested</x:v>
+      </x:c>
+      <x:c r="T132" s="17" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="U132" s="17" t="n">
+        <x:v>46238</x:v>
+      </x:c>
+      <x:c r="V132" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W132" t="str">
+        <x:v>https://github.com/pipeworx-io/mcp-medical-codes</x:v>
+      </x:c>
+      <x:c r="X132" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="Y132" t="str">
+        <x:v>https://github.com/pipeworx-io/mcp-medical-codes/blob/main/README.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="133">
+      <x:c r="A133" t="str">
+        <x:v>RWE-0244</x:v>
+      </x:c>
+      <x:c r="B133" t="str">
+        <x:v>RNAcentral MCP Server</x:v>
+      </x:c>
+      <x:c r="C133" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D133" t="str">
+        <x:v>Biomedical &amp; RWE Infrastructure</x:v>
+      </x:c>
+      <x:c r="E133" t="str">
+        <x:v>Official RNAcentral server for non-coding RNA search, sequence mapping, genomic analysis, and metadata retrieval across the consolidated ncRNA database; published on PyPI.</x:v>
+      </x:c>
+      <x:c r="F133" t="str">
+        <x:v>Biomedical data | Research infrastructure | Identifier resolution</x:v>
+      </x:c>
+      <x:c r="G133" t="str">
+        <x:v>Biomedical evidence enrichment | Identifier and dataset discovery | Translational context for RWE</x:v>
+      </x:c>
+      <x:c r="H133" t="str">
+        <x:v>Sequence Search: Search for RNA sequences across multiple databases to find identical or similar entries. | Bulk Sequence Export: Export search results in FASTA or Parquet formats, ideal for downstream analysis or machine learning datasets. | 2D Structure Diagrams: Retrieve secondary structure (2D) diagrams in SVG format for RNAs with known or predicted folds.</x:v>
+      </x:c>
+      <x:c r="I133" t="str">
+        <x:v>Biomedical, personal-health, or translational evidence does not by itself establish clinical effectiveness or causal validity. Source versions, identifiers, coverage, consent, licensing, and cross-database consistency require verification.</x:v>
+      </x:c>
+      <x:c r="J133" t="str">
+        <x:v>Static documentation and repository metadata reviewed.</x:v>
+      </x:c>
+      <x:c r="K133" t="str">
+        <x:v>Canonical public source resolved: https://github.com/RNAcentral/rnacentral-mcp-server</x:v>
+      </x:c>
+      <x:c r="L133" t="str">
+        <x:v>Repository README and declared capability surface statically reviewed: https://github.com/RNAcentral/rnacentral-mcp-server/blob/main/readme.md</x:v>
+      </x:c>
+      <x:c r="M133" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N133" t="str">
+        <x:v>RNAcentral</x:v>
+      </x:c>
+      <x:c r="O133" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P133" t="str">
+        <x:v>Source repository</x:v>
+      </x:c>
+      <x:c r="Q133" t="str">
+        <x:v>See project documentation; transport was not independently tested</x:v>
+      </x:c>
+      <x:c r="R133" t="str">
+        <x:v>See project documentation; read/write scope was not independently tested</x:v>
+      </x:c>
+      <x:c r="S133" t="str">
+        <x:v>See project documentation; authentication was not independently tested</x:v>
+      </x:c>
+      <x:c r="T133" s="17" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="U133" s="17" t="n">
+        <x:v>46179</x:v>
+      </x:c>
+      <x:c r="V133" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W133" t="str">
+        <x:v>https://github.com/RNAcentral/rnacentral-mcp-server</x:v>
+      </x:c>
+      <x:c r="X133" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="Y133" t="str">
+        <x:v>https://github.com/RNAcentral/rnacentral-mcp-server/blob/main/readme.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="134">
+      <x:c r="A134" t="str">
+        <x:v>RWE-0227</x:v>
+      </x:c>
+      <x:c r="B134" t="str">
+        <x:v>Secure FHIR MCP</x:v>
+      </x:c>
+      <x:c r="C134" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D134" t="str">
+        <x:v>Clinical Data &amp; Interoperability</x:v>
+      </x:c>
+      <x:c r="E134" t="str">
+        <x:v>HIPAA-hardened FHIR MCP with PHI masking, break-glass access, OWASP security, and audit logging.</x:v>
+      </x:c>
+      <x:c r="F134" t="str">
+        <x:v>FHIR / clinical data | Interoperability | Governed access</x:v>
+      </x:c>
+      <x:c r="G134" t="str">
+        <x:v>Clinical-source inspection | Interoperability prototyping | Cohort and data-availability assessment</x:v>
+      </x:c>
+      <x:c r="H134" t="str">
+        <x:v>📊 Comprehensive FHIR Support: Read, search, create, and update operations | 🏥 HL7 Terminology: ValueSet expansion, CodeSystem lookup, and concept translation | 🔧 Interoperable: Works with HAPI FHIR, Firely, and other R4/R4B servers</x:v>
+      </x:c>
+      <x:c r="I134" t="str">
+        <x:v>Clinical systems can contain PHI and may expose write operations. Production use requires explicit authorization, least privilege, audit logging, retention controls, source-system validation, and organization-specific governance.</x:v>
+      </x:c>
+      <x:c r="J134" t="str">
+        <x:v>Static documentation and repository metadata reviewed.</x:v>
+      </x:c>
+      <x:c r="K134" t="str">
+        <x:v>Canonical public source resolved: https://github.com/xSoVx/fhir-mcp</x:v>
+      </x:c>
+      <x:c r="L134" t="str">
+        <x:v>Repository README and declared capability surface statically reviewed: https://github.com/xSoVx/fhir-mcp/blob/master/README.md</x:v>
+      </x:c>
+      <x:c r="M134" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N134" t="str">
+        <x:v>xSoVx</x:v>
+      </x:c>
+      <x:c r="O134" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P134" t="str">
+        <x:v>Source repository</x:v>
+      </x:c>
+      <x:c r="Q134" t="str">
+        <x:v>See project documentation; transport was not independently tested</x:v>
+      </x:c>
+      <x:c r="R134" t="str">
+        <x:v>See project documentation; read/write scope was not independently tested</x:v>
+      </x:c>
+      <x:c r="S134" t="str">
+        <x:v>See project documentation; authentication was not independently tested</x:v>
+      </x:c>
+      <x:c r="T134" s="17" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="U134" s="17" t="n">
+        <x:v>45912</x:v>
+      </x:c>
+      <x:c r="V134" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W134" t="str">
+        <x:v>https://github.com/xSoVx/fhir-mcp</x:v>
+      </x:c>
+      <x:c r="X134" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="Y134" t="str">
+        <x:v>https://github.com/xSoVx/fhir-mcp/blob/master/README.md</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -6677,7 +10528,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ff42825c9cf4779"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R45d450cf979444b3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add DAG and study design WebMCP registry cards
</commit_message>
<xml_diff>
--- a/public-data/rwe-mcp-verified-capability-cards.xlsx
+++ b/public-data/rwe-mcp-verified-capability-cards.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verified RWE Capability Cards" sheetId="1" r:id="Rf41ef0355b9e4062"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verified RWE Capability Cards" sheetId="1" r:id="R837546b434314108"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -75,7 +75,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="18">
+  <x:cellXfs count="19">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -114,6 +114,9 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -122,7 +125,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ReviewedCapabilityCards" displayName="ReviewedCapabilityCards" ref="A4:Y134" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ReviewedCapabilityCards" displayName="ReviewedCapabilityCards" ref="A4:Y136" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="25">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Name"/>
@@ -378,7 +381,7 @@
   <x:sheetData>
     <x:row r="1" ht="36" customHeight="1">
       <x:c r="A1" s="2" t="str">
-        <x:v>RWE MCP Registry — 130 Reviewed Capability Cards</x:v>
+        <x:v>RWE MCP Registry — 132 Reviewed Capability Cards</x:v>
       </x:c>
       <x:c r="B1" s="2"/>
       <x:c r="C1" s="2"/>
@@ -407,7 +410,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="5" t="str">
-        <x:v>Source-reviewed catalogue for RWE workflows · identity and static documentation review only · no installation, runtime, security, privacy, clinical, methodological, or regulatory validation · CC BY 4.0 · reviewed 2026-08-25</x:v>
+        <x:v>Source-reviewed catalogue for RWE workflows · identity and static review only · no independent runtime or methodological validation · CC BY 4.0 · WebMCP additions reviewed 2026-09-06; prior entries retain their review dates</x:v>
       </x:c>
       <x:c r="B2" s="5"/>
       <x:c r="C2" s="5"/>
@@ -10521,6 +10524,160 @@
         <x:v>https://github.com/xSoVx/fhir-mcp/blob/master/README.md</x:v>
       </x:c>
     </x:row>
+    <x:row r="135" ht="145.1999969482422" hidden="0" customHeight="1">
+      <x:c r="A135" s="11" t="str">
+        <x:v>RWE-0257</x:v>
+      </x:c>
+      <x:c r="B135" s="11" t="str">
+        <x:v>DAG Studio WebMCP</x:v>
+      </x:c>
+      <x:c r="C135" s="11" t="str">
+        <x:v>WebMCP + remote MCP bridge</x:v>
+      </x:c>
+      <x:c r="D135" s="11" t="str">
+        <x:v>Causal Inference &amp; Analytics</x:v>
+      </x:c>
+      <x:c r="E135" s="11" t="str">
+        <x:v>Shared causal DAG canvas where a researcher and an agent inspect, edit, analyze, and simulate the same graph through nine predefined tools.</x:v>
+      </x:c>
+      <x:c r="F135" s="11" t="str">
+        <x:v>Live DAG canvas | Adjustment sets | WebMCP</x:v>
+      </x:c>
+      <x:c r="G135" s="11" t="str">
+        <x:v>Causal-assumption review | Adjustment-set exploration | Study-design collaboration</x:v>
+      </x:c>
+      <x:c r="H135" s="11" t="str">
+        <x:v>Read the live DAG and make visible, undoable node and edge edits | Analyze backdoor paths and adjustment sets; generate R or Python code | Simulate linear Gaussian SEM data under the encoded graph assumptions</x:v>
+      </x:c>
+      <x:c r="I135" s="11" t="str">
+        <x:v>Causal conclusions depend on researcher-supplied assumptions. This canvas integration is distinct from dagstudio-mcp. Remote use requires Connect MCP, a custom Authorization header, and an open tab; keys expire after two hours and study content passes through a relay to the agent provider.</x:v>
+      </x:c>
+      <x:c r="J135" s="11" t="str">
+        <x:v>Static documentation, tool definitions, and official registry metadata reviewed</x:v>
+      </x:c>
+      <x:c r="K135" s="11" t="str">
+        <x:v>Canonical source and active official listing confirmed: io.github.Black-Swan-Causal-Labs/dag-studio-webmcp</x:v>
+      </x:c>
+      <x:c r="L135" s="11" t="str">
+        <x:v>README, bridge documentation and tool definitions reviewed. https://github.com/Black-Swan-Causal-Labs/dag-studio-webmcp/blob/main/README.md | https://github.com/Black-Swan-Causal-Labs/dag-studio-webmcp/blob/main/webmcp-tools.js | https://github.com/Black-Swan-Causal-Labs/dag-studio-webmcp/blob/main/mcp-bridge/README.md | https://registry.modelcontextprotocol.io/v0.1/servers/io.github.Black-Swan-Causal-Labs%2Fdag-studio-webmcp/versions/latest</x:v>
+      </x:c>
+      <x:c r="M135" s="11" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N135" s="11" t="str">
+        <x:v>Black Swan Causal Labs</x:v>
+      </x:c>
+      <x:c r="O135" s="11" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P135" s="11" t="str">
+        <x:v>io.github.Black-Swan-Causal-Labs/dag-studio-webmcp 1.0.0</x:v>
+      </x:c>
+      <x:c r="Q135" s="11" t="str">
+        <x:v>Native WebMCP; optional Streamable HTTP bridge</x:v>
+      </x:c>
+      <x:c r="R135" s="11" t="str">
+        <x:v>Read and write current browser canvas; undoable edits</x:v>
+      </x:c>
+      <x:c r="S135" s="11" t="str">
+        <x:v>Opt-in Connect MCP; Authorization bearer key; open tab; two-hour expiry</x:v>
+      </x:c>
+      <x:c r="T135" s="14" t="n">
+        <x:v>46271</x:v>
+      </x:c>
+      <x:c r="U135" s="14" t="n">
+        <x:v>46272.258263888885</x:v>
+      </x:c>
+      <x:c r="V135" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W135" s="11" t="str">
+        <x:v>https://github.com/Black-Swan-Causal-Labs/dag-studio-webmcp</x:v>
+      </x:c>
+      <x:c r="X135" s="11" t="str">
+        <x:v>https://dag-studio-webmcp-sandbox.pages.dev</x:v>
+      </x:c>
+      <x:c r="Y135" s="11" t="str">
+        <x:v>https://github.com/Black-Swan-Causal-Labs/dag-studio-webmcp/blob/main/README.md | https://github.com/Black-Swan-Causal-Labs/dag-studio-webmcp/blob/main/webmcp-tools.js | https://github.com/Black-Swan-Causal-Labs/dag-studio-webmcp/blob/main/mcp-bridge/README.md | https://registry.modelcontextprotocol.io/v0.1/servers/io.github.Black-Swan-Causal-Labs%2Fdag-studio-webmcp/versions/latest</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="136" ht="145.1999969482422" hidden="0" customHeight="1">
+      <x:c r="A136" s="11" t="str">
+        <x:v>RWE-0258</x:v>
+      </x:c>
+      <x:c r="B136" s="11" t="str">
+        <x:v>Study Design Diagram Studio WebMCP</x:v>
+      </x:c>
+      <x:c r="C136" s="11" t="str">
+        <x:v>WebMCP + remote MCP bridge</x:v>
+      </x:c>
+      <x:c r="D136" s="11" t="str">
+        <x:v>Trials &amp; Study Design</x:v>
+      </x:c>
+      <x:c r="E136" s="11" t="str">
+        <x:v>Shared epidemiologic study-design workspace exposing ten tools for timeline windows, study details, completeness review, and SVG schematic export.</x:v>
+      </x:c>
+      <x:c r="F136" s="11" t="str">
+        <x:v>Study-design timelines | Assessment windows | WebMCP</x:v>
+      </x:c>
+      <x:c r="G136" s="11" t="str">
+        <x:v>Protocol-to-diagram specification | Time-zero and assessment-window review | Study-design communication</x:v>
+      </x:c>
+      <x:c r="H136" s="11" t="str">
+        <x:v>Read and edit washout, eligibility, covariate, and follow-up windows relative to an index event | Update study details, reorder rows, and import or clear designs with revision checks and Undo | Check information completeness and return an SVG schematic; the manual UI also exports JSON, PDF, and editable PowerPoint</x:v>
+      </x:c>
+      <x:c r="I136" s="11" t="str">
+        <x:v>Completeness checks do not establish methodological validity or source accuracy, and the app does not extract PDFs. Save JSON to preserve session-only edits. Remote use requires an open tab and a temporary Authorization key; content passes through a relay. No application-source license is granted.</x:v>
+      </x:c>
+      <x:c r="J136" s="11" t="str">
+        <x:v>Static documentation, tool definitions, and official registry metadata reviewed</x:v>
+      </x:c>
+      <x:c r="K136" s="11" t="str">
+        <x:v>Canonical source and active official listing confirmed: io.github.Black-Swan-Causal-Labs/sdds-webmcp</x:v>
+      </x:c>
+      <x:c r="L136" s="11" t="str">
+        <x:v>README, bridge documentation and tool definitions reviewed. https://github.com/Black-Swan-Causal-Labs/study-design-diagram-studio/blob/main/README.md | https://github.com/Black-Swan-Causal-Labs/study-design-diagram-studio/blob/main/lib/study/webmcp.ts | https://github.com/Black-Swan-Causal-Labs/study-design-diagram-studio/blob/main/mcp-bridge/README.md | https://registry.modelcontextprotocol.io/v0.1/servers/io.github.Black-Swan-Causal-Labs%2Fsdds-webmcp/versions/latest</x:v>
+      </x:c>
+      <x:c r="M136" s="11" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N136" s="11" t="str">
+        <x:v>Black Swan Causal Labs</x:v>
+      </x:c>
+      <x:c r="O136" s="11" t="str">
+        <x:v>No application-source license granted</x:v>
+      </x:c>
+      <x:c r="P136" s="11" t="str">
+        <x:v>io.github.Black-Swan-Causal-Labs/sdds-webmcp 1.0.0</x:v>
+      </x:c>
+      <x:c r="Q136" s="11" t="str">
+        <x:v>Native WebMCP; optional Streamable HTTP bridge</x:v>
+      </x:c>
+      <x:c r="R136" s="11" t="str">
+        <x:v>Read and write current browser canvas; undoable edits</x:v>
+      </x:c>
+      <x:c r="S136" s="11" t="str">
+        <x:v>Opt-in Connect MCP; Authorization bearer key; open tab; two-hour expiry</x:v>
+      </x:c>
+      <x:c r="T136" s="14" t="n">
+        <x:v>46271</x:v>
+      </x:c>
+      <x:c r="U136" s="14" t="n">
+        <x:v>46272.262604166666</x:v>
+      </x:c>
+      <x:c r="V136" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W136" s="11" t="str">
+        <x:v>https://github.com/Black-Swan-Causal-Labs/study-design-diagram-studio</x:v>
+      </x:c>
+      <x:c r="X136" s="11" t="str">
+        <x:v>https://sdds.blackswancausallabs.com</x:v>
+      </x:c>
+      <x:c r="Y136" s="11" t="str">
+        <x:v>https://github.com/Black-Swan-Causal-Labs/study-design-diagram-studio/blob/main/README.md | https://github.com/Black-Swan-Causal-Labs/study-design-diagram-studio/blob/main/lib/study/webmcp.ts | https://github.com/Black-Swan-Causal-Labs/study-design-diagram-studio/blob/main/mcp-bridge/README.md | https://registry.modelcontextprotocol.io/v0.1/servers/io.github.Black-Swan-Causal-Labs%2Fsdds-webmcp/versions/latest</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:Y1"/>
@@ -10528,7 +10685,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R45d450cf979444b3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a435f362f484d89"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add 45 reviewed RWE capabilities from 59-candidate pass
</commit_message>
<xml_diff>
--- a/public-data/rwe-mcp-verified-capability-cards.xlsx
+++ b/public-data/rwe-mcp-verified-capability-cards.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verified RWE Capability Cards" sheetId="1" r:id="R837546b434314108"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verified RWE Capability Cards" sheetId="1" r:id="Rac84e77290254ea8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -125,7 +125,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ReviewedCapabilityCards" displayName="ReviewedCapabilityCards" ref="A4:Y136" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ReviewedCapabilityCards" displayName="ReviewedCapabilityCards" ref="A4:Y181" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="25">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Name"/>
@@ -381,7 +381,7 @@
   <x:sheetData>
     <x:row r="1" ht="36" customHeight="1">
       <x:c r="A1" s="2" t="str">
-        <x:v>RWE MCP Registry — 132 Reviewed Capability Cards</x:v>
+        <x:v>RWE MCP Registry — 177 Reviewed Capability Cards</x:v>
       </x:c>
       <x:c r="B1" s="2"/>
       <x:c r="C1" s="2"/>
@@ -410,7 +410,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="5" t="str">
-        <x:v>Source-reviewed catalogue for RWE workflows · identity and static review only · no independent runtime or methodological validation · CC BY 4.0 · WebMCP additions reviewed 2026-09-06; prior entries retain their review dates</x:v>
+        <x:v>Source-reviewed catalogue for RWE workflows · identity and static review only · no independent runtime or methodological validation · CC BY 4.0 · 45 additions reviewed 2026-09-07 UTC; prior entries retain their review dates</x:v>
       </x:c>
       <x:c r="B2" s="5"/>
       <x:c r="C2" s="5"/>
@@ -10678,6 +10678,3471 @@
         <x:v>https://github.com/Black-Swan-Causal-Labs/study-design-diagram-studio/blob/main/README.md | https://github.com/Black-Swan-Causal-Labs/study-design-diagram-studio/blob/main/lib/study/webmcp.ts | https://github.com/Black-Swan-Causal-Labs/study-design-diagram-studio/blob/main/mcp-bridge/README.md | https://registry.modelcontextprotocol.io/v0.1/servers/io.github.Black-Swan-Causal-Labs%2Fsdds-webmcp/versions/latest</x:v>
       </x:c>
     </x:row>
+    <x:row r="137" ht="118.80000305175781" hidden="0" customHeight="1">
+      <x:c r="A137" s="11" t="str">
+        <x:v>RWE-0010</x:v>
+      </x:c>
+      <x:c r="B137" s="11" t="str">
+        <x:v>Tebra MCP Server</x:v>
+      </x:c>
+      <x:c r="C137" s="11" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D137" s="11" t="str">
+        <x:v>Clinical Data &amp; Interoperability</x:v>
+      </x:c>
+      <x:c r="E137" s="11" t="str">
+        <x:v>Connects agents to Tebra clinical and practice records through SOAP and FHIR interfaces.</x:v>
+      </x:c>
+      <x:c r="F137" s="11" t="str">
+        <x:v>Clinical Data | MCP server</x:v>
+      </x:c>
+      <x:c r="G137" s="11" t="str">
+        <x:v>Clinical Data &amp; Interoperability | Source inspection and research preparation</x:v>
+      </x:c>
+      <x:c r="H137" s="11" t="str">
+        <x:v>Retrieve patients, encounters, clinical documents and related records | Expose SOAP operations and optional FHIR access to agent workflows</x:v>
+      </x:c>
+      <x:c r="I137" s="11" t="str">
+        <x:v>Includes write operations and identifiable clinical data. Practice records require research permissions, population definitions and quality assessment before reuse.</x:v>
+      </x:c>
+      <x:c r="J137" s="11" t="str">
+        <x:v>Static source and documentation reviewed</x:v>
+      </x:c>
+      <x:c r="K137" s="11" t="str">
+        <x:v>Canonical repository metadata reviewed at commit 0ad77451f4a089ea66e580bdde0fb9a02be603a6</x:v>
+      </x:c>
+      <x:c r="L137" s="11" t="str">
+        <x:v>https://github.com/jamesrosing/tebra-mcp-server/blob/0ad77451f4a089ea66e580bdde0fb9a02be603a6/README.md | https://github.com/jamesrosing/tebra-mcp-server/blob/0ad77451f4a089ea66e580bdde0fb9a02be603a6/package.json | https://github.com/jamesrosing/tebra-mcp-server/blob/0ad77451f4a089ea66e580bdde0fb9a02be603a6/server.json | https://github.com/jamesrosing/tebra-mcp-server/blob/0ad77451f4a089ea66e580bdde0fb9a02be603a6/skills/tebra/SKILL.md</x:v>
+      </x:c>
+      <x:c r="M137" s="11" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N137" s="11" t="str">
+        <x:v>jamesrosing</x:v>
+      </x:c>
+      <x:c r="O137" s="11" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P137" s="11" t="str">
+        <x:v>See pinned project manifest and setup documentation</x:v>
+      </x:c>
+      <x:c r="Q137" s="11" t="str">
+        <x:v>See pinned setup; varies by component</x:v>
+      </x:c>
+      <x:c r="R137" s="11" t="str">
+        <x:v>See capability and limitation fields; no runtime actions performed</x:v>
+      </x:c>
+      <x:c r="S137" s="11" t="str">
+        <x:v>Tebra SOAP credentials and customer key; optional SMART on FHIR credentials.</x:v>
+      </x:c>
+      <x:c r="T137" s="14" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+      <x:c r="U137" s="14" t="n">
+        <x:v>46271.770150462966</x:v>
+      </x:c>
+      <x:c r="V137" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="W137" s="11" t="str">
+        <x:v>https://github.com/jamesrosing/tebra-mcp-server</x:v>
+      </x:c>
+      <x:c r="X137" s="11" t="str">
+        <x:v>https://github.com/jamesrosing/tebra-mcp-server</x:v>
+      </x:c>
+      <x:c r="Y137" s="11" t="str">
+        <x:v>https://github.com/jamesrosing/tebra-mcp-server/blob/0ad77451f4a089ea66e580bdde0fb9a02be603a6/README.md | https://github.com/jamesrosing/tebra-mcp-server/blob/0ad77451f4a089ea66e580bdde0fb9a02be603a6/package.json | https://github.com/jamesrosing/tebra-mcp-server/blob/0ad77451f4a089ea66e580bdde0fb9a02be603a6/server.json | https://github.com/jamesrosing/tebra-mcp-server/blob/0ad77451f4a089ea66e580bdde0fb9a02be603a6/skills/tebra/SKILL.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="138" ht="184.8000030517578" hidden="0" customHeight="1">
+      <x:c r="A138" s="11" t="str">
+        <x:v>RWE-0021</x:v>
+      </x:c>
+      <x:c r="B138" s="11" t="str">
+        <x:v>Healthcare FHIR MCP (CSOAI)</x:v>
+      </x:c>
+      <x:c r="C138" s="11" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D138" s="11" t="str">
+        <x:v>Clinical Data &amp; Interoperability</x:v>
+      </x:c>
+      <x:c r="E138" s="11" t="str">
+        <x:v>FHIR connector exposing clinical resource queries and workflow operations.</x:v>
+      </x:c>
+      <x:c r="F138" s="11" t="str">
+        <x:v>Clinical Data | MCP server</x:v>
+      </x:c>
+      <x:c r="G138" s="11" t="str">
+        <x:v>Clinical Data &amp; Interoperability | Source inspection and research preparation</x:v>
+      </x:c>
+      <x:c r="H138" s="11" t="str">
+        <x:v>Query patient and clinical resources from a configured FHIR endpoint | Expose FHIR workflow tools with a separate service-metering layer</x:v>
+      </x:c>
+      <x:c r="I138" s="11" t="str">
+        <x:v>Source review does not substantiate compliance claims. Metering middleware fails open and is not a patient-data authorization boundary; enforce access at the FHIR service.</x:v>
+      </x:c>
+      <x:c r="J138" s="11" t="str">
+        <x:v>Static source and documentation reviewed</x:v>
+      </x:c>
+      <x:c r="K138" s="11" t="str">
+        <x:v>Canonical repository metadata reviewed at commit e61c14881f22cd4a4f8e17d50ff1487d9a637901</x:v>
+      </x:c>
+      <x:c r="L138" s="11" t="str">
+        <x:v>https://github.com/CSOAI-ORG/healthcare-fhir-mcp/blob/e61c14881f22cd4a4f8e17d50ff1487d9a637901/README.md | https://github.com/CSOAI-ORG/healthcare-fhir-mcp/blob/e61c14881f22cd4a4f8e17d50ff1487d9a637901/package.json | https://github.com/CSOAI-ORG/healthcare-fhir-mcp/blob/e61c14881f22cd4a4f8e17d50ff1487d9a637901/pyproject.toml | https://github.com/CSOAI-ORG/healthcare-fhir-mcp/blob/e61c14881f22cd4a4f8e17d50ff1487d9a637901/server.json | https://github.com/CSOAI-ORG/healthcare-fhir-mcp/blob/e61c14881f22cd4a4f8e17d50ff1487d9a637901/server.py | https://github.com/CSOAI-ORG/healthcare-fhir-mcp/blob/e61c14881f22cd4a4f8e17d50ff1487d9a637901/auth_middleware.py</x:v>
+      </x:c>
+      <x:c r="M138" s="11" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N138" s="11" t="str">
+        <x:v>CSOAI-ORG</x:v>
+      </x:c>
+      <x:c r="O138" s="11" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P138" s="11" t="str">
+        <x:v>See pinned project manifest and setup documentation</x:v>
+      </x:c>
+      <x:c r="Q138" s="11" t="str">
+        <x:v>See pinned setup; varies by component</x:v>
+      </x:c>
+      <x:c r="R138" s="11" t="str">
+        <x:v>See capability and limitation fields; no runtime actions performed</x:v>
+      </x:c>
+      <x:c r="S138" s="11" t="str">
+        <x:v>FHIR endpoint configuration; optional MEOK service key with external verification.</x:v>
+      </x:c>
+      <x:c r="T138" s="14" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+      <x:c r="U138" s="14" t="n">
+        <x:v>46269.52755787037</x:v>
+      </x:c>
+      <x:c r="V138" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W138" s="11" t="str">
+        <x:v>https://github.com/CSOAI-ORG/healthcare-fhir-mcp</x:v>
+      </x:c>
+      <x:c r="X138" s="11" t="str">
+        <x:v>https://github.com/CSOAI-ORG/healthcare-fhir-mcp</x:v>
+      </x:c>
+      <x:c r="Y138" s="11" t="str">
+        <x:v>https://github.com/CSOAI-ORG/healthcare-fhir-mcp/blob/e61c14881f22cd4a4f8e17d50ff1487d9a637901/README.md | https://github.com/CSOAI-ORG/healthcare-fhir-mcp/blob/e61c14881f22cd4a4f8e17d50ff1487d9a637901/package.json | https://github.com/CSOAI-ORG/healthcare-fhir-mcp/blob/e61c14881f22cd4a4f8e17d50ff1487d9a637901/pyproject.toml | https://github.com/CSOAI-ORG/healthcare-fhir-mcp/blob/e61c14881f22cd4a4f8e17d50ff1487d9a637901/server.json | https://github.com/CSOAI-ORG/healthcare-fhir-mcp/blob/e61c14881f22cd4a4f8e17d50ff1487d9a637901/server.py | https://github.com/CSOAI-ORG/healthcare-fhir-mcp/blob/e61c14881f22cd4a4f8e17d50ff1487d9a637901/auth_middleware.py</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="139" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A139" s="11" t="str">
+        <x:v>RWE-0090</x:v>
+      </x:c>
+      <x:c r="B139" s="11" t="str">
+        <x:v>Withings MCP</x:v>
+      </x:c>
+      <x:c r="C139" s="11" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D139" s="11" t="str">
+        <x:v>Clinical Data &amp; Interoperability</x:v>
+      </x:c>
+      <x:c r="E139" s="11" t="str">
+        <x:v>Retrieves account-level Withings measurements and wearable time series.</x:v>
+      </x:c>
+      <x:c r="F139" s="11" t="str">
+        <x:v>Clinical Data | MCP server</x:v>
+      </x:c>
+      <x:c r="G139" s="11" t="str">
+        <x:v>Clinical Data &amp; Interoperability | Source inspection and research preparation</x:v>
+      </x:c>
+      <x:c r="H139" s="11" t="str">
+        <x:v>Retrieve activity, sleep and body measurements | Access supported heart-rate, HRV and ECG account records</x:v>
+      </x:c>
+      <x:c r="I139" s="11" t="str">
+        <x:v>Availability depends on device and account scopes. Proprietary measurements need validation for the intended endpoint; a personal account is not a representative cohort.</x:v>
+      </x:c>
+      <x:c r="J139" s="11" t="str">
+        <x:v>Static source and documentation reviewed</x:v>
+      </x:c>
+      <x:c r="K139" s="11" t="str">
+        <x:v>Canonical repository metadata reviewed at commit 3a78c2eee6d52f1efa8dc247fdfce23b7f293f8c</x:v>
+      </x:c>
+      <x:c r="L139" s="11" t="str">
+        <x:v>https://github.com/akutishevsky/withings-mcp/blob/3a78c2eee6d52f1efa8dc247fdfce23b7f293f8c/README.md | https://github.com/akutishevsky/withings-mcp/blob/3a78c2eee6d52f1efa8dc247fdfce23b7f293f8c/package.json | https://github.com/akutishevsky/withings-mcp/blob/3a78c2eee6d52f1efa8dc247fdfce23b7f293f8c/server.json</x:v>
+      </x:c>
+      <x:c r="M139" s="11" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N139" s="11" t="str">
+        <x:v>akutishevsky</x:v>
+      </x:c>
+      <x:c r="O139" s="11" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P139" s="11" t="str">
+        <x:v>See pinned project manifest and setup documentation</x:v>
+      </x:c>
+      <x:c r="Q139" s="11" t="str">
+        <x:v>See pinned setup; varies by component</x:v>
+      </x:c>
+      <x:c r="R139" s="11" t="str">
+        <x:v>See capability and limitation fields; no runtime actions performed</x:v>
+      </x:c>
+      <x:c r="S139" s="11" t="str">
+        <x:v>Withings OAuth application and authorized user account.</x:v>
+      </x:c>
+      <x:c r="T139" s="14" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+      <x:c r="U139" s="14" t="n">
+        <x:v>46264.33883101852</x:v>
+      </x:c>
+      <x:c r="V139" s="11" t="n">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="W139" s="11" t="str">
+        <x:v>https://github.com/akutishevsky/withings-mcp</x:v>
+      </x:c>
+      <x:c r="X139" s="11" t="str">
+        <x:v>https://github.com/akutishevsky/withings-mcp</x:v>
+      </x:c>
+      <x:c r="Y139" s="11" t="str">
+        <x:v>https://github.com/akutishevsky/withings-mcp/blob/3a78c2eee6d52f1efa8dc247fdfce23b7f293f8c/README.md | https://github.com/akutishevsky/withings-mcp/blob/3a78c2eee6d52f1efa8dc247fdfce23b7f293f8c/package.json | https://github.com/akutishevsky/withings-mcp/blob/3a78c2eee6d52f1efa8dc247fdfce23b7f293f8c/server.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="140" ht="224.39999389648438" hidden="0" customHeight="1">
+      <x:c r="A140" s="11" t="str">
+        <x:v>RWE-0004</x:v>
+      </x:c>
+      <x:c r="B140" s="11" t="str">
+        <x:v>ENCODE Toolkit</x:v>
+      </x:c>
+      <x:c r="C140" s="11" t="str">
+        <x:v>MCP server + skill collection</x:v>
+      </x:c>
+      <x:c r="D140" s="11" t="str">
+        <x:v>Biomedical &amp; RWE Infrastructure</x:v>
+      </x:c>
+      <x:c r="E140" s="11" t="str">
+        <x:v>Combines ENCODE MCP tools with bioinformatics skills for functional-genomics research.</x:v>
+      </x:c>
+      <x:c r="F140" s="11" t="str">
+        <x:v>Biomedical | MCP server + skill collection</x:v>
+      </x:c>
+      <x:c r="G140" s="11" t="str">
+        <x:v>Biomedical &amp; RWE Infrastructure | Source inspection and research preparation</x:v>
+      </x:c>
+      <x:c r="H140" s="11" t="str">
+        <x:v>Search ENCODE experiments and retrieve metadata and files | Track experiments and citations; guide downstream bioinformatics workflows</x:v>
+      </x:c>
+      <x:c r="I140" s="11" t="str">
+        <x:v>Additional database integrations are skills or external dependencies, not all built-in MCP tools. Functional-genomics results do not by themselves establish patient-level causal effects.</x:v>
+      </x:c>
+      <x:c r="J140" s="11" t="str">
+        <x:v>Static source and documentation reviewed</x:v>
+      </x:c>
+      <x:c r="K140" s="11" t="str">
+        <x:v>Canonical repository metadata reviewed at commit b1d90bc9e7ead40d49b8c89f0b9b9e7b8e592a5b</x:v>
+      </x:c>
+      <x:c r="L140" s="11" t="str">
+        <x:v>https://github.com/ammawla/encode-toolkit/blob/b1d90bc9e7ead40d49b8c89f0b9b9e7b8e592a5b/README.md | https://github.com/ammawla/encode-toolkit/blob/b1d90bc9e7ead40d49b8c89f0b9b9e7b8e592a5b/package.json | https://github.com/ammawla/encode-toolkit/blob/b1d90bc9e7ead40d49b8c89f0b9b9e7b8e592a5b/pyproject.toml | https://github.com/ammawla/encode-toolkit/blob/b1d90bc9e7ead40d49b8c89f0b9b9e7b8e592a5b/server.json | https://github.com/ammawla/encode-toolkit/blob/b1d90bc9e7ead40d49b8c89f0b9b9e7b8e592a5b/plugin/skills/accessibility-aggregation/SKILL.md | https://github.com/ammawla/encode-toolkit/blob/b1d90bc9e7ead40d49b8c89f0b9b9e7b8e592a5b/plugin/skills/batch-analysis/SKILL.md | https://github.com/ammawla/encode-toolkit/blob/b1d90bc9e7ead40d49b8c89f0b9b9e7b8e592a5b/plugin/skills/bioinformatics-installer/SKILL.md</x:v>
+      </x:c>
+      <x:c r="M140" s="11" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N140" s="11" t="str">
+        <x:v>ammawla</x:v>
+      </x:c>
+      <x:c r="O140" s="11" t="str">
+        <x:v>AGPL-3.0</x:v>
+      </x:c>
+      <x:c r="P140" s="11" t="str">
+        <x:v>See pinned project manifest and setup documentation</x:v>
+      </x:c>
+      <x:c r="Q140" s="11" t="str">
+        <x:v>See pinned setup; varies by component</x:v>
+      </x:c>
+      <x:c r="R140" s="11" t="str">
+        <x:v>See capability and limitation fields; no runtime actions performed</x:v>
+      </x:c>
+      <x:c r="S140" s="11" t="str">
+        <x:v>See pinned project setup; external data access may require credentials.</x:v>
+      </x:c>
+      <x:c r="T140" s="14" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+      <x:c r="U140" s="14" t="n">
+        <x:v>46229.057118055556</x:v>
+      </x:c>
+      <x:c r="V140" s="11" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="W140" s="11" t="str">
+        <x:v>https://github.com/ammawla/encode-toolkit</x:v>
+      </x:c>
+      <x:c r="X140" s="11" t="str">
+        <x:v>https://github.com/ammawla/encode-toolkit</x:v>
+      </x:c>
+      <x:c r="Y140" s="11" t="str">
+        <x:v>https://github.com/ammawla/encode-toolkit/blob/b1d90bc9e7ead40d49b8c89f0b9b9e7b8e592a5b/README.md | https://github.com/ammawla/encode-toolkit/blob/b1d90bc9e7ead40d49b8c89f0b9b9e7b8e592a5b/package.json | https://github.com/ammawla/encode-toolkit/blob/b1d90bc9e7ead40d49b8c89f0b9b9e7b8e592a5b/pyproject.toml | https://github.com/ammawla/encode-toolkit/blob/b1d90bc9e7ead40d49b8c89f0b9b9e7b8e592a5b/server.json | https://github.com/ammawla/encode-toolkit/blob/b1d90bc9e7ead40d49b8c89f0b9b9e7b8e592a5b/plugin/skills/accessibility-aggregation/SKILL.md | https://github.com/ammawla/encode-toolkit/blob/b1d90bc9e7ead40d49b8c89f0b9b9e7b8e592a5b/plugin/skills/batch-analysis/SKILL.md | https://github.com/ammawla/encode-toolkit/blob/b1d90bc9e7ead40d49b8c89f0b9b9e7b8e592a5b/plugin/skills/bioinformatics-installer/SKILL.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="141" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A141" s="11" t="str">
+        <x:v>RWE-0249</x:v>
+      </x:c>
+      <x:c r="B141" s="11" t="str">
+        <x:v>Apple Health MCP Server (Momentum)</x:v>
+      </x:c>
+      <x:c r="C141" s="11" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D141" s="11" t="str">
+        <x:v>Clinical Data &amp; Interoperability</x:v>
+      </x:c>
+      <x:c r="E141" s="11" t="str">
+        <x:v>Queries imported Apple Health export data using a local DuckDB workflow.</x:v>
+      </x:c>
+      <x:c r="F141" s="11" t="str">
+        <x:v>Clinical Data | MCP server</x:v>
+      </x:c>
+      <x:c r="G141" s="11" t="str">
+        <x:v>Clinical Data &amp; Interoperability | Source inspection and research preparation</x:v>
+      </x:c>
+      <x:c r="H141" s="11" t="str">
+        <x:v>Import Apple Health export records | Query measurements and time series through SQL-oriented tools</x:v>
+      </x:c>
+      <x:c r="I141" s="11" t="str">
+        <x:v>Exports contain sensitive personal data. Check units, device provenance, missingness and time zones; agent-generated SQL and derived summaries need review.</x:v>
+      </x:c>
+      <x:c r="J141" s="11" t="str">
+        <x:v>Static source and documentation reviewed</x:v>
+      </x:c>
+      <x:c r="K141" s="11" t="str">
+        <x:v>Canonical repository metadata reviewed at commit 638e05a2451a6fb6e5e619e9f49a3052e0e99985</x:v>
+      </x:c>
+      <x:c r="L141" s="11" t="str">
+        <x:v>https://github.com/the-momentum/apple-health-mcp-server/blob/638e05a2451a6fb6e5e619e9f49a3052e0e99985/README.md | https://github.com/the-momentum/apple-health-mcp-server/blob/638e05a2451a6fb6e5e619e9f49a3052e0e99985/pyproject.toml</x:v>
+      </x:c>
+      <x:c r="M141" s="11" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N141" s="11" t="str">
+        <x:v>the-momentum</x:v>
+      </x:c>
+      <x:c r="O141" s="11" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P141" s="11" t="str">
+        <x:v>See pinned project manifest and setup documentation</x:v>
+      </x:c>
+      <x:c r="Q141" s="11" t="str">
+        <x:v>See pinned setup; varies by component</x:v>
+      </x:c>
+      <x:c r="R141" s="11" t="str">
+        <x:v>See capability and limitation fields; no runtime actions performed</x:v>
+      </x:c>
+      <x:c r="S141" s="11" t="str">
+        <x:v>See pinned project setup; external data access may require credentials.</x:v>
+      </x:c>
+      <x:c r="T141" s="14" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+      <x:c r="U141" s="14" t="n">
+        <x:v>46212.45636574074</x:v>
+      </x:c>
+      <x:c r="V141" s="11" t="n">
+        <x:v>264</x:v>
+      </x:c>
+      <x:c r="W141" s="11" t="str">
+        <x:v>https://github.com/the-momentum/apple-health-mcp-server</x:v>
+      </x:c>
+      <x:c r="X141" s="11" t="str">
+        <x:v>https://github.com/the-momentum/apple-health-mcp-server</x:v>
+      </x:c>
+      <x:c r="Y141" s="11" t="str">
+        <x:v>https://github.com/the-momentum/apple-health-mcp-server/blob/638e05a2451a6fb6e5e619e9f49a3052e0e99985/README.md | https://github.com/the-momentum/apple-health-mcp-server/blob/638e05a2451a6fb6e5e619e9f49a3052e0e99985/pyproject.toml</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="142" ht="92.4000015258789" hidden="0" customHeight="1">
+      <x:c r="A142" s="11" t="str">
+        <x:v>RWE-0192</x:v>
+      </x:c>
+      <x:c r="B142" s="11" t="str">
+        <x:v>DaktariTB MCP</x:v>
+      </x:c>
+      <x:c r="C142" s="11" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D142" s="11" t="str">
+        <x:v>Clinical Data &amp; Interoperability</x:v>
+      </x:c>
+      <x:c r="E142" s="11" t="str">
+        <x:v>Connects TB and HIV clinical workflows to FHIR records and associated care operations.</x:v>
+      </x:c>
+      <x:c r="F142" s="11" t="str">
+        <x:v>Clinical Data | MCP server</x:v>
+      </x:c>
+      <x:c r="G142" s="11" t="str">
+        <x:v>Clinical Data &amp; Interoperability | Source inspection and research preparation</x:v>
+      </x:c>
+      <x:c r="H142" s="11" t="str">
+        <x:v>Access clinical records for TB/HIV workflow support | Expose laboratory-order and related clinical workflow actions</x:v>
+      </x:c>
+      <x:c r="I142" s="11" t="str">
+        <x:v>Includes treatment-oriented calculations and write actions. Inclusion covers clinical-data connectivity, not validation of dosing, treatment advice or local guideline compliance.</x:v>
+      </x:c>
+      <x:c r="J142" s="11" t="str">
+        <x:v>Static source and documentation reviewed</x:v>
+      </x:c>
+      <x:c r="K142" s="11" t="str">
+        <x:v>Canonical repository metadata reviewed at commit 6030b39469f02a38b23f2610760bd168ce244b34</x:v>
+      </x:c>
+      <x:c r="L142" s="11" t="str">
+        <x:v>https://github.com/its-kios09/daktaritb-mcp/blob/6030b39469f02a38b23f2610760bd168ce244b34/README.md | https://github.com/its-kios09/daktaritb-mcp/blob/6030b39469f02a38b23f2610760bd168ce244b34/pyproject.toml | https://github.com/its-kios09/daktaritb-mcp/blob/6030b39469f02a38b23f2610760bd168ce244b34/src/daktaritb_mcp/server.py</x:v>
+      </x:c>
+      <x:c r="M142" s="11" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N142" s="11" t="str">
+        <x:v>its-kios09</x:v>
+      </x:c>
+      <x:c r="O142" s="11" t="str">
+        <x:v>NOASSERTION</x:v>
+      </x:c>
+      <x:c r="P142" s="11" t="str">
+        <x:v>See pinned project manifest and setup documentation</x:v>
+      </x:c>
+      <x:c r="Q142" s="11" t="str">
+        <x:v>See pinned setup; varies by component</x:v>
+      </x:c>
+      <x:c r="R142" s="11" t="str">
+        <x:v>See capability and limitation fields; no runtime actions performed</x:v>
+      </x:c>
+      <x:c r="S142" s="11" t="str">
+        <x:v>See pinned project setup; external data access may require credentials.</x:v>
+      </x:c>
+      <x:c r="T142" s="14" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+      <x:c r="U142" s="14" t="n">
+        <x:v>46131.77717592593</x:v>
+      </x:c>
+      <x:c r="V142" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="W142" s="11" t="str">
+        <x:v>https://github.com/its-kios09/daktaritb-mcp</x:v>
+      </x:c>
+      <x:c r="X142" s="11" t="str">
+        <x:v>https://github.com/its-kios09/daktaritb-mcp</x:v>
+      </x:c>
+      <x:c r="Y142" s="11" t="str">
+        <x:v>https://github.com/its-kios09/daktaritb-mcp/blob/6030b39469f02a38b23f2610760bd168ce244b34/README.md | https://github.com/its-kios09/daktaritb-mcp/blob/6030b39469f02a38b23f2610760bd168ce244b34/pyproject.toml | https://github.com/its-kios09/daktaritb-mcp/blob/6030b39469f02a38b23f2610760bd168ce244b34/src/daktaritb_mcp/server.py</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="143" ht="105.5999984741211" hidden="0" customHeight="1">
+      <x:c r="A143" s="11" t="str">
+        <x:v>RWE-0250</x:v>
+      </x:c>
+      <x:c r="B143" s="11" t="str">
+        <x:v>Google Health MCP (davidmosiah)</x:v>
+      </x:c>
+      <x:c r="C143" s="11" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D143" s="11" t="str">
+        <x:v>Clinical Data &amp; Interoperability</x:v>
+      </x:c>
+      <x:c r="E143" s="11" t="str">
+        <x:v>Local connector to Google Health API data from supported Fitbit and Pixel Watch accounts.</x:v>
+      </x:c>
+      <x:c r="F143" s="11" t="str">
+        <x:v>Clinical Data | MCP server</x:v>
+      </x:c>
+      <x:c r="G143" s="11" t="str">
+        <x:v>Clinical Data &amp; Interoperability | Source inspection and research preparation</x:v>
+      </x:c>
+      <x:c r="H143" s="11" t="str">
+        <x:v>Retrieve supported account health and activity measurements | Serve tools through stdio or local HTTP</x:v>
+      </x:c>
+      <x:c r="I143" s="11" t="str">
+        <x:v>Beta upstream access and account/device support can vary. Verify measurement provenance and OAuth scopes before research use.</x:v>
+      </x:c>
+      <x:c r="J143" s="11" t="str">
+        <x:v>Static source and documentation reviewed</x:v>
+      </x:c>
+      <x:c r="K143" s="11" t="str">
+        <x:v>Canonical repository metadata reviewed at commit e0322e872b44cf21f898ffee4a550bc164ee8392</x:v>
+      </x:c>
+      <x:c r="L143" s="11" t="str">
+        <x:v>https://github.com/davidmosiah/google-health-mcp/blob/e0322e872b44cf21f898ffee4a550bc164ee8392/README.md | https://github.com/davidmosiah/google-health-mcp/blob/e0322e872b44cf21f898ffee4a550bc164ee8392/package.json | https://github.com/davidmosiah/google-health-mcp/blob/e0322e872b44cf21f898ffee4a550bc164ee8392/server.json | https://github.com/davidmosiah/google-health-mcp/blob/e0322e872b44cf21f898ffee4a550bc164ee8392/skill/SKILL.md</x:v>
+      </x:c>
+      <x:c r="M143" s="11" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N143" s="11" t="str">
+        <x:v>davidmosiah</x:v>
+      </x:c>
+      <x:c r="O143" s="11" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P143" s="11" t="str">
+        <x:v>See pinned project manifest and setup documentation</x:v>
+      </x:c>
+      <x:c r="Q143" s="11" t="str">
+        <x:v>See pinned setup; varies by component</x:v>
+      </x:c>
+      <x:c r="R143" s="11" t="str">
+        <x:v>See capability and limitation fields; no runtime actions performed</x:v>
+      </x:c>
+      <x:c r="S143" s="11" t="str">
+        <x:v>Google OAuth application and authorized Google Health account.</x:v>
+      </x:c>
+      <x:c r="T143" s="14" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+      <x:c r="U143" s="14" t="n">
+        <x:v>46263.4372337963</x:v>
+      </x:c>
+      <x:c r="V143" s="11" t="n">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="W143" s="11" t="str">
+        <x:v>https://github.com/davidmosiah/google-health-mcp</x:v>
+      </x:c>
+      <x:c r="X143" s="11" t="str">
+        <x:v>https://github.com/davidmosiah/google-health-mcp</x:v>
+      </x:c>
+      <x:c r="Y143" s="11" t="str">
+        <x:v>https://github.com/davidmosiah/google-health-mcp/blob/e0322e872b44cf21f898ffee4a550bc164ee8392/README.md | https://github.com/davidmosiah/google-health-mcp/blob/e0322e872b44cf21f898ffee4a550bc164ee8392/package.json | https://github.com/davidmosiah/google-health-mcp/blob/e0322e872b44cf21f898ffee4a550bc164ee8392/server.json | https://github.com/davidmosiah/google-health-mcp/blob/e0322e872b44cf21f898ffee4a550bc164ee8392/skill/SKILL.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="144" ht="118.80000305175781" hidden="0" customHeight="1">
+      <x:c r="A144" s="11" t="str">
+        <x:v>RWE-0200</x:v>
+      </x:c>
+      <x:c r="B144" s="11" t="str">
+        <x:v>MedAdapt Content Server</x:v>
+      </x:c>
+      <x:c r="C144" s="11" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D144" s="11" t="str">
+        <x:v>Literature &amp; Evidence Synthesis</x:v>
+      </x:c>
+      <x:c r="E144" s="11" t="str">
+        <x:v>Retrieves and caches medical literature and textbook content alongside user-provided documents.</x:v>
+      </x:c>
+      <x:c r="F144" s="11" t="str">
+        <x:v>Literature | MCP server</x:v>
+      </x:c>
+      <x:c r="G144" s="11" t="str">
+        <x:v>Literature &amp; Evidence Synthesis | Source inspection and research preparation</x:v>
+      </x:c>
+      <x:c r="H144" s="11" t="str">
+        <x:v>Search PubMed, NCBI Bookshelf and a local resource database | Retrieve cached source content and import local learning documents</x:v>
+      </x:c>
+      <x:c r="I144" s="11" t="str">
+        <x:v>Educational overviews and key-point extraction use simplified heuristics and generic fallbacks. Local-cache preference can limit fresh retrieval; not a systematic-review search engine.</x:v>
+      </x:c>
+      <x:c r="J144" s="11" t="str">
+        <x:v>Static source and documentation reviewed</x:v>
+      </x:c>
+      <x:c r="K144" s="11" t="str">
+        <x:v>Canonical repository metadata reviewed at commit 8ae3d033684db57b08f2578184b19aa4b2072426</x:v>
+      </x:c>
+      <x:c r="L144" s="11" t="str">
+        <x:v>https://github.com/ryoureddy/medadapt-content-server/blob/8ae3d033684db57b08f2578184b19aa4b2072426/README.md | https://github.com/ryoureddy/medadapt-content-server/blob/8ae3d033684db57b08f2578184b19aa4b2072426/content_server.py | https://github.com/ryoureddy/medadapt-content-server/blob/8ae3d033684db57b08f2578184b19aa4b2072426/pubmed_utils.py</x:v>
+      </x:c>
+      <x:c r="M144" s="11" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N144" s="11" t="str">
+        <x:v>ryoureddy</x:v>
+      </x:c>
+      <x:c r="O144" s="11" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P144" s="11" t="str">
+        <x:v>See pinned project manifest and setup documentation</x:v>
+      </x:c>
+      <x:c r="Q144" s="11" t="str">
+        <x:v>See pinned setup; varies by component</x:v>
+      </x:c>
+      <x:c r="R144" s="11" t="str">
+        <x:v>See capability and limitation fields; no runtime actions performed</x:v>
+      </x:c>
+      <x:c r="S144" s="11" t="str">
+        <x:v>See pinned project setup; external data access may require credentials.</x:v>
+      </x:c>
+      <x:c r="T144" s="14" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+      <x:c r="U144" s="14" t="n">
+        <x:v>45744.266875</x:v>
+      </x:c>
+      <x:c r="V144" s="11" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="W144" s="11" t="str">
+        <x:v>https://github.com/ryoureddy/medadapt-content-server</x:v>
+      </x:c>
+      <x:c r="X144" s="11" t="str">
+        <x:v>https://github.com/ryoureddy/medadapt-content-server</x:v>
+      </x:c>
+      <x:c r="Y144" s="11" t="str">
+        <x:v>https://github.com/ryoureddy/medadapt-content-server/blob/8ae3d033684db57b08f2578184b19aa4b2072426/README.md | https://github.com/ryoureddy/medadapt-content-server/blob/8ae3d033684db57b08f2578184b19aa4b2072426/content_server.py | https://github.com/ryoureddy/medadapt-content-server/blob/8ae3d033684db57b08f2578184b19aa4b2072426/pubmed_utils.py</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="145" ht="92.4000015258789" hidden="0" customHeight="1">
+      <x:c r="A145" s="11" t="str">
+        <x:v>RWE-0205</x:v>
+      </x:c>
+      <x:c r="B145" s="11" t="str">
+        <x:v>NCCN Guidelines MCP</x:v>
+      </x:c>
+      <x:c r="C145" s="11" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D145" s="11" t="str">
+        <x:v>Literature &amp; Evidence Synthesis</x:v>
+      </x:c>
+      <x:c r="E145" s="11" t="str">
+        <x:v>Searches a guideline index and retrieves NCCN PDF content for evidence-reference workflows.</x:v>
+      </x:c>
+      <x:c r="F145" s="11" t="str">
+        <x:v>Literature | MCP server</x:v>
+      </x:c>
+      <x:c r="G145" s="11" t="str">
+        <x:v>Literature &amp; Evidence Synthesis | Source inspection and research preparation</x:v>
+      </x:c>
+      <x:c r="H145" s="11" t="str">
+        <x:v>Search indexed guideline metadata | Download authorized guideline PDFs and extract page content</x:v>
+      </x:c>
+      <x:c r="I145" s="11" t="str">
+        <x:v>NCCN access and reuse restrictions apply. Cached content can lag updates; verify guideline version, page context and extraction accuracy.</x:v>
+      </x:c>
+      <x:c r="J145" s="11" t="str">
+        <x:v>Static source and documentation reviewed</x:v>
+      </x:c>
+      <x:c r="K145" s="11" t="str">
+        <x:v>Canonical repository metadata reviewed at commit dcc65a6392a67ba26eab697c1d87f446dc1cfc21</x:v>
+      </x:c>
+      <x:c r="L145" s="11" t="str">
+        <x:v>https://github.com/gscfwid/NCCN_guidelines_MCP/blob/dcc65a6392a67ba26eab697c1d87f446dc1cfc21/README.md | https://github.com/gscfwid/NCCN_guidelines_MCP/blob/dcc65a6392a67ba26eab697c1d87f446dc1cfc21/pyproject.toml | https://github.com/gscfwid/NCCN_guidelines_MCP/blob/dcc65a6392a67ba26eab697c1d87f446dc1cfc21/server.py</x:v>
+      </x:c>
+      <x:c r="M145" s="11" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N145" s="11" t="str">
+        <x:v>gscfwid</x:v>
+      </x:c>
+      <x:c r="O145" s="11" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P145" s="11" t="str">
+        <x:v>See pinned project manifest and setup documentation</x:v>
+      </x:c>
+      <x:c r="Q145" s="11" t="str">
+        <x:v>See pinned setup; varies by component</x:v>
+      </x:c>
+      <x:c r="R145" s="11" t="str">
+        <x:v>See capability and limitation fields; no runtime actions performed</x:v>
+      </x:c>
+      <x:c r="S145" s="11" t="str">
+        <x:v>NCCN login for restricted PDFs; local PDF cache.</x:v>
+      </x:c>
+      <x:c r="T145" s="14" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+      <x:c r="U145" s="14" t="n">
+        <x:v>45860.645474537036</x:v>
+      </x:c>
+      <x:c r="V145" s="11" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="W145" s="11" t="str">
+        <x:v>https://github.com/gscfwid/NCCN_guidelines_MCP</x:v>
+      </x:c>
+      <x:c r="X145" s="11" t="str">
+        <x:v>https://github.com/gscfwid/NCCN_guidelines_MCP</x:v>
+      </x:c>
+      <x:c r="Y145" s="11" t="str">
+        <x:v>https://github.com/gscfwid/NCCN_guidelines_MCP/blob/dcc65a6392a67ba26eab697c1d87f446dc1cfc21/README.md | https://github.com/gscfwid/NCCN_guidelines_MCP/blob/dcc65a6392a67ba26eab697c1d87f446dc1cfc21/pyproject.toml | https://github.com/gscfwid/NCCN_guidelines_MCP/blob/dcc65a6392a67ba26eab697c1d87f446dc1cfc21/server.py</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="146" ht="118.80000305175781" hidden="0" customHeight="1">
+      <x:c r="A146" s="11" t="str">
+        <x:v>RWE-0206</x:v>
+      </x:c>
+      <x:c r="B146" s="11" t="str">
+        <x:v>NexOnco MCP</x:v>
+      </x:c>
+      <x:c r="C146" s="11" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D146" s="11" t="str">
+        <x:v>Literature &amp; Evidence Synthesis</x:v>
+      </x:c>
+      <x:c r="E146" s="11" t="str">
+        <x:v>Retrieves structured cancer-variant evidence from CIViC.</x:v>
+      </x:c>
+      <x:c r="F146" s="11" t="str">
+        <x:v>Literature | MCP server</x:v>
+      </x:c>
+      <x:c r="G146" s="11" t="str">
+        <x:v>Literature &amp; Evidence Synthesis | Source inspection and research preparation</x:v>
+      </x:c>
+      <x:c r="H146" s="11" t="str">
+        <x:v>Filter evidence by disease, therapy, variant and evidence type | Inspect evidence direction and source-provided ratings</x:v>
+      </x:c>
+      <x:c r="I146" s="11" t="str">
+        <x:v>CIViC classifications and ratings are source annotations, not independent comparative-effectiveness estimates. Check record dates and underlying publications.</x:v>
+      </x:c>
+      <x:c r="J146" s="11" t="str">
+        <x:v>Static source and documentation reviewed</x:v>
+      </x:c>
+      <x:c r="K146" s="11" t="str">
+        <x:v>Canonical repository metadata reviewed at commit d0b45e147a5cd764d4ceea27f5607014cbde213b</x:v>
+      </x:c>
+      <x:c r="L146" s="11" t="str">
+        <x:v>https://github.com/Nexgene-Research/nexonco-mcp/blob/d0b45e147a5cd764d4ceea27f5607014cbde213b/README.md | https://github.com/Nexgene-Research/nexonco-mcp/blob/d0b45e147a5cd764d4ceea27f5607014cbde213b/pyproject.toml | https://github.com/Nexgene-Research/nexonco-mcp/blob/d0b45e147a5cd764d4ceea27f5607014cbde213b/src/nexonco/server.py</x:v>
+      </x:c>
+      <x:c r="M146" s="11" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N146" s="11" t="str">
+        <x:v>Nexgene-Research</x:v>
+      </x:c>
+      <x:c r="O146" s="11" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P146" s="11" t="str">
+        <x:v>See pinned project manifest and setup documentation</x:v>
+      </x:c>
+      <x:c r="Q146" s="11" t="str">
+        <x:v>See pinned setup; varies by component</x:v>
+      </x:c>
+      <x:c r="R146" s="11" t="str">
+        <x:v>See capability and limitation fields; no runtime actions performed</x:v>
+      </x:c>
+      <x:c r="S146" s="11" t="str">
+        <x:v>See pinned project setup; external data access may require credentials.</x:v>
+      </x:c>
+      <x:c r="T146" s="14" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+      <x:c r="U146" s="14" t="n">
+        <x:v>45881.46251157407</x:v>
+      </x:c>
+      <x:c r="V146" s="11" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="W146" s="11" t="str">
+        <x:v>https://github.com/Nexgene-Research/nexonco-mcp</x:v>
+      </x:c>
+      <x:c r="X146" s="11" t="str">
+        <x:v>https://github.com/Nexgene-Research/nexonco-mcp</x:v>
+      </x:c>
+      <x:c r="Y146" s="11" t="str">
+        <x:v>https://github.com/Nexgene-Research/nexonco-mcp/blob/d0b45e147a5cd764d4ceea27f5607014cbde213b/README.md | https://github.com/Nexgene-Research/nexonco-mcp/blob/d0b45e147a5cd764d4ceea27f5607014cbde213b/pyproject.toml | https://github.com/Nexgene-Research/nexonco-mcp/blob/d0b45e147a5cd764d4ceea27f5607014cbde213b/src/nexonco/server.py</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="147" ht="105.5999984741211" hidden="0" customHeight="1">
+      <x:c r="A147" s="11" t="str">
+        <x:v>RWE-0207</x:v>
+      </x:c>
+      <x:c r="B147" s="11" t="str">
+        <x:v>OncoFiles</x:v>
+      </x:c>
+      <x:c r="C147" s="11" t="str">
+        <x:v>Clinical agent application + MCP tools</x:v>
+      </x:c>
+      <x:c r="D147" s="11" t="str">
+        <x:v>Clinical Data &amp; Interoperability</x:v>
+      </x:c>
+      <x:c r="E147" s="11" t="str">
+        <x:v>Organizes patient-provided oncology documents and longitudinal records with research lookups.</x:v>
+      </x:c>
+      <x:c r="F147" s="11" t="str">
+        <x:v>Clinical Data | Clinical agent application + MCP tools</x:v>
+      </x:c>
+      <x:c r="G147" s="11" t="str">
+        <x:v>Clinical Data &amp; Interoperability | Source inspection and research preparation</x:v>
+      </x:c>
+      <x:c r="H147" s="11" t="str">
+        <x:v>Extract records and construct laboratory or treatment timelines | Connect document sources and retrieve PubMed or trial references</x:v>
+      </x:c>
+      <x:c r="I147" s="11" t="str">
+        <x:v>OCR and timeline extraction need source verification. Gmail, Drive and calendar integrations can read or write sensitive data; patient records are not a validated outcomes dataset.</x:v>
+      </x:c>
+      <x:c r="J147" s="11" t="str">
+        <x:v>Static source and documentation reviewed</x:v>
+      </x:c>
+      <x:c r="K147" s="11" t="str">
+        <x:v>Canonical repository metadata reviewed at commit 0abd270f46a16dbf1600c95d4a1663ba20b5ad04</x:v>
+      </x:c>
+      <x:c r="L147" s="11" t="str">
+        <x:v>https://github.com/peter-fusek/oncofiles/blob/0abd270f46a16dbf1600c95d4a1663ba20b5ad04/README.md | https://github.com/peter-fusek/oncofiles/blob/0abd270f46a16dbf1600c95d4a1663ba20b5ad04/pyproject.toml | https://github.com/peter-fusek/oncofiles/blob/0abd270f46a16dbf1600c95d4a1663ba20b5ad04/server.json | https://github.com/peter-fusek/oncofiles/blob/0abd270f46a16dbf1600c95d4a1663ba20b5ad04/src/oncofiles/server.py</x:v>
+      </x:c>
+      <x:c r="M147" s="11" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N147" s="11" t="str">
+        <x:v>peter-fusek</x:v>
+      </x:c>
+      <x:c r="O147" s="11" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P147" s="11" t="str">
+        <x:v>See pinned project manifest and setup documentation</x:v>
+      </x:c>
+      <x:c r="Q147" s="11" t="str">
+        <x:v>See pinned setup; varies by component</x:v>
+      </x:c>
+      <x:c r="R147" s="11" t="str">
+        <x:v>See capability and limitation fields; no runtime actions performed</x:v>
+      </x:c>
+      <x:c r="S147" s="11" t="str">
+        <x:v>See pinned project setup; external data access may require credentials.</x:v>
+      </x:c>
+      <x:c r="T147" s="14" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+      <x:c r="U147" s="14" t="n">
+        <x:v>46241.55070601852</x:v>
+      </x:c>
+      <x:c r="V147" s="11" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="W147" s="11" t="str">
+        <x:v>https://github.com/peter-fusek/oncofiles</x:v>
+      </x:c>
+      <x:c r="X147" s="11" t="str">
+        <x:v>https://github.com/peter-fusek/oncofiles</x:v>
+      </x:c>
+      <x:c r="Y147" s="11" t="str">
+        <x:v>https://github.com/peter-fusek/oncofiles/blob/0abd270f46a16dbf1600c95d4a1663ba20b5ad04/README.md | https://github.com/peter-fusek/oncofiles/blob/0abd270f46a16dbf1600c95d4a1663ba20b5ad04/pyproject.toml | https://github.com/peter-fusek/oncofiles/blob/0abd270f46a16dbf1600c95d4a1663ba20b5ad04/server.json | https://github.com/peter-fusek/oncofiles/blob/0abd270f46a16dbf1600c95d4a1663ba20b5ad04/src/oncofiles/server.py</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="148" ht="158.39999389648438" hidden="0" customHeight="1">
+      <x:c r="A148" s="11" t="str">
+        <x:v>RWE-0247</x:v>
+      </x:c>
+      <x:c r="B148" s="11" t="str">
+        <x:v>Apple Health Export MCP</x:v>
+      </x:c>
+      <x:c r="C148" s="11" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D148" s="11" t="str">
+        <x:v>Clinical Data &amp; Interoperability</x:v>
+      </x:c>
+      <x:c r="E148" s="11" t="str">
+        <x:v>Imports Apple Health ZIP exports into SQLite for local metric exploration.</x:v>
+      </x:c>
+      <x:c r="F148" s="11" t="str">
+        <x:v>Clinical Data | MCP server</x:v>
+      </x:c>
+      <x:c r="G148" s="11" t="str">
+        <x:v>Clinical Data &amp; Interoperability | Source inspection and research preparation</x:v>
+      </x:c>
+      <x:c r="H148" s="11" t="str">
+        <x:v>Inspect record types, sources and date coverage | Aggregate measurements, sleep records and workouts</x:v>
+      </x:c>
+      <x:c r="I148" s="11" t="str">
+        <x:v>Imported observations may overlap across devices. Validate deduplication, units, time zones and endpoint definitions; export ingestion writes a local database.</x:v>
+      </x:c>
+      <x:c r="J148" s="11" t="str">
+        <x:v>Static source and documentation reviewed</x:v>
+      </x:c>
+      <x:c r="K148" s="11" t="str">
+        <x:v>Canonical repository metadata reviewed at commit 02e9ce9fe48910fe57033c915d23d0512a64233c</x:v>
+      </x:c>
+      <x:c r="L148" s="11" t="str">
+        <x:v>https://github.com/burakdirin/apple-health-export-mcp/blob/02e9ce9fe48910fe57033c915d23d0512a64233c/README.md | https://github.com/burakdirin/apple-health-export-mcp/blob/02e9ce9fe48910fe57033c915d23d0512a64233c/pyproject.toml | https://github.com/burakdirin/apple-health-export-mcp/blob/02e9ce9fe48910fe57033c915d23d0512a64233c/src/apple_health_export_mcp/server.py | https://github.com/burakdirin/apple-health-export-mcp/blob/02e9ce9fe48910fe57033c915d23d0512a64233c/src/apple_health_export_mcp/tools.py</x:v>
+      </x:c>
+      <x:c r="M148" s="11" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N148" s="11" t="str">
+        <x:v>burakdirin</x:v>
+      </x:c>
+      <x:c r="O148" s="11" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P148" s="11" t="str">
+        <x:v>See pinned project manifest and setup documentation</x:v>
+      </x:c>
+      <x:c r="Q148" s="11" t="str">
+        <x:v>See pinned setup; varies by component</x:v>
+      </x:c>
+      <x:c r="R148" s="11" t="str">
+        <x:v>See capability and limitation fields; no runtime actions performed</x:v>
+      </x:c>
+      <x:c r="S148" s="11" t="str">
+        <x:v>See pinned project setup; external data access may require credentials.</x:v>
+      </x:c>
+      <x:c r="T148" s="14" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+      <x:c r="U148" s="14" t="n">
+        <x:v>46203.84407407408</x:v>
+      </x:c>
+      <x:c r="V148" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W148" s="11" t="str">
+        <x:v>https://github.com/burakdirin/apple-health-export-mcp</x:v>
+      </x:c>
+      <x:c r="X148" s="11" t="str">
+        <x:v>https://github.com/burakdirin/apple-health-export-mcp</x:v>
+      </x:c>
+      <x:c r="Y148" s="11" t="str">
+        <x:v>https://github.com/burakdirin/apple-health-export-mcp/blob/02e9ce9fe48910fe57033c915d23d0512a64233c/README.md | https://github.com/burakdirin/apple-health-export-mcp/blob/02e9ce9fe48910fe57033c915d23d0512a64233c/pyproject.toml | https://github.com/burakdirin/apple-health-export-mcp/blob/02e9ce9fe48910fe57033c915d23d0512a64233c/src/apple_health_export_mcp/server.py | https://github.com/burakdirin/apple-health-export-mcp/blob/02e9ce9fe48910fe57033c915d23d0512a64233c/src/apple_health_export_mcp/tools.py</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="149" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A149" s="11" t="str">
+        <x:v>RWE-0190</x:v>
+      </x:c>
+      <x:c r="B149" s="11" t="str">
+        <x:v>CareTrace MCP</x:v>
+      </x:c>
+      <x:c r="C149" s="11" t="str">
+        <x:v>Experimental MCP server</x:v>
+      </x:c>
+      <x:c r="D149" s="11" t="str">
+        <x:v>Clinical Data &amp; Interoperability</x:v>
+      </x:c>
+      <x:c r="E149" s="11" t="str">
+        <x:v>Experimental clinical-text pipeline for entity extraction, FHIR bundle generation and timeline reconstruction.</x:v>
+      </x:c>
+      <x:c r="F149" s="11" t="str">
+        <x:v>Clinical Data | Experimental MCP server</x:v>
+      </x:c>
+      <x:c r="G149" s="11" t="str">
+        <x:v>Clinical Data &amp; Interoperability | Source inspection and research preparation</x:v>
+      </x:c>
+      <x:c r="H149" s="11" t="str">
+        <x:v>Extract medical entities from text | Build a FHIR bundle and reconstruct a clinical timeline</x:v>
+      </x:c>
+      <x:c r="I149" s="11" t="str">
+        <x:v>Generated concepts, dates and resources require manual validation against originals. Local Ollama and remote model configurations have different data-governance implications.</x:v>
+      </x:c>
+      <x:c r="J149" s="11" t="str">
+        <x:v>Static source and documentation reviewed</x:v>
+      </x:c>
+      <x:c r="K149" s="11" t="str">
+        <x:v>Canonical repository metadata reviewed at commit ec363224d72f7db67b47d1465f2f21b13e3bf889</x:v>
+      </x:c>
+      <x:c r="L149" s="11" t="str">
+        <x:v>https://github.com/jefftrojan/caretrace-mcp/blob/ec363224d72f7db67b47d1465f2f21b13e3bf889/README.md | https://github.com/jefftrojan/caretrace-mcp/blob/ec363224d72f7db67b47d1465f2f21b13e3bf889/mcp_server/server.py</x:v>
+      </x:c>
+      <x:c r="M149" s="11" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N149" s="11" t="str">
+        <x:v>jefftrojan</x:v>
+      </x:c>
+      <x:c r="O149" s="11" t="str">
+        <x:v>Not specified</x:v>
+      </x:c>
+      <x:c r="P149" s="11" t="str">
+        <x:v>See pinned project manifest and setup documentation</x:v>
+      </x:c>
+      <x:c r="Q149" s="11" t="str">
+        <x:v>See pinned setup; varies by component</x:v>
+      </x:c>
+      <x:c r="R149" s="11" t="str">
+        <x:v>See capability and limitation fields; no runtime actions performed</x:v>
+      </x:c>
+      <x:c r="S149" s="11" t="str">
+        <x:v>See pinned project setup; external data access may require credentials.</x:v>
+      </x:c>
+      <x:c r="T149" s="14" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+      <x:c r="U149" s="14" t="n">
+        <x:v>46155.03962962963</x:v>
+      </x:c>
+      <x:c r="V149" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W149" s="11" t="str">
+        <x:v>https://github.com/jefftrojan/caretrace-mcp</x:v>
+      </x:c>
+      <x:c r="X149" s="11" t="str">
+        <x:v>https://github.com/jefftrojan/caretrace-mcp</x:v>
+      </x:c>
+      <x:c r="Y149" s="11" t="str">
+        <x:v>https://github.com/jefftrojan/caretrace-mcp/blob/ec363224d72f7db67b47d1465f2f21b13e3bf889/README.md | https://github.com/jefftrojan/caretrace-mcp/blob/ec363224d72f7db67b47d1465f2f21b13e3bf889/mcp_server/server.py</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="150" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A150" s="11" t="str">
+        <x:v>RWE-0251</x:v>
+      </x:c>
+      <x:c r="B150" s="11" t="str">
+        <x:v>Google Health MCP (akshaygoyal)</x:v>
+      </x:c>
+      <x:c r="C150" s="11" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D150" s="11" t="str">
+        <x:v>Clinical Data &amp; Interoperability</x:v>
+      </x:c>
+      <x:c r="E150" s="11" t="str">
+        <x:v>Self-hosted remote MCP connector for Google Health account measurements.</x:v>
+      </x:c>
+      <x:c r="F150" s="11" t="str">
+        <x:v>Clinical Data | MCP server</x:v>
+      </x:c>
+      <x:c r="G150" s="11" t="str">
+        <x:v>Clinical Data &amp; Interoperability | Source inspection and research preparation</x:v>
+      </x:c>
+      <x:c r="H150" s="11" t="str">
+        <x:v>Expose supported Google Health measurement tools | Use an OAuth-backed hosted connector for agent access</x:v>
+      </x:c>
+      <x:c r="I150" s="11" t="str">
+        <x:v>Account and device coverage constrain completeness. Hosting, token storage and health-data access require appropriate controls; distinct deployment from the local Google Health connector.</x:v>
+      </x:c>
+      <x:c r="J150" s="11" t="str">
+        <x:v>Static source and documentation reviewed</x:v>
+      </x:c>
+      <x:c r="K150" s="11" t="str">
+        <x:v>Canonical repository metadata reviewed at commit e2f4564c2ce050f077f4759aa66416dd2c6d3cad</x:v>
+      </x:c>
+      <x:c r="L150" s="11" t="str">
+        <x:v>https://github.com/akshaygoyal/google-health-mcp/blob/e2f4564c2ce050f077f4759aa66416dd2c6d3cad/README.md | https://github.com/akshaygoyal/google-health-mcp/blob/e2f4564c2ce050f077f4759aa66416dd2c6d3cad/package.json | https://github.com/akshaygoyal/google-health-mcp/blob/e2f4564c2ce050f077f4759aa66416dd2c6d3cad/src/tools.ts</x:v>
+      </x:c>
+      <x:c r="M150" s="11" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N150" s="11" t="str">
+        <x:v>akshaygoyal</x:v>
+      </x:c>
+      <x:c r="O150" s="11" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P150" s="11" t="str">
+        <x:v>See pinned project manifest and setup documentation</x:v>
+      </x:c>
+      <x:c r="Q150" s="11" t="str">
+        <x:v>See pinned setup; varies by component</x:v>
+      </x:c>
+      <x:c r="R150" s="11" t="str">
+        <x:v>See capability and limitation fields; no runtime actions performed</x:v>
+      </x:c>
+      <x:c r="S150" s="11" t="str">
+        <x:v>Google OAuth; self-hosted Cloudflare configuration.</x:v>
+      </x:c>
+      <x:c r="T150" s="14" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+      <x:c r="U150" s="14" t="n">
+        <x:v>46203.902349537035</x:v>
+      </x:c>
+      <x:c r="V150" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="W150" s="11" t="str">
+        <x:v>https://github.com/akshaygoyal/google-health-mcp</x:v>
+      </x:c>
+      <x:c r="X150" s="11" t="str">
+        <x:v>https://github.com/akshaygoyal/google-health-mcp</x:v>
+      </x:c>
+      <x:c r="Y150" s="11" t="str">
+        <x:v>https://github.com/akshaygoyal/google-health-mcp/blob/e2f4564c2ce050f077f4759aa66416dd2c6d3cad/README.md | https://github.com/akshaygoyal/google-health-mcp/blob/e2f4564c2ce050f077f4759aa66416dd2c6d3cad/package.json | https://github.com/akshaygoyal/google-health-mcp/blob/e2f4564c2ce050f077f4759aa66416dd2c6d3cad/src/tools.ts</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="151" ht="171.60000610351562" hidden="0" customHeight="1">
+      <x:c r="A151" s="11" t="str">
+        <x:v>RWE-0204</x:v>
+      </x:c>
+      <x:c r="B151" s="11" t="str">
+        <x:v>MedVision MCP</x:v>
+      </x:c>
+      <x:c r="C151" s="11" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D151" s="11" t="str">
+        <x:v>Biomedical &amp; RWE Infrastructure</x:v>
+      </x:c>
+      <x:c r="E151" s="11" t="str">
+        <x:v>Research imaging tools for pathology classification, radiology embeddings and image retrieval.</x:v>
+      </x:c>
+      <x:c r="F151" s="11" t="str">
+        <x:v>Biomedical | MCP server</x:v>
+      </x:c>
+      <x:c r="G151" s="11" t="str">
+        <x:v>Biomedical &amp; RWE Infrastructure | Source inspection and research preparation</x:v>
+      </x:c>
+      <x:c r="H151" s="11" t="str">
+        <x:v>Generate model-based imaging features and classifications | Index image embeddings and inspect DICOM or region-of-interest data</x:v>
+      </x:c>
+      <x:c r="I151" s="11" t="str">
+        <x:v>Models and similarity results are not independently validated for diagnosis. Planned segmentation is not counted as an implemented capability; assess dataset shift and image privacy.</x:v>
+      </x:c>
+      <x:c r="J151" s="11" t="str">
+        <x:v>Static source and documentation reviewed</x:v>
+      </x:c>
+      <x:c r="K151" s="11" t="str">
+        <x:v>Canonical repository metadata reviewed at commit 0dfd8b5c6e0f9baba8cf2b1bb4a1615eee7bd040</x:v>
+      </x:c>
+      <x:c r="L151" s="11" t="str">
+        <x:v>https://github.com/u9401066/medvision-mcp/blob/0dfd8b5c6e0f9baba8cf2b1bb4a1615eee7bd040/README.md | https://github.com/u9401066/medvision-mcp/blob/0dfd8b5c6e0f9baba8cf2b1bb4a1615eee7bd040/pyproject.toml | https://github.com/u9401066/medvision-mcp/blob/0dfd8b5c6e0f9baba8cf2b1bb4a1615eee7bd040/.claude/skills/bug-fix/SKILL.md | https://github.com/u9401066/medvision-mcp/blob/0dfd8b5c6e0f9baba8cf2b1bb4a1615eee7bd040/.claude/skills/changelog-updater/SKILL.md | https://github.com/u9401066/medvision-mcp/blob/0dfd8b5c6e0f9baba8cf2b1bb4a1615eee7bd040/.claude/skills/code-refactor/SKILL.md</x:v>
+      </x:c>
+      <x:c r="M151" s="11" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N151" s="11" t="str">
+        <x:v>u9401066</x:v>
+      </x:c>
+      <x:c r="O151" s="11" t="str">
+        <x:v>Not specified</x:v>
+      </x:c>
+      <x:c r="P151" s="11" t="str">
+        <x:v>See pinned project manifest and setup documentation</x:v>
+      </x:c>
+      <x:c r="Q151" s="11" t="str">
+        <x:v>See pinned setup; varies by component</x:v>
+      </x:c>
+      <x:c r="R151" s="11" t="str">
+        <x:v>See capability and limitation fields; no runtime actions performed</x:v>
+      </x:c>
+      <x:c r="S151" s="11" t="str">
+        <x:v>See pinned project setup; external data access may require credentials.</x:v>
+      </x:c>
+      <x:c r="T151" s="14" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+      <x:c r="U151" s="14" t="n">
+        <x:v>46055.376238425924</x:v>
+      </x:c>
+      <x:c r="V151" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W151" s="11" t="str">
+        <x:v>https://github.com/u9401066/medvision-mcp</x:v>
+      </x:c>
+      <x:c r="X151" s="11" t="str">
+        <x:v>https://github.com/u9401066/medvision-mcp</x:v>
+      </x:c>
+      <x:c r="Y151" s="11" t="str">
+        <x:v>https://github.com/u9401066/medvision-mcp/blob/0dfd8b5c6e0f9baba8cf2b1bb4a1615eee7bd040/README.md | https://github.com/u9401066/medvision-mcp/blob/0dfd8b5c6e0f9baba8cf2b1bb4a1615eee7bd040/pyproject.toml | https://github.com/u9401066/medvision-mcp/blob/0dfd8b5c6e0f9baba8cf2b1bb4a1615eee7bd040/.claude/skills/bug-fix/SKILL.md | https://github.com/u9401066/medvision-mcp/blob/0dfd8b5c6e0f9baba8cf2b1bb4a1615eee7bd040/.claude/skills/changelog-updater/SKILL.md | https://github.com/u9401066/medvision-mcp/blob/0dfd8b5c6e0f9baba8cf2b1bb4a1615eee7bd040/.claude/skills/code-refactor/SKILL.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="152" ht="92.4000015258789" hidden="0" customHeight="1">
+      <x:c r="A152" s="11" t="str">
+        <x:v>RWE-0224</x:v>
+      </x:c>
+      <x:c r="B152" s="11" t="str">
+        <x:v>Open Dental MCP</x:v>
+      </x:c>
+      <x:c r="C152" s="11" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D152" s="11" t="str">
+        <x:v>Clinical Data &amp; Interoperability</x:v>
+      </x:c>
+      <x:c r="E152" s="11" t="str">
+        <x:v>Connects agents to Open Dental patient and procedure records.</x:v>
+      </x:c>
+      <x:c r="F152" s="11" t="str">
+        <x:v>Clinical Data | MCP server</x:v>
+      </x:c>
+      <x:c r="G152" s="11" t="str">
+        <x:v>Clinical Data &amp; Interoperability | Source inspection and research preparation</x:v>
+      </x:c>
+      <x:c r="H152" s="11" t="str">
+        <x:v>Retrieve patient and procedure-log information | Expose appointment and record-management operations</x:v>
+      </x:c>
+      <x:c r="I152" s="11" t="str">
+        <x:v>Contains write actions and identifiable dental records. Research reuse requires authorized extraction and validation of procedure coding and longitudinal completeness.</x:v>
+      </x:c>
+      <x:c r="J152" s="11" t="str">
+        <x:v>Static source and documentation reviewed</x:v>
+      </x:c>
+      <x:c r="K152" s="11" t="str">
+        <x:v>Canonical repository metadata reviewed at commit fb12b4c0dc03dcc4a81334f0adcc6c9612172f7c</x:v>
+      </x:c>
+      <x:c r="L152" s="11" t="str">
+        <x:v>https://github.com/sanjibani/open-dental-mcp/blob/fb12b4c0dc03dcc4a81334f0adcc6c9612172f7c/README.md | https://github.com/sanjibani/open-dental-mcp/blob/fb12b4c0dc03dcc4a81334f0adcc6c9612172f7c/pyproject.toml | https://github.com/sanjibani/open-dental-mcp/blob/fb12b4c0dc03dcc4a81334f0adcc6c9612172f7c/src/open_dental_mcp/server.py</x:v>
+      </x:c>
+      <x:c r="M152" s="11" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N152" s="11" t="str">
+        <x:v>sanjibani</x:v>
+      </x:c>
+      <x:c r="O152" s="11" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P152" s="11" t="str">
+        <x:v>See pinned project manifest and setup documentation</x:v>
+      </x:c>
+      <x:c r="Q152" s="11" t="str">
+        <x:v>See pinned setup; varies by component</x:v>
+      </x:c>
+      <x:c r="R152" s="11" t="str">
+        <x:v>See capability and limitation fields; no runtime actions performed</x:v>
+      </x:c>
+      <x:c r="S152" s="11" t="str">
+        <x:v>Open Dental developer/customer API credentials.</x:v>
+      </x:c>
+      <x:c r="T152" s="14" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+      <x:c r="U152" s="14" t="n">
+        <x:v>46199.473449074074</x:v>
+      </x:c>
+      <x:c r="V152" s="11" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="W152" s="11" t="str">
+        <x:v>https://github.com/sanjibani/open-dental-mcp</x:v>
+      </x:c>
+      <x:c r="X152" s="11" t="str">
+        <x:v>https://github.com/sanjibani/open-dental-mcp</x:v>
+      </x:c>
+      <x:c r="Y152" s="11" t="str">
+        <x:v>https://github.com/sanjibani/open-dental-mcp/blob/fb12b4c0dc03dcc4a81334f0adcc6c9612172f7c/README.md | https://github.com/sanjibani/open-dental-mcp/blob/fb12b4c0dc03dcc4a81334f0adcc6c9612172f7c/pyproject.toml | https://github.com/sanjibani/open-dental-mcp/blob/fb12b4c0dc03dcc4a81334f0adcc6c9612172f7c/src/open_dental_mcp/server.py</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="153" ht="66" hidden="0" customHeight="1">
+      <x:c r="A153" s="11" t="str">
+        <x:v>RWE-0254</x:v>
+      </x:c>
+      <x:c r="B153" s="11" t="str">
+        <x:v>Oura MCP Server (Schimmilab)</x:v>
+      </x:c>
+      <x:c r="C153" s="11" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D153" s="11" t="str">
+        <x:v>Clinical Data &amp; Interoperability</x:v>
+      </x:c>
+      <x:c r="E153" s="11" t="str">
+        <x:v>Retrieves Oura sleep, activity and related wearable measurements for personal longitudinal analysis.</x:v>
+      </x:c>
+      <x:c r="F153" s="11" t="str">
+        <x:v>Clinical Data | MCP server</x:v>
+      </x:c>
+      <x:c r="G153" s="11" t="str">
+        <x:v>Clinical Data &amp; Interoperability | Source inspection and research preparation</x:v>
+      </x:c>
+      <x:c r="H153" s="11" t="str">
+        <x:v>Retrieve sleep, HRV, tags and workout records | Explore correlations and deviations across measurements</x:v>
+      </x:c>
+      <x:c r="I153" s="11" t="str">
+        <x:v>Readiness advice, anomalies and correlations are exploratory outputs. They do not establish clinical validity or causality; device algorithms and account coverage affect interpretation.</x:v>
+      </x:c>
+      <x:c r="J153" s="11" t="str">
+        <x:v>Static source and documentation reviewed</x:v>
+      </x:c>
+      <x:c r="K153" s="11" t="str">
+        <x:v>Canonical repository metadata reviewed at commit 3343258a40e6a0734a867ce1d89201eae82a005a</x:v>
+      </x:c>
+      <x:c r="L153" s="11" t="str">
+        <x:v>https://github.com/Schimmilab/oura-mcp-server/blob/3343258a40e6a0734a867ce1d89201eae82a005a/README.md | https://github.com/Schimmilab/oura-mcp-server/blob/3343258a40e6a0734a867ce1d89201eae82a005a/src/oura_mcp/core/server.py</x:v>
+      </x:c>
+      <x:c r="M153" s="11" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N153" s="11" t="str">
+        <x:v>Schimmilab</x:v>
+      </x:c>
+      <x:c r="O153" s="11" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P153" s="11" t="str">
+        <x:v>See pinned project manifest and setup documentation</x:v>
+      </x:c>
+      <x:c r="Q153" s="11" t="str">
+        <x:v>See pinned setup; varies by component</x:v>
+      </x:c>
+      <x:c r="R153" s="11" t="str">
+        <x:v>See capability and limitation fields; no runtime actions performed</x:v>
+      </x:c>
+      <x:c r="S153" s="11" t="str">
+        <x:v>Authorized Oura account credentials or OAuth configuration.</x:v>
+      </x:c>
+      <x:c r="T153" s="14" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+      <x:c r="U153" s="14" t="n">
+        <x:v>46263.78020833333</x:v>
+      </x:c>
+      <x:c r="V153" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W153" s="11" t="str">
+        <x:v>https://github.com/Schimmilab/oura-mcp-server</x:v>
+      </x:c>
+      <x:c r="X153" s="11" t="str">
+        <x:v>https://github.com/Schimmilab/oura-mcp-server</x:v>
+      </x:c>
+      <x:c r="Y153" s="11" t="str">
+        <x:v>https://github.com/Schimmilab/oura-mcp-server/blob/3343258a40e6a0734a867ce1d89201eae82a005a/README.md | https://github.com/Schimmilab/oura-mcp-server/blob/3343258a40e6a0734a867ce1d89201eae82a005a/src/oura_mcp/core/server.py</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="154" ht="105.5999984741211" hidden="0" customHeight="1">
+      <x:c r="A154" s="11" t="str">
+        <x:v>RWE-0124</x:v>
+      </x:c>
+      <x:c r="B154" s="11" t="str">
+        <x:v>AIGroup Econ MCP</x:v>
+      </x:c>
+      <x:c r="C154" s="11" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D154" s="11" t="str">
+        <x:v>Causal Inference &amp; Analytics</x:v>
+      </x:c>
+      <x:c r="E154" s="11" t="str">
+        <x:v>Exposes statistical and econometric analysis tools relevant to observational research.</x:v>
+      </x:c>
+      <x:c r="F154" s="11" t="str">
+        <x:v>Causal Inference | MCP server</x:v>
+      </x:c>
+      <x:c r="G154" s="11" t="str">
+        <x:v>Causal Inference &amp; Analytics | Source inspection and research preparation</x:v>
+      </x:c>
+      <x:c r="H154" s="11" t="str">
+        <x:v>Run supported regression, missing-data and descriptive analyses | Explore DID, IV, matching, regression discontinuity and synthetic-control methods</x:v>
+      </x:c>
+      <x:c r="I154" s="11" t="str">
+        <x:v>Method availability is source-reviewed only. Check estimands, identification assumptions, diagnostics, uncertainty and implementation-specific behavior before relying on estimates.</x:v>
+      </x:c>
+      <x:c r="J154" s="11" t="str">
+        <x:v>Static source and documentation reviewed</x:v>
+      </x:c>
+      <x:c r="K154" s="11" t="str">
+        <x:v>Canonical repository metadata reviewed at commit 467ab6443f374bb55c47f9326c4847b91b234c38</x:v>
+      </x:c>
+      <x:c r="L154" s="11" t="str">
+        <x:v>https://github.com/jackdark425/aigroup-econ-mcp/blob/467ab6443f374bb55c47f9326c4847b91b234c38/README.md | https://github.com/jackdark425/aigroup-econ-mcp/blob/467ab6443f374bb55c47f9326c4847b91b234c38/pyproject.toml | https://github.com/jackdark425/aigroup-econ-mcp/blob/467ab6443f374bb55c47f9326c4847b91b234c38/aigroup_econ_mcp/server.py</x:v>
+      </x:c>
+      <x:c r="M154" s="11" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N154" s="11" t="str">
+        <x:v>jackdark425</x:v>
+      </x:c>
+      <x:c r="O154" s="11" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P154" s="11" t="str">
+        <x:v>See pinned project manifest and setup documentation</x:v>
+      </x:c>
+      <x:c r="Q154" s="11" t="str">
+        <x:v>See pinned setup; varies by component</x:v>
+      </x:c>
+      <x:c r="R154" s="11" t="str">
+        <x:v>See capability and limitation fields; no runtime actions performed</x:v>
+      </x:c>
+      <x:c r="S154" s="11" t="str">
+        <x:v>See pinned project setup; external data access may require credentials.</x:v>
+      </x:c>
+      <x:c r="T154" s="14" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+      <x:c r="U154" s="14" t="n">
+        <x:v>46129.65809027778</x:v>
+      </x:c>
+      <x:c r="V154" s="11" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="W154" s="11" t="str">
+        <x:v>https://github.com/jackdark425/aigroup-econ-mcp</x:v>
+      </x:c>
+      <x:c r="X154" s="11" t="str">
+        <x:v>https://github.com/jackdark425/aigroup-econ-mcp</x:v>
+      </x:c>
+      <x:c r="Y154" s="11" t="str">
+        <x:v>https://github.com/jackdark425/aigroup-econ-mcp/blob/467ab6443f374bb55c47f9326c4847b91b234c38/README.md | https://github.com/jackdark425/aigroup-econ-mcp/blob/467ab6443f374bb55c47f9326c4847b91b234c38/pyproject.toml | https://github.com/jackdark425/aigroup-econ-mcp/blob/467ab6443f374bb55c47f9326c4847b91b234c38/aigroup_econ_mcp/server.py</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="155" ht="277.20001220703125" hidden="0" customHeight="1">
+      <x:c r="A155" s="11" t="str">
+        <x:v>RWE-0160</x:v>
+      </x:c>
+      <x:c r="B155" s="11" t="str">
+        <x:v>AlterLab Academic Skills</x:v>
+      </x:c>
+      <x:c r="C155" s="11" t="str">
+        <x:v>Agent skill collection</x:v>
+      </x:c>
+      <x:c r="D155" s="11" t="str">
+        <x:v>Biomedical &amp; RWE Infrastructure</x:v>
+      </x:c>
+      <x:c r="E155" s="11" t="str">
+        <x:v>Academic skill collection with statistical-analysis, survival and clinical-research components.</x:v>
+      </x:c>
+      <x:c r="F155" s="11" t="str">
+        <x:v>Biomedical | Agent skill collection</x:v>
+      </x:c>
+      <x:c r="G155" s="11" t="str">
+        <x:v>Biomedical &amp; RWE Infrastructure | Source inspection and research preparation</x:v>
+      </x:c>
+      <x:c r="H155" s="11" t="str">
+        <x:v>Provide statistical and survival-analysis workflow guidance | Supply clinical-research and database-specific agent skills</x:v>
+      </x:c>
+      <x:c r="I155" s="11" t="str">
+        <x:v>A collection of instructions and dependencies, not a standalone MCP server. Individual skills require review and adaptation; installation does not validate generated methods.</x:v>
+      </x:c>
+      <x:c r="J155" s="11" t="str">
+        <x:v>Static source and documentation reviewed</x:v>
+      </x:c>
+      <x:c r="K155" s="11" t="str">
+        <x:v>Canonical repository metadata reviewed at commit 4a5b75358026b33d3e53101bf551331e12113bee</x:v>
+      </x:c>
+      <x:c r="L155" s="11" t="str">
+        <x:v>https://github.com/AlterLab-IEU/AlterLab-Academic-Skills/blob/4a5b75358026b33d3e53101bf551331e12113bee/README.md | https://github.com/AlterLab-IEU/AlterLab-Academic-Skills/blob/4a5b75358026b33d3e53101bf551331e12113bee/package.json | https://github.com/AlterLab-IEU/AlterLab-Academic-Skills/blob/4a5b75358026b33d3e53101bf551331e12113bee/pyproject.toml | https://github.com/AlterLab-IEU/AlterLab-Academic-Skills/blob/4a5b75358026b33d3e53101bf551331e12113bee/mcp-servers/chemistry/server.py | https://github.com/AlterLab-IEU/AlterLab-Academic-Skills/blob/4a5b75358026b33d3e53101bf551331e12113bee/mcp-servers/genes-ontologies/server.py | https://github.com/AlterLab-IEU/AlterLab-Academic-Skills/blob/4a5b75358026b33d3e53101bf551331e12113bee/mcp-servers/structures/server.py | https://github.com/AlterLab-IEU/AlterLab-Academic-Skills/blob/4a5b75358026b33d3e53101bf551331e12113bee/skills/data-science/alterlab-statistical-analysis/SKILL.md</x:v>
+      </x:c>
+      <x:c r="M155" s="11" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N155" s="11" t="str">
+        <x:v>AlterLab-IEU</x:v>
+      </x:c>
+      <x:c r="O155" s="11" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P155" s="11" t="str">
+        <x:v>See pinned project manifest and setup documentation</x:v>
+      </x:c>
+      <x:c r="Q155" s="11" t="str">
+        <x:v>See pinned setup; varies by component</x:v>
+      </x:c>
+      <x:c r="R155" s="11" t="str">
+        <x:v>See capability and limitation fields; no runtime actions performed</x:v>
+      </x:c>
+      <x:c r="S155" s="11" t="str">
+        <x:v>See pinned project setup; external data access may require credentials.</x:v>
+      </x:c>
+      <x:c r="T155" s="14" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+      <x:c r="U155" s="14" t="n">
+        <x:v>46269.575532407405</x:v>
+      </x:c>
+      <x:c r="V155" s="11" t="n">
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="W155" s="11" t="str">
+        <x:v>https://github.com/AlterLab-IEU/AlterLab-Academic-Skills</x:v>
+      </x:c>
+      <x:c r="X155" s="11" t="str">
+        <x:v>https://github.com/AlterLab-IEU/AlterLab-Academic-Skills</x:v>
+      </x:c>
+      <x:c r="Y155" s="11" t="str">
+        <x:v>https://github.com/AlterLab-IEU/AlterLab-Academic-Skills/blob/4a5b75358026b33d3e53101bf551331e12113bee/README.md | https://github.com/AlterLab-IEU/AlterLab-Academic-Skills/blob/4a5b75358026b33d3e53101bf551331e12113bee/package.json | https://github.com/AlterLab-IEU/AlterLab-Academic-Skills/blob/4a5b75358026b33d3e53101bf551331e12113bee/pyproject.toml | https://github.com/AlterLab-IEU/AlterLab-Academic-Skills/blob/4a5b75358026b33d3e53101bf551331e12113bee/mcp-servers/chemistry/server.py | https://github.com/AlterLab-IEU/AlterLab-Academic-Skills/blob/4a5b75358026b33d3e53101bf551331e12113bee/mcp-servers/genes-ontologies/server.py | https://github.com/AlterLab-IEU/AlterLab-Academic-Skills/blob/4a5b75358026b33d3e53101bf551331e12113bee/mcp-servers/structures/server.py | https://github.com/AlterLab-IEU/AlterLab-Academic-Skills/blob/4a5b75358026b33d3e53101bf551331e12113bee/skills/data-science/alterlab-statistical-analysis/SKILL.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="156" ht="184.8000030517578" hidden="0" customHeight="1">
+      <x:c r="A156" s="11" t="str">
+        <x:v>RWE-0164</x:v>
+      </x:c>
+      <x:c r="B156" s="11" t="str">
+        <x:v>Clinical Skills (aizech)</x:v>
+      </x:c>
+      <x:c r="C156" s="11" t="str">
+        <x:v>Agent skill collection</x:v>
+      </x:c>
+      <x:c r="D156" s="11" t="str">
+        <x:v>Biomedical &amp; RWE Infrastructure</x:v>
+      </x:c>
+      <x:c r="E156" s="11" t="str">
+        <x:v>Agent skills for imaging research, clinical documentation and related data preparation.</x:v>
+      </x:c>
+      <x:c r="F156" s="11" t="str">
+        <x:v>Biomedical | Agent skill collection</x:v>
+      </x:c>
+      <x:c r="G156" s="11" t="str">
+        <x:v>Biomedical &amp; RWE Infrastructure | Source inspection and research preparation</x:v>
+      </x:c>
+      <x:c r="H156" s="11" t="str">
+        <x:v>Guide imaging-study review and radiology-report analysis | Support structured reporting and imaging-data workflows</x:v>
+      </x:c>
+      <x:c r="I156" s="11" t="str">
+        <x:v>Instructions do not establish diagnostic performance or reporting correctness. Verify DICOM handling, source citations and generated outputs in the intended research setting.</x:v>
+      </x:c>
+      <x:c r="J156" s="11" t="str">
+        <x:v>Static source and documentation reviewed</x:v>
+      </x:c>
+      <x:c r="K156" s="11" t="str">
+        <x:v>Canonical repository metadata reviewed at commit 743831b202a38977ed594eb5b1f21032800c41b2</x:v>
+      </x:c>
+      <x:c r="L156" s="11" t="str">
+        <x:v>https://github.com/aizech/clinical-skills/blob/743831b202a38977ed594eb5b1f21032800c41b2/README.md | https://github.com/aizech/clinical-skills/blob/743831b202a38977ed594eb5b1f21032800c41b2/.agents/skills/ai-detection-pipeline/SKILL.md | https://github.com/aizech/clinical-skills/blob/743831b202a38977ed594eb5b1f21032800c41b2/.agents/skills/ai-quality-review/SKILL.md | https://github.com/aizech/clinical-skills/blob/743831b202a38977ed594eb5b1f21032800c41b2/.agents/skills/ai-report-assist/SKILL.md | https://github.com/aizech/clinical-skills/blob/743831b202a38977ed594eb5b1f21032800c41b2/skills/clinical-documentation/imaging-study-review/SKILL.md</x:v>
+      </x:c>
+      <x:c r="M156" s="11" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N156" s="11" t="str">
+        <x:v>aizech</x:v>
+      </x:c>
+      <x:c r="O156" s="11" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P156" s="11" t="str">
+        <x:v>See pinned project manifest and setup documentation</x:v>
+      </x:c>
+      <x:c r="Q156" s="11" t="str">
+        <x:v>See pinned setup; varies by component</x:v>
+      </x:c>
+      <x:c r="R156" s="11" t="str">
+        <x:v>See capability and limitation fields; no runtime actions performed</x:v>
+      </x:c>
+      <x:c r="S156" s="11" t="str">
+        <x:v>See pinned project setup; external data access may require credentials.</x:v>
+      </x:c>
+      <x:c r="T156" s="14" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+      <x:c r="U156" s="14" t="n">
+        <x:v>46194.853993055556</x:v>
+      </x:c>
+      <x:c r="V156" s="11" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="W156" s="11" t="str">
+        <x:v>https://github.com/aizech/clinical-skills</x:v>
+      </x:c>
+      <x:c r="X156" s="11" t="str">
+        <x:v>https://github.com/aizech/clinical-skills</x:v>
+      </x:c>
+      <x:c r="Y156" s="11" t="str">
+        <x:v>https://github.com/aizech/clinical-skills/blob/743831b202a38977ed594eb5b1f21032800c41b2/README.md | https://github.com/aizech/clinical-skills/blob/743831b202a38977ed594eb5b1f21032800c41b2/.agents/skills/ai-detection-pipeline/SKILL.md | https://github.com/aizech/clinical-skills/blob/743831b202a38977ed594eb5b1f21032800c41b2/.agents/skills/ai-quality-review/SKILL.md | https://github.com/aizech/clinical-skills/blob/743831b202a38977ed594eb5b1f21032800c41b2/.agents/skills/ai-report-assist/SKILL.md | https://github.com/aizech/clinical-skills/blob/743831b202a38977ed594eb5b1f21032800c41b2/skills/clinical-documentation/imaging-study-review/SKILL.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="157" ht="132" hidden="0" customHeight="1">
+      <x:c r="A157" s="11" t="str">
+        <x:v>RWE-0169</x:v>
+      </x:c>
+      <x:c r="B157" s="11" t="str">
+        <x:v>ClinicalAI MCP</x:v>
+      </x:c>
+      <x:c r="C157" s="11" t="str">
+        <x:v>MCP server collection</x:v>
+      </x:c>
+      <x:c r="D157" s="11" t="str">
+        <x:v>Biomedical &amp; RWE Infrastructure</x:v>
+      </x:c>
+      <x:c r="E157" s="11" t="str">
+        <x:v>Collection of clinical MCP components for evidence, terminology, drugs and calculations.</x:v>
+      </x:c>
+      <x:c r="F157" s="11" t="str">
+        <x:v>Biomedical | MCP server collection</x:v>
+      </x:c>
+      <x:c r="G157" s="11" t="str">
+        <x:v>Biomedical &amp; RWE Infrastructure | Source inspection and research preparation</x:v>
+      </x:c>
+      <x:c r="H157" s="11" t="str">
+        <x:v>Expose modular clinical-reference and evidence tools | Support terminology and calculation workflows with shared utilities</x:v>
+      </x:c>
+      <x:c r="I157" s="11" t="str">
+        <x:v>Publisher identifies clinician validation as pending. Do not infer calculator validity or privacy compliance; some terminology and data sources need separate licenses.</x:v>
+      </x:c>
+      <x:c r="J157" s="11" t="str">
+        <x:v>Static source and documentation reviewed</x:v>
+      </x:c>
+      <x:c r="K157" s="11" t="str">
+        <x:v>Canonical repository metadata reviewed at commit ec1447a16fcc37f63c8d3031da325b2bd63c1f4f</x:v>
+      </x:c>
+      <x:c r="L157" s="11" t="str">
+        <x:v>https://github.com/OpenClinicalAI/clinicalai-mcp/blob/ec1447a16fcc37f63c8d3031da325b2bd63c1f4f/README.md | https://github.com/OpenClinicalAI/clinicalai-mcp/blob/ec1447a16fcc37f63c8d3031da325b2bd63c1f4f/package.json | https://github.com/OpenClinicalAI/clinicalai-mcp/blob/ec1447a16fcc37f63c8d3031da325b2bd63c1f4f/packages/calc/src/tools.ts | https://github.com/OpenClinicalAI/clinicalai-mcp/blob/ec1447a16fcc37f63c8d3031da325b2bd63c1f4f/packages/shared/src/server.ts</x:v>
+      </x:c>
+      <x:c r="M157" s="11" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N157" s="11" t="str">
+        <x:v>OpenClinicalAI</x:v>
+      </x:c>
+      <x:c r="O157" s="11" t="str">
+        <x:v>Apache-2.0</x:v>
+      </x:c>
+      <x:c r="P157" s="11" t="str">
+        <x:v>See pinned project manifest and setup documentation</x:v>
+      </x:c>
+      <x:c r="Q157" s="11" t="str">
+        <x:v>See pinned setup; varies by component</x:v>
+      </x:c>
+      <x:c r="R157" s="11" t="str">
+        <x:v>See capability and limitation fields; no runtime actions performed</x:v>
+      </x:c>
+      <x:c r="S157" s="11" t="str">
+        <x:v>See pinned project setup; external data access may require credentials.</x:v>
+      </x:c>
+      <x:c r="T157" s="14" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+      <x:c r="U157" s="14" t="n">
+        <x:v>46168.10497685185</x:v>
+      </x:c>
+      <x:c r="V157" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="W157" s="11" t="str">
+        <x:v>https://github.com/OpenClinicalAI/clinicalai-mcp</x:v>
+      </x:c>
+      <x:c r="X157" s="11" t="str">
+        <x:v>https://github.com/OpenClinicalAI/clinicalai-mcp</x:v>
+      </x:c>
+      <x:c r="Y157" s="11" t="str">
+        <x:v>https://github.com/OpenClinicalAI/clinicalai-mcp/blob/ec1447a16fcc37f63c8d3031da325b2bd63c1f4f/README.md | https://github.com/OpenClinicalAI/clinicalai-mcp/blob/ec1447a16fcc37f63c8d3031da325b2bd63c1f4f/package.json | https://github.com/OpenClinicalAI/clinicalai-mcp/blob/ec1447a16fcc37f63c8d3031da325b2bd63c1f4f/packages/calc/src/tools.ts | https://github.com/OpenClinicalAI/clinicalai-mcp/blob/ec1447a16fcc37f63c8d3031da325b2bd63c1f4f/packages/shared/src/server.ts</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="158" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A158" s="11" t="str">
+        <x:v>RWE-0176</x:v>
+      </x:c>
+      <x:c r="B158" s="11" t="str">
+        <x:v>ClinicalTrials MCP Server (JackKuo666)</x:v>
+      </x:c>
+      <x:c r="C158" s="11" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D158" s="11" t="str">
+        <x:v>Trials &amp; Study Design</x:v>
+      </x:c>
+      <x:c r="E158" s="11" t="str">
+        <x:v>Queries ClinicalTrials.gov and supports local trial-result exports.</x:v>
+      </x:c>
+      <x:c r="F158" s="11" t="str">
+        <x:v>Trials | MCP server</x:v>
+      </x:c>
+      <x:c r="G158" s="11" t="str">
+        <x:v>Trials &amp; Study Design | Source inspection and research preparation</x:v>
+      </x:c>
+      <x:c r="H158" s="11" t="str">
+        <x:v>Search trials and retrieve NCT study details | Save or load CSV results and inspect trial statistics</x:v>
+      </x:c>
+      <x:c r="I158" s="11" t="str">
+        <x:v>Registry entries can be incomplete or revised. Preserve query and retrieval dates; a saved CSV is a snapshot, not evidence that a search is exhaustive.</x:v>
+      </x:c>
+      <x:c r="J158" s="11" t="str">
+        <x:v>Static source and documentation reviewed</x:v>
+      </x:c>
+      <x:c r="K158" s="11" t="str">
+        <x:v>Canonical repository metadata reviewed at commit 2f9e1dce94f3fe158c7dc62cffa428d74583e9e7</x:v>
+      </x:c>
+      <x:c r="L158" s="11" t="str">
+        <x:v>https://github.com/JackKuo666/ClinicalTrials-MCP-Server/blob/2f9e1dce94f3fe158c7dc62cffa428d74583e9e7/README.md</x:v>
+      </x:c>
+      <x:c r="M158" s="11" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N158" s="11" t="str">
+        <x:v>JackKuo666</x:v>
+      </x:c>
+      <x:c r="O158" s="11" t="str">
+        <x:v>Not specified</x:v>
+      </x:c>
+      <x:c r="P158" s="11" t="str">
+        <x:v>See pinned project manifest and setup documentation</x:v>
+      </x:c>
+      <x:c r="Q158" s="11" t="str">
+        <x:v>See pinned setup; varies by component</x:v>
+      </x:c>
+      <x:c r="R158" s="11" t="str">
+        <x:v>See capability and limitation fields; no runtime actions performed</x:v>
+      </x:c>
+      <x:c r="S158" s="11" t="str">
+        <x:v>See pinned project setup; external data access may require credentials.</x:v>
+      </x:c>
+      <x:c r="T158" s="14" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+      <x:c r="U158" s="14" t="n">
+        <x:v>45756.477268518516</x:v>
+      </x:c>
+      <x:c r="V158" s="11" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="W158" s="11" t="str">
+        <x:v>https://github.com/JackKuo666/ClinicalTrials-MCP-Server</x:v>
+      </x:c>
+      <x:c r="X158" s="11" t="str">
+        <x:v>https://github.com/JackKuo666/ClinicalTrials-MCP-Server</x:v>
+      </x:c>
+      <x:c r="Y158" s="11" t="str">
+        <x:v>https://github.com/JackKuo666/ClinicalTrials-MCP-Server/blob/2f9e1dce94f3fe158c7dc62cffa428d74583e9e7/README.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="159" ht="118.80000305175781" hidden="0" customHeight="1">
+      <x:c r="A159" s="11" t="str">
+        <x:v>RWE-0178</x:v>
+      </x:c>
+      <x:c r="B159" s="11" t="str">
+        <x:v>Drug Pipeline MCP</x:v>
+      </x:c>
+      <x:c r="C159" s="11" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D159" s="11" t="str">
+        <x:v>Pharmacovigilance &amp; safety</x:v>
+      </x:c>
+      <x:c r="E159" s="11" t="str">
+        <x:v>Combines trial, regulatory and safety-source retrieval for drug evidence exploration.</x:v>
+      </x:c>
+      <x:c r="F159" s="11" t="str">
+        <x:v>Pharmacovigilance | MCP server</x:v>
+      </x:c>
+      <x:c r="G159" s="11" t="str">
+        <x:v>Pharmacovigilance &amp; safety | Source inspection and research preparation</x:v>
+      </x:c>
+      <x:c r="H159" s="11" t="str">
+        <x:v>Retrieve trial protocols, results and locations | Explore FDA/EMA product records and FAERS-based safety information</x:v>
+      </x:c>
+      <x:c r="I159" s="11" t="str">
+        <x:v>Spontaneous-report signals are not incidence or causal estimates. Verify source coverage, dates and derived calculations; pipeline and patent estimates need separate confirmation.</x:v>
+      </x:c>
+      <x:c r="J159" s="11" t="str">
+        <x:v>Static source and documentation reviewed</x:v>
+      </x:c>
+      <x:c r="K159" s="11" t="str">
+        <x:v>Canonical repository metadata reviewed at commit c9bcae8d108789fb450a2c812739e96998fbbbb2</x:v>
+      </x:c>
+      <x:c r="L159" s="11" t="str">
+        <x:v>https://github.com/DasClown/drug-pipeline-mcp/blob/c9bcae8d108789fb450a2c812739e96998fbbbb2/README.md | https://github.com/DasClown/drug-pipeline-mcp/blob/c9bcae8d108789fb450a2c812739e96998fbbbb2/pyproject.toml | https://github.com/DasClown/drug-pipeline-mcp/blob/c9bcae8d108789fb450a2c812739e96998fbbbb2/server.json | https://github.com/DasClown/drug-pipeline-mcp/blob/c9bcae8d108789fb450a2c812739e96998fbbbb2/drug_pipeline/server.py</x:v>
+      </x:c>
+      <x:c r="M159" s="11" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N159" s="11" t="str">
+        <x:v>DasClown</x:v>
+      </x:c>
+      <x:c r="O159" s="11" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P159" s="11" t="str">
+        <x:v>See pinned project manifest and setup documentation</x:v>
+      </x:c>
+      <x:c r="Q159" s="11" t="str">
+        <x:v>See pinned setup; varies by component</x:v>
+      </x:c>
+      <x:c r="R159" s="11" t="str">
+        <x:v>See capability and limitation fields; no runtime actions performed</x:v>
+      </x:c>
+      <x:c r="S159" s="11" t="str">
+        <x:v>See pinned project setup; external data access may require credentials.</x:v>
+      </x:c>
+      <x:c r="T159" s="14" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+      <x:c r="U159" s="14" t="n">
+        <x:v>46210.255833333336</x:v>
+      </x:c>
+      <x:c r="V159" s="11" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="W159" s="11" t="str">
+        <x:v>https://github.com/DasClown/drug-pipeline-mcp</x:v>
+      </x:c>
+      <x:c r="X159" s="11" t="str">
+        <x:v>https://github.com/DasClown/drug-pipeline-mcp</x:v>
+      </x:c>
+      <x:c r="Y159" s="11" t="str">
+        <x:v>https://github.com/DasClown/drug-pipeline-mcp/blob/c9bcae8d108789fb450a2c812739e96998fbbbb2/README.md | https://github.com/DasClown/drug-pipeline-mcp/blob/c9bcae8d108789fb450a2c812739e96998fbbbb2/pyproject.toml | https://github.com/DasClown/drug-pipeline-mcp/blob/c9bcae8d108789fb450a2c812739e96998fbbbb2/server.json | https://github.com/DasClown/drug-pipeline-mcp/blob/c9bcae8d108789fb450a2c812739e96998fbbbb2/drug_pipeline/server.py</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="160" ht="132" hidden="0" customHeight="1">
+      <x:c r="A160" s="11" t="str">
+        <x:v>RWE-0153</x:v>
+      </x:c>
+      <x:c r="B160" s="11" t="str">
+        <x:v>FDA Approvals MCP</x:v>
+      </x:c>
+      <x:c r="C160" s="11" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D160" s="11" t="str">
+        <x:v>Regulatory &amp; Product Data</x:v>
+      </x:c>
+      <x:c r="E160" s="11" t="str">
+        <x:v>Hosted connector for FDA product, labeling, recall and safety-source searches.</x:v>
+      </x:c>
+      <x:c r="F160" s="11" t="str">
+        <x:v>Regulatory | MCP server</x:v>
+      </x:c>
+      <x:c r="G160" s="11" t="str">
+        <x:v>Regulatory &amp; Product Data | Source inspection and research preparation</x:v>
+      </x:c>
+      <x:c r="H160" s="11" t="str">
+        <x:v>Search approval, labeling and recall information | Retrieve adverse-event and device-related source records</x:v>
+      </x:c>
+      <x:c r="I160" s="11" t="str">
+        <x:v>Hosted service access and limits may change. Deduplication and synthesis claims were not independently validated; check source identifiers and reporting limitations.</x:v>
+      </x:c>
+      <x:c r="J160" s="11" t="str">
+        <x:v>Static source and documentation reviewed</x:v>
+      </x:c>
+      <x:c r="K160" s="11" t="str">
+        <x:v>Canonical repository metadata reviewed at commit 73940ca6b152bc52fb7f8fe65b24b0305eb888e1</x:v>
+      </x:c>
+      <x:c r="L160" s="11" t="str">
+        <x:v>https://github.com/guptaprakhariitr/fda-approvals-mcp/blob/73940ca6b152bc52fb7f8fe65b24b0305eb888e1/README.md | https://github.com/guptaprakhariitr/fda-approvals-mcp/blob/73940ca6b152bc52fb7f8fe65b24b0305eb888e1/package.json | https://github.com/guptaprakhariitr/fda-approvals-mcp/blob/73940ca6b152bc52fb7f8fe65b24b0305eb888e1/server.json | https://github.com/guptaprakhariitr/fda-approvals-mcp/blob/73940ca6b152bc52fb7f8fe65b24b0305eb888e1/src/tools.ts</x:v>
+      </x:c>
+      <x:c r="M160" s="11" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N160" s="11" t="str">
+        <x:v>guptaprakhariitr</x:v>
+      </x:c>
+      <x:c r="O160" s="11" t="str">
+        <x:v>NOASSERTION</x:v>
+      </x:c>
+      <x:c r="P160" s="11" t="str">
+        <x:v>See pinned project manifest and setup documentation</x:v>
+      </x:c>
+      <x:c r="Q160" s="11" t="str">
+        <x:v>See pinned setup; varies by component</x:v>
+      </x:c>
+      <x:c r="R160" s="11" t="str">
+        <x:v>See capability and limitation fields; no runtime actions performed</x:v>
+      </x:c>
+      <x:c r="S160" s="11" t="str">
+        <x:v>Hosted service credentials and plan-dependent access; see publisher setup.</x:v>
+      </x:c>
+      <x:c r="T160" s="14" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+      <x:c r="U160" s="14" t="n">
+        <x:v>46184.36068287037</x:v>
+      </x:c>
+      <x:c r="V160" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="W160" s="11" t="str">
+        <x:v>https://github.com/guptaprakhariitr/fda-approvals-mcp</x:v>
+      </x:c>
+      <x:c r="X160" s="11" t="str">
+        <x:v>https://github.com/guptaprakhariitr/fda-approvals-mcp</x:v>
+      </x:c>
+      <x:c r="Y160" s="11" t="str">
+        <x:v>https://github.com/guptaprakhariitr/fda-approvals-mcp/blob/73940ca6b152bc52fb7f8fe65b24b0305eb888e1/README.md | https://github.com/guptaprakhariitr/fda-approvals-mcp/blob/73940ca6b152bc52fb7f8fe65b24b0305eb888e1/package.json | https://github.com/guptaprakhariitr/fda-approvals-mcp/blob/73940ca6b152bc52fb7f8fe65b24b0305eb888e1/server.json | https://github.com/guptaprakhariitr/fda-approvals-mcp/blob/73940ca6b152bc52fb7f8fe65b24b0305eb888e1/src/tools.ts</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="161" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A161" s="11" t="str">
+        <x:v>RWE-0155</x:v>
+      </x:c>
+      <x:c r="B161" s="11" t="str">
+        <x:v>FDA MCP (Limecooler)</x:v>
+      </x:c>
+      <x:c r="C161" s="11" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D161" s="11" t="str">
+        <x:v>Regulatory &amp; Product Data</x:v>
+      </x:c>
+      <x:c r="E161" s="11" t="str">
+        <x:v>Searches FDA datasets and retrieves linked regulatory document content.</x:v>
+      </x:c>
+      <x:c r="F161" s="11" t="str">
+        <x:v>Regulatory | MCP server</x:v>
+      </x:c>
+      <x:c r="G161" s="11" t="str">
+        <x:v>Regulatory &amp; Product Data | Source inspection and research preparation</x:v>
+      </x:c>
+      <x:c r="H161" s="11" t="str">
+        <x:v>Search records, count results and inspect available fields | Retrieve supported decision documents and extract PDF text</x:v>
+      </x:c>
+      <x:c r="I161" s="11" t="str">
+        <x:v>Field availability and source indexing vary. PDF/OCR text and count queries require verification; data retrieval does not establish safety or effectiveness.</x:v>
+      </x:c>
+      <x:c r="J161" s="11" t="str">
+        <x:v>Static source and documentation reviewed</x:v>
+      </x:c>
+      <x:c r="K161" s="11" t="str">
+        <x:v>Canonical repository metadata reviewed at commit 23ed29d5d8fc465967bed554875f1ebd0a6720b9</x:v>
+      </x:c>
+      <x:c r="L161" s="11" t="str">
+        <x:v>https://github.com/Limecooler/fda-mcp/blob/23ed29d5d8fc465967bed554875f1ebd0a6720b9/README.md | https://github.com/Limecooler/fda-mcp/blob/23ed29d5d8fc465967bed554875f1ebd0a6720b9/pyproject.toml | https://github.com/Limecooler/fda-mcp/blob/23ed29d5d8fc465967bed554875f1ebd0a6720b9/src/fda_mcp/server.py</x:v>
+      </x:c>
+      <x:c r="M161" s="11" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N161" s="11" t="str">
+        <x:v>Limecooler</x:v>
+      </x:c>
+      <x:c r="O161" s="11" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P161" s="11" t="str">
+        <x:v>See pinned project manifest and setup documentation</x:v>
+      </x:c>
+      <x:c r="Q161" s="11" t="str">
+        <x:v>See pinned setup; varies by component</x:v>
+      </x:c>
+      <x:c r="R161" s="11" t="str">
+        <x:v>See capability and limitation fields; no runtime actions performed</x:v>
+      </x:c>
+      <x:c r="S161" s="11" t="str">
+        <x:v>See pinned project setup; external data access may require credentials.</x:v>
+      </x:c>
+      <x:c r="T161" s="14" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+      <x:c r="U161" s="14" t="n">
+        <x:v>46073.15766203704</x:v>
+      </x:c>
+      <x:c r="V161" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="W161" s="11" t="str">
+        <x:v>https://github.com/Limecooler/fda-mcp</x:v>
+      </x:c>
+      <x:c r="X161" s="11" t="str">
+        <x:v>https://github.com/Limecooler/fda-mcp</x:v>
+      </x:c>
+      <x:c r="Y161" s="11" t="str">
+        <x:v>https://github.com/Limecooler/fda-mcp/blob/23ed29d5d8fc465967bed554875f1ebd0a6720b9/README.md | https://github.com/Limecooler/fda-mcp/blob/23ed29d5d8fc465967bed554875f1ebd0a6720b9/pyproject.toml | https://github.com/Limecooler/fda-mcp/blob/23ed29d5d8fc465967bed554875f1ebd0a6720b9/src/fda_mcp/server.py</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="162" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A162" s="11" t="str">
+        <x:v>RWE-0179</x:v>
+      </x:c>
+      <x:c r="B162" s="11" t="str">
+        <x:v>Helix</x:v>
+      </x:c>
+      <x:c r="C162" s="11" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D162" s="11" t="str">
+        <x:v>Literature &amp; Evidence Synthesis</x:v>
+      </x:c>
+      <x:c r="E162" s="11" t="str">
+        <x:v>Combines ClinicalTrials.gov, PubMed and FDA labeling retrieval with preliminary evidence ranking.</x:v>
+      </x:c>
+      <x:c r="F162" s="11" t="str">
+        <x:v>Literature | MCP server</x:v>
+      </x:c>
+      <x:c r="G162" s="11" t="str">
+        <x:v>Literature &amp; Evidence Synthesis | Source inspection and research preparation</x:v>
+      </x:c>
+      <x:c r="H162" s="11" t="str">
+        <x:v>Retrieve trial, publication and drug-label context | Produce heuristic evidence and eligibility-oriented rankings</x:v>
+      </x:c>
+      <x:c r="I162" s="11" t="str">
+        <x:v>Ranking formulas are not validated evidence grades or clinical eligibility determinations. Review original records and use a prespecified synthesis protocol.</x:v>
+      </x:c>
+      <x:c r="J162" s="11" t="str">
+        <x:v>Static source and documentation reviewed</x:v>
+      </x:c>
+      <x:c r="K162" s="11" t="str">
+        <x:v>Canonical repository metadata reviewed at commit eb725da1d89a90968a916c2efa327861a7d1291d</x:v>
+      </x:c>
+      <x:c r="L162" s="11" t="str">
+        <x:v>https://github.com/Al1Abdullah/Helix/blob/eb725da1d89a90968a916c2efa327861a7d1291d/README.md | https://github.com/Al1Abdullah/Helix/blob/eb725da1d89a90968a916c2efa327861a7d1291d/pyproject.toml | https://github.com/Al1Abdullah/Helix/blob/eb725da1d89a90968a916c2efa327861a7d1291d/src/helix/server.py</x:v>
+      </x:c>
+      <x:c r="M162" s="11" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N162" s="11" t="str">
+        <x:v>Al1Abdullah</x:v>
+      </x:c>
+      <x:c r="O162" s="11" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P162" s="11" t="str">
+        <x:v>See pinned project manifest and setup documentation</x:v>
+      </x:c>
+      <x:c r="Q162" s="11" t="str">
+        <x:v>See pinned setup; varies by component</x:v>
+      </x:c>
+      <x:c r="R162" s="11" t="str">
+        <x:v>See capability and limitation fields; no runtime actions performed</x:v>
+      </x:c>
+      <x:c r="S162" s="11" t="str">
+        <x:v>See pinned project setup; external data access may require credentials.</x:v>
+      </x:c>
+      <x:c r="T162" s="14" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+      <x:c r="U162" s="14" t="n">
+        <x:v>46171.382835648146</x:v>
+      </x:c>
+      <x:c r="V162" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="W162" s="11" t="str">
+        <x:v>https://github.com/Al1Abdullah/Helix</x:v>
+      </x:c>
+      <x:c r="X162" s="11" t="str">
+        <x:v>https://github.com/Al1Abdullah/Helix</x:v>
+      </x:c>
+      <x:c r="Y162" s="11" t="str">
+        <x:v>https://github.com/Al1Abdullah/Helix/blob/eb725da1d89a90968a916c2efa327861a7d1291d/README.md | https://github.com/Al1Abdullah/Helix/blob/eb725da1d89a90968a916c2efa327861a7d1291d/pyproject.toml | https://github.com/Al1Abdullah/Helix/blob/eb725da1d89a90968a916c2efa327861a7d1291d/src/helix/server.py</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="163" ht="184.8000030517578" hidden="0" customHeight="1">
+      <x:c r="A163" s="11" t="str">
+        <x:v>RWE-0165</x:v>
+      </x:c>
+      <x:c r="B163" s="11" t="str">
+        <x:v>LabClaw</x:v>
+      </x:c>
+      <x:c r="C163" s="11" t="str">
+        <x:v>Agent skill collection</x:v>
+      </x:c>
+      <x:c r="D163" s="11" t="str">
+        <x:v>Biomedical &amp; RWE Infrastructure</x:v>
+      </x:c>
+      <x:c r="E163" s="11" t="str">
+        <x:v>Agent skill collection spanning biomedical analysis, literature retrieval and statistical workflows.</x:v>
+      </x:c>
+      <x:c r="F163" s="11" t="str">
+        <x:v>Biomedical | Agent skill collection</x:v>
+      </x:c>
+      <x:c r="G163" s="11" t="str">
+        <x:v>Biomedical &amp; RWE Infrastructure | Source inspection and research preparation</x:v>
+      </x:c>
+      <x:c r="H163" s="11" t="str">
+        <x:v>Provide clinical-trial and literature-search skills | Guide survival and statistical-analysis workflows</x:v>
+      </x:c>
+      <x:c r="I163" s="11" t="str">
+        <x:v>Skills may wrap or reproduce upstream tools and require their dependencies. Repository affiliation and method claims are not independent validation.</x:v>
+      </x:c>
+      <x:c r="J163" s="11" t="str">
+        <x:v>Static source and documentation reviewed</x:v>
+      </x:c>
+      <x:c r="K163" s="11" t="str">
+        <x:v>Canonical repository metadata reviewed at commit 205972f93402f874a54b9a5e1b590151ece6432b</x:v>
+      </x:c>
+      <x:c r="L163" s="11" t="str">
+        <x:v>https://github.com/bilalmirza96/LabClaw/blob/205972f93402f874a54b9a5e1b590151ece6432b/README.md | https://github.com/bilalmirza96/LabClaw/blob/205972f93402f874a54b9a5e1b590151ece6432b/skills/bio/alphafold-database/SKILL.md | https://github.com/bilalmirza96/LabClaw/blob/205972f93402f874a54b9a5e1b590151ece6432b/skills/bio/analyze_lab_video_cell_behavior/SKILL.md | https://github.com/bilalmirza96/LabClaw/blob/205972f93402f874a54b9a5e1b590151ece6432b/skills/bio/anndata/SKILL.md | https://github.com/bilalmirza96/LabClaw/blob/205972f93402f874a54b9a5e1b590151ece6432b/skills/literature/clinical-trials-search/SKILL.md</x:v>
+      </x:c>
+      <x:c r="M163" s="11" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N163" s="11" t="str">
+        <x:v>bilalmirza96</x:v>
+      </x:c>
+      <x:c r="O163" s="11" t="str">
+        <x:v>Not specified</x:v>
+      </x:c>
+      <x:c r="P163" s="11" t="str">
+        <x:v>See pinned project manifest and setup documentation</x:v>
+      </x:c>
+      <x:c r="Q163" s="11" t="str">
+        <x:v>See pinned setup; varies by component</x:v>
+      </x:c>
+      <x:c r="R163" s="11" t="str">
+        <x:v>See capability and limitation fields; no runtime actions performed</x:v>
+      </x:c>
+      <x:c r="S163" s="11" t="str">
+        <x:v>See pinned project setup; external data access may require credentials.</x:v>
+      </x:c>
+      <x:c r="T163" s="14" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+      <x:c r="U163" s="14" t="n">
+        <x:v>46116.10565972222</x:v>
+      </x:c>
+      <x:c r="V163" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="W163" s="11" t="str">
+        <x:v>https://github.com/bilalmirza96/LabClaw</x:v>
+      </x:c>
+      <x:c r="X163" s="11" t="str">
+        <x:v>https://github.com/bilalmirza96/LabClaw</x:v>
+      </x:c>
+      <x:c r="Y163" s="11" t="str">
+        <x:v>https://github.com/bilalmirza96/LabClaw/blob/205972f93402f874a54b9a5e1b590151ece6432b/README.md | https://github.com/bilalmirza96/LabClaw/blob/205972f93402f874a54b9a5e1b590151ece6432b/skills/bio/alphafold-database/SKILL.md | https://github.com/bilalmirza96/LabClaw/blob/205972f93402f874a54b9a5e1b590151ece6432b/skills/bio/analyze_lab_video_cell_behavior/SKILL.md | https://github.com/bilalmirza96/LabClaw/blob/205972f93402f874a54b9a5e1b590151ece6432b/skills/bio/anndata/SKILL.md | https://github.com/bilalmirza96/LabClaw/blob/205972f93402f874a54b9a5e1b590151ece6432b/skills/literature/clinical-trials-search/SKILL.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="164" ht="132" hidden="0" customHeight="1">
+      <x:c r="A164" s="11" t="str">
+        <x:v>RWE-0166</x:v>
+      </x:c>
+      <x:c r="B164" s="11" t="str">
+        <x:v>MedgeClaw</x:v>
+      </x:c>
+      <x:c r="C164" s="11" t="str">
+        <x:v>Agent workflow + skill integration</x:v>
+      </x:c>
+      <x:c r="D164" s="11" t="str">
+        <x:v>Biomedical &amp; RWE Infrastructure</x:v>
+      </x:c>
+      <x:c r="E164" s="11" t="str">
+        <x:v>Biomedical agent workflow combining OpenClaw, coding agents and research skills.</x:v>
+      </x:c>
+      <x:c r="F164" s="11" t="str">
+        <x:v>Biomedical | Agent workflow + skill integration</x:v>
+      </x:c>
+      <x:c r="G164" s="11" t="str">
+        <x:v>Biomedical &amp; RWE Infrastructure | Source inspection and research preparation</x:v>
+      </x:c>
+      <x:c r="H164" s="11" t="str">
+        <x:v>Coordinate biomedical analysis through coding-agent workflows | Support R/Python research environments and external skill integrations</x:v>
+      </x:c>
+      <x:c r="I164" s="11" t="str">
+        <x:v>Runs generated code and may connect messaging services. Review data routing, dependencies and generated analyses; underlying skills are not new independently validated methods.</x:v>
+      </x:c>
+      <x:c r="J164" s="11" t="str">
+        <x:v>Static source and documentation reviewed</x:v>
+      </x:c>
+      <x:c r="K164" s="11" t="str">
+        <x:v>Canonical repository metadata reviewed at commit fef51d37ee3e1f5754790d9ae20f72c006c78dcc</x:v>
+      </x:c>
+      <x:c r="L164" s="11" t="str">
+        <x:v>https://github.com/xjtulyc/MedgeClaw/blob/fef51d37ee3e1f5754790d9ae20f72c006c78dcc/README.md | https://github.com/xjtulyc/MedgeClaw/blob/fef51d37ee3e1f5754790d9ae20f72c006c78dcc/skills/biomed-dispatch/SKILL.md | https://github.com/xjtulyc/MedgeClaw/blob/fef51d37ee3e1f5754790d9ae20f72c006c78dcc/skills/charls-reproduce/SKILL.md | https://github.com/xjtulyc/MedgeClaw/blob/fef51d37ee3e1f5754790d9ae20f72c006c78dcc/skills/cjk-viz/SKILL.md</x:v>
+      </x:c>
+      <x:c r="M164" s="11" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N164" s="11" t="str">
+        <x:v>xjtulyc</x:v>
+      </x:c>
+      <x:c r="O164" s="11" t="str">
+        <x:v>Not specified</x:v>
+      </x:c>
+      <x:c r="P164" s="11" t="str">
+        <x:v>See pinned project manifest and setup documentation</x:v>
+      </x:c>
+      <x:c r="Q164" s="11" t="str">
+        <x:v>See pinned setup; varies by component</x:v>
+      </x:c>
+      <x:c r="R164" s="11" t="str">
+        <x:v>See capability and limitation fields; no runtime actions performed</x:v>
+      </x:c>
+      <x:c r="S164" s="11" t="str">
+        <x:v>See pinned project setup; external data access may require credentials.</x:v>
+      </x:c>
+      <x:c r="T164" s="14" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+      <x:c r="U164" s="14" t="n">
+        <x:v>46093.315729166665</x:v>
+      </x:c>
+      <x:c r="V164" s="11" t="n">
+        <x:v>642</x:v>
+      </x:c>
+      <x:c r="W164" s="11" t="str">
+        <x:v>https://github.com/xjtulyc/MedgeClaw</x:v>
+      </x:c>
+      <x:c r="X164" s="11" t="str">
+        <x:v>https://github.com/xjtulyc/MedgeClaw</x:v>
+      </x:c>
+      <x:c r="Y164" s="11" t="str">
+        <x:v>https://github.com/xjtulyc/MedgeClaw/blob/fef51d37ee3e1f5754790d9ae20f72c006c78dcc/README.md | https://github.com/xjtulyc/MedgeClaw/blob/fef51d37ee3e1f5754790d9ae20f72c006c78dcc/skills/biomed-dispatch/SKILL.md | https://github.com/xjtulyc/MedgeClaw/blob/fef51d37ee3e1f5754790d9ae20f72c006c78dcc/skills/charls-reproduce/SKILL.md | https://github.com/xjtulyc/MedgeClaw/blob/fef51d37ee3e1f5754790d9ae20f72c006c78dcc/skills/cjk-viz/SKILL.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="165" ht="92.4000015258789" hidden="0" customHeight="1">
+      <x:c r="A165" s="11" t="str">
+        <x:v>RWE-0168</x:v>
+      </x:c>
+      <x:c r="B165" s="11" t="str">
+        <x:v>Metis PH</x:v>
+      </x:c>
+      <x:c r="C165" s="11" t="str">
+        <x:v>Research assistant + MCP integration</x:v>
+      </x:c>
+      <x:c r="D165" s="11" t="str">
+        <x:v>Literature &amp; Evidence Synthesis</x:v>
+      </x:c>
+      <x:c r="E165" s="11" t="str">
+        <x:v>Research assistant for querying a local reference library and developing epidemiologic analysis workflows.</x:v>
+      </x:c>
+      <x:c r="F165" s="11" t="str">
+        <x:v>Literature | Research assistant + MCP integration</x:v>
+      </x:c>
+      <x:c r="G165" s="11" t="str">
+        <x:v>Literature &amp; Evidence Synthesis | Source inspection and research preparation</x:v>
+      </x:c>
+      <x:c r="H165" s="11" t="str">
+        <x:v>Search and cite a local research library | Use epidemiology-oriented skills and model-assisted reasoning</x:v>
+      </x:c>
+      <x:c r="I165" s="11" t="str">
+        <x:v>Evidence coverage depends on the supplied corpus. External model calls may transmit research content; generated methodological assertions need expert and source review.</x:v>
+      </x:c>
+      <x:c r="J165" s="11" t="str">
+        <x:v>Static source and documentation reviewed</x:v>
+      </x:c>
+      <x:c r="K165" s="11" t="str">
+        <x:v>Canonical repository metadata reviewed at commit c9902186aae622430e63260d4e96111bde44739b</x:v>
+      </x:c>
+      <x:c r="L165" s="11" t="str">
+        <x:v>https://github.com/SVerITG/Metis_PH/blob/c9902186aae622430e63260d4e96111bde44739b/README.md | https://github.com/SVerITG/Metis_PH/blob/c9902186aae622430e63260d4e96111bde44739b/server.json | https://github.com/SVerITG/Metis_PH/blob/c9902186aae622430e63260d4e96111bde44739b/system/mcp-server/src/metis_mcp/server.py</x:v>
+      </x:c>
+      <x:c r="M165" s="11" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N165" s="11" t="str">
+        <x:v>SVerITG</x:v>
+      </x:c>
+      <x:c r="O165" s="11" t="str">
+        <x:v>AGPL-3.0</x:v>
+      </x:c>
+      <x:c r="P165" s="11" t="str">
+        <x:v>See pinned project manifest and setup documentation</x:v>
+      </x:c>
+      <x:c r="Q165" s="11" t="str">
+        <x:v>See pinned setup; varies by component</x:v>
+      </x:c>
+      <x:c r="R165" s="11" t="str">
+        <x:v>See capability and limitation fields; no runtime actions performed</x:v>
+      </x:c>
+      <x:c r="S165" s="11" t="str">
+        <x:v>See pinned project setup; external data access may require credentials.</x:v>
+      </x:c>
+      <x:c r="T165" s="14" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+      <x:c r="U165" s="14" t="n">
+        <x:v>46271.58241898148</x:v>
+      </x:c>
+      <x:c r="V165" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="W165" s="11" t="str">
+        <x:v>https://github.com/SVerITG/Metis_PH</x:v>
+      </x:c>
+      <x:c r="X165" s="11" t="str">
+        <x:v>https://github.com/SVerITG/Metis_PH</x:v>
+      </x:c>
+      <x:c r="Y165" s="11" t="str">
+        <x:v>https://github.com/SVerITG/Metis_PH/blob/c9902186aae622430e63260d4e96111bde44739b/README.md | https://github.com/SVerITG/Metis_PH/blob/c9902186aae622430e63260d4e96111bde44739b/server.json | https://github.com/SVerITG/Metis_PH/blob/c9902186aae622430e63260d4e96111bde44739b/system/mcp-server/src/metis_mcp/server.py</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="166" ht="198" hidden="0" customHeight="1">
+      <x:c r="A166" s="11" t="str">
+        <x:v>RWE-0159</x:v>
+      </x:c>
+      <x:c r="B166" s="11" t="str">
+        <x:v>OpenFDA Semantic MCP</x:v>
+      </x:c>
+      <x:c r="C166" s="11" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D166" s="11" t="str">
+        <x:v>Regulatory &amp; Product Data</x:v>
+      </x:c>
+      <x:c r="E166" s="11" t="str">
+        <x:v>Provides domain-oriented tools over openFDA drug and safety information.</x:v>
+      </x:c>
+      <x:c r="F166" s="11" t="str">
+        <x:v>Regulatory | MCP server</x:v>
+      </x:c>
+      <x:c r="G166" s="11" t="str">
+        <x:v>Regulatory &amp; Product Data | Source inspection and research preparation</x:v>
+      </x:c>
+      <x:c r="H166" s="11" t="str">
+        <x:v>Retrieve semantic drug and product profiles | Explore source records through structured FDA-oriented queries</x:v>
+      </x:c>
+      <x:c r="I166" s="11" t="str">
+        <x:v>Semantic summaries and report counts need source verification. No independent support is claimed for anti-hallucination guarantees or causal safety conclusions.</x:v>
+      </x:c>
+      <x:c r="J166" s="11" t="str">
+        <x:v>Static source and documentation reviewed</x:v>
+      </x:c>
+      <x:c r="K166" s="11" t="str">
+        <x:v>Canonical repository metadata reviewed at commit bcd0e65abeb1e0271e8ee89686a1ad75f3fbac24</x:v>
+      </x:c>
+      <x:c r="L166" s="11" t="str">
+        <x:v>https://github.com/SuyashEkhande/OpenFDA-Semantic-MCP/blob/bcd0e65abeb1e0271e8ee89686a1ad75f3fbac24/README.md | https://github.com/SuyashEkhande/OpenFDA-Semantic-MCP/blob/bcd0e65abeb1e0271e8ee89686a1ad75f3fbac24/pyproject.toml | https://github.com/SuyashEkhande/OpenFDA-Semantic-MCP/blob/bcd0e65abeb1e0271e8ee89686a1ad75f3fbac24/src/openfda_mcp/domains/animal_veterinary/tools.py | https://github.com/SuyashEkhande/OpenFDA-Semantic-MCP/blob/bcd0e65abeb1e0271e8ee89686a1ad75f3fbac24/src/openfda_mcp/domains/cosmetics/tools.py | https://github.com/SuyashEkhande/OpenFDA-Semantic-MCP/blob/bcd0e65abeb1e0271e8ee89686a1ad75f3fbac24/src/openfda_mcp/domains/device/tools.py</x:v>
+      </x:c>
+      <x:c r="M166" s="11" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N166" s="11" t="str">
+        <x:v>SuyashEkhande</x:v>
+      </x:c>
+      <x:c r="O166" s="11" t="str">
+        <x:v>Not specified</x:v>
+      </x:c>
+      <x:c r="P166" s="11" t="str">
+        <x:v>See pinned project manifest and setup documentation</x:v>
+      </x:c>
+      <x:c r="Q166" s="11" t="str">
+        <x:v>See pinned setup; varies by component</x:v>
+      </x:c>
+      <x:c r="R166" s="11" t="str">
+        <x:v>See capability and limitation fields; no runtime actions performed</x:v>
+      </x:c>
+      <x:c r="S166" s="11" t="str">
+        <x:v>See pinned project setup; external data access may require credentials.</x:v>
+      </x:c>
+      <x:c r="T166" s="14" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+      <x:c r="U166" s="14" t="n">
+        <x:v>46124.55065972222</x:v>
+      </x:c>
+      <x:c r="V166" s="11" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="W166" s="11" t="str">
+        <x:v>https://github.com/SuyashEkhande/OpenFDA-Semantic-MCP</x:v>
+      </x:c>
+      <x:c r="X166" s="11" t="str">
+        <x:v>https://github.com/SuyashEkhande/OpenFDA-Semantic-MCP</x:v>
+      </x:c>
+      <x:c r="Y166" s="11" t="str">
+        <x:v>https://github.com/SuyashEkhande/OpenFDA-Semantic-MCP/blob/bcd0e65abeb1e0271e8ee89686a1ad75f3fbac24/README.md | https://github.com/SuyashEkhande/OpenFDA-Semantic-MCP/blob/bcd0e65abeb1e0271e8ee89686a1ad75f3fbac24/pyproject.toml | https://github.com/SuyashEkhande/OpenFDA-Semantic-MCP/blob/bcd0e65abeb1e0271e8ee89686a1ad75f3fbac24/src/openfda_mcp/domains/animal_veterinary/tools.py | https://github.com/SuyashEkhande/OpenFDA-Semantic-MCP/blob/bcd0e65abeb1e0271e8ee89686a1ad75f3fbac24/src/openfda_mcp/domains/cosmetics/tools.py | https://github.com/SuyashEkhande/OpenFDA-Semantic-MCP/blob/bcd0e65abeb1e0271e8ee89686a1ad75f3fbac24/src/openfda_mcp/domains/device/tools.py</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="167" ht="237.60000610351562" hidden="0" customHeight="1">
+      <x:c r="A167" s="11" t="str">
+        <x:v>RWE-0180</x:v>
+      </x:c>
+      <x:c r="B167" s="11" t="str">
+        <x:v>Research Workflow Assistant</x:v>
+      </x:c>
+      <x:c r="C167" s="11" t="str">
+        <x:v>Agent workflow + MCP integrations</x:v>
+      </x:c>
+      <x:c r="D167" s="11" t="str">
+        <x:v>Literature &amp; Evidence Synthesis</x:v>
+      </x:c>
+      <x:c r="E167" s="11" t="str">
+        <x:v>Agent workflow for literature work, citations and reproducible research documents.</x:v>
+      </x:c>
+      <x:c r="F167" s="11" t="str">
+        <x:v>Literature | Agent workflow + MCP integrations</x:v>
+      </x:c>
+      <x:c r="G167" s="11" t="str">
+        <x:v>Literature &amp; Evidence Synthesis | Source inspection and research preparation</x:v>
+      </x:c>
+      <x:c r="H167" s="11" t="str">
+        <x:v>Coordinate database and Zotero integrations | Guide systematic-review and Quarto research-document workflows</x:v>
+      </x:c>
+      <x:c r="I167" s="11" t="str">
+        <x:v>Generated searches, citations and reports require protocol review. Availability depends on external agents and MCP services; reporting-compliance claims are not independently verified.</x:v>
+      </x:c>
+      <x:c r="J167" s="11" t="str">
+        <x:v>Static source and documentation reviewed</x:v>
+      </x:c>
+      <x:c r="K167" s="11" t="str">
+        <x:v>Canonical repository metadata reviewed at commit 51dcaa8a22b8ee54cdcc864a7d3e92d63f2c4a1d</x:v>
+      </x:c>
+      <x:c r="L167" s="11" t="str">
+        <x:v>https://github.com/Intersect-Collaborations-LLC/research-workflow-assistant/blob/51dcaa8a22b8ee54cdcc864a7d3e92d63f2c4a1d/README.md | https://github.com/Intersect-Collaborations-LLC/research-workflow-assistant/blob/51dcaa8a22b8ee54cdcc864a7d3e92d63f2c4a1d/pyproject.toml | https://github.com/Intersect-Collaborations-LLC/research-workflow-assistant/blob/51dcaa8a22b8ee54cdcc864a7d3e92d63f2c4a1d/mcp-servers/bibliography-manager/src/bibliography_manager/server.py | https://github.com/Intersect-Collaborations-LLC/research-workflow-assistant/blob/51dcaa8a22b8ee54cdcc864a7d3e92d63f2c4a1d/mcp-servers/chat-exporter/src/chat_exporter/server.py | https://github.com/Intersect-Collaborations-LLC/research-workflow-assistant/blob/51dcaa8a22b8ee54cdcc864a7d3e92d63f2c4a1d/mcp-servers/crossref-server/src/crossref_server/server.py</x:v>
+      </x:c>
+      <x:c r="M167" s="11" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N167" s="11" t="str">
+        <x:v>Intersect-Collaborations-LLC</x:v>
+      </x:c>
+      <x:c r="O167" s="11" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P167" s="11" t="str">
+        <x:v>See pinned project manifest and setup documentation</x:v>
+      </x:c>
+      <x:c r="Q167" s="11" t="str">
+        <x:v>See pinned setup; varies by component</x:v>
+      </x:c>
+      <x:c r="R167" s="11" t="str">
+        <x:v>See capability and limitation fields; no runtime actions performed</x:v>
+      </x:c>
+      <x:c r="S167" s="11" t="str">
+        <x:v>See pinned project setup; external data access may require credentials.</x:v>
+      </x:c>
+      <x:c r="T167" s="14" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+      <x:c r="U167" s="14" t="n">
+        <x:v>46263.60564814815</x:v>
+      </x:c>
+      <x:c r="V167" s="11" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="W167" s="11" t="str">
+        <x:v>https://github.com/Intersect-Collaborations-LLC/research-workflow-assistant</x:v>
+      </x:c>
+      <x:c r="X167" s="11" t="str">
+        <x:v>https://github.com/Intersect-Collaborations-LLC/research-workflow-assistant</x:v>
+      </x:c>
+      <x:c r="Y167" s="11" t="str">
+        <x:v>https://github.com/Intersect-Collaborations-LLC/research-workflow-assistant/blob/51dcaa8a22b8ee54cdcc864a7d3e92d63f2c4a1d/README.md | https://github.com/Intersect-Collaborations-LLC/research-workflow-assistant/blob/51dcaa8a22b8ee54cdcc864a7d3e92d63f2c4a1d/pyproject.toml | https://github.com/Intersect-Collaborations-LLC/research-workflow-assistant/blob/51dcaa8a22b8ee54cdcc864a7d3e92d63f2c4a1d/mcp-servers/bibliography-manager/src/bibliography_manager/server.py | https://github.com/Intersect-Collaborations-LLC/research-workflow-assistant/blob/51dcaa8a22b8ee54cdcc864a7d3e92d63f2c4a1d/mcp-servers/chat-exporter/src/chat_exporter/server.py | https://github.com/Intersect-Collaborations-LLC/research-workflow-assistant/blob/51dcaa8a22b8ee54cdcc864a7d3e92d63f2c4a1d/mcp-servers/crossref-server/src/crossref_server/server.py</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="168" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A168" s="11" t="str">
+        <x:v>RWE-0131</x:v>
+      </x:c>
+      <x:c r="B168" s="11" t="str">
+        <x:v>Shiranui</x:v>
+      </x:c>
+      <x:c r="C168" s="11" t="str">
+        <x:v>R package + MCP server</x:v>
+      </x:c>
+      <x:c r="D168" s="11" t="str">
+        <x:v>OMOP &amp; terminology</x:v>
+      </x:c>
+      <x:c r="E168" s="11" t="str">
+        <x:v>R interface and MCP tooling for CDISC Library standards metadata.</x:v>
+      </x:c>
+      <x:c r="F168" s="11" t="str">
+        <x:v>OMOP | R package + MCP server</x:v>
+      </x:c>
+      <x:c r="G168" s="11" t="str">
+        <x:v>OMOP &amp; terminology | Source inspection and research preparation</x:v>
+      </x:c>
+      <x:c r="H168" s="11" t="str">
+        <x:v>Retrieve ADaM, SDTM, CDASH and SEND metadata | Explore controlled terminology and biomedical concepts</x:v>
+      </x:c>
+      <x:c r="I168" s="11" t="str">
+        <x:v>Provides standards references, not automatic conformity validation or a completed data transformation. Preserve standard versions and applicable access terms.</x:v>
+      </x:c>
+      <x:c r="J168" s="11" t="str">
+        <x:v>Static source and documentation reviewed</x:v>
+      </x:c>
+      <x:c r="K168" s="11" t="str">
+        <x:v>Canonical repository metadata reviewed at commit 2d77554e4a33b065ab826a73580e9a7e2644296e</x:v>
+      </x:c>
+      <x:c r="L168" s="11" t="str">
+        <x:v>https://github.com/i-akiya/Shiranui/blob/2d77554e4a33b065ab826a73580e9a7e2644296e/README.md | https://github.com/i-akiya/Shiranui/blob/2d77554e4a33b065ab826a73580e9a7e2644296e/pyproject.toml | https://github.com/i-akiya/Shiranui/blob/2d77554e4a33b065ab826a73580e9a7e2644296e/src/shiranui/server.py</x:v>
+      </x:c>
+      <x:c r="M168" s="11" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N168" s="11" t="str">
+        <x:v>i-akiya</x:v>
+      </x:c>
+      <x:c r="O168" s="11" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P168" s="11" t="str">
+        <x:v>See pinned project manifest and setup documentation</x:v>
+      </x:c>
+      <x:c r="Q168" s="11" t="str">
+        <x:v>See pinned setup; varies by component</x:v>
+      </x:c>
+      <x:c r="R168" s="11" t="str">
+        <x:v>See capability and limitation fields; no runtime actions performed</x:v>
+      </x:c>
+      <x:c r="S168" s="11" t="str">
+        <x:v>CDISC Library API key.</x:v>
+      </x:c>
+      <x:c r="T168" s="14" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+      <x:c r="U168" s="14" t="n">
+        <x:v>46032.52027777778</x:v>
+      </x:c>
+      <x:c r="V168" s="11" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="W168" s="11" t="str">
+        <x:v>https://github.com/i-akiya/Shiranui</x:v>
+      </x:c>
+      <x:c r="X168" s="11" t="str">
+        <x:v>https://github.com/i-akiya/Shiranui</x:v>
+      </x:c>
+      <x:c r="Y168" s="11" t="str">
+        <x:v>https://github.com/i-akiya/Shiranui/blob/2d77554e4a33b065ab826a73580e9a7e2644296e/README.md | https://github.com/i-akiya/Shiranui/blob/2d77554e4a33b065ab826a73580e9a7e2644296e/pyproject.toml | https://github.com/i-akiya/Shiranui/blob/2d77554e4a33b065ab826a73580e9a7e2644296e/src/shiranui/server.py</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="169" ht="118.80000305175781" hidden="0" customHeight="1">
+      <x:c r="A169" s="11" t="str">
+        <x:v>RWE-0162</x:v>
+      </x:c>
+      <x:c r="B169" s="11" t="str">
+        <x:v>Claude Research Skills (drkamarul)</x:v>
+      </x:c>
+      <x:c r="C169" s="11" t="str">
+        <x:v>Agent skill collection</x:v>
+      </x:c>
+      <x:c r="D169" s="11" t="str">
+        <x:v>Causal Inference &amp; Analytics</x:v>
+      </x:c>
+      <x:c r="E169" s="11" t="str">
+        <x:v>Research skill collection covering data preparation, R modeling and medical-research workflows.</x:v>
+      </x:c>
+      <x:c r="F169" s="11" t="str">
+        <x:v>Causal Inference | Agent skill collection</x:v>
+      </x:c>
+      <x:c r="G169" s="11" t="str">
+        <x:v>Causal Inference &amp; Analytics | Source inspection and research preparation</x:v>
+      </x:c>
+      <x:c r="H169" s="11" t="str">
+        <x:v>Guide mixed-model analyses and data wrangling | Support medical-research, Quarto and spatial-analysis workflows</x:v>
+      </x:c>
+      <x:c r="I169" s="11" t="str">
+        <x:v>Some search guidance favors recent English open-access and highly cited work. Those selection rules require explicit protocol justification and can introduce bias.</x:v>
+      </x:c>
+      <x:c r="J169" s="11" t="str">
+        <x:v>Static source and documentation reviewed</x:v>
+      </x:c>
+      <x:c r="K169" s="11" t="str">
+        <x:v>Canonical repository metadata reviewed at commit 55daeb6d8fcbfe2c96d2806d7e0838cb3c3ebd46</x:v>
+      </x:c>
+      <x:c r="L169" s="11" t="str">
+        <x:v>https://github.com/drkamarul/claude-skills/blob/55daeb6d8fcbfe2c96d2806d7e0838cb3c3ebd46/datamanagement/SKILL.md | https://github.com/drkamarul/claude-skills/blob/55daeb6d8fcbfe2c96d2806d7e0838cb3c3ebd46/lmer-mixed-effects/SKILL.md | https://github.com/drkamarul/claude-skills/blob/55daeb6d8fcbfe2c96d2806d7e0838cb3c3ebd46/medical-research/SKILL.md</x:v>
+      </x:c>
+      <x:c r="M169" s="11" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N169" s="11" t="str">
+        <x:v>drkamarul</x:v>
+      </x:c>
+      <x:c r="O169" s="11" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P169" s="11" t="str">
+        <x:v>See pinned project manifest and setup documentation</x:v>
+      </x:c>
+      <x:c r="Q169" s="11" t="str">
+        <x:v>See pinned setup; varies by component</x:v>
+      </x:c>
+      <x:c r="R169" s="11" t="str">
+        <x:v>See capability and limitation fields; no runtime actions performed</x:v>
+      </x:c>
+      <x:c r="S169" s="11" t="str">
+        <x:v>See pinned project setup; external data access may require credentials.</x:v>
+      </x:c>
+      <x:c r="T169" s="14" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+      <x:c r="U169" s="14" t="n">
+        <x:v>46230.162083333336</x:v>
+      </x:c>
+      <x:c r="V169" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W169" s="11" t="str">
+        <x:v>https://github.com/drkamarul/claude-skills</x:v>
+      </x:c>
+      <x:c r="X169" s="11" t="str">
+        <x:v>https://github.com/drkamarul/claude-skills</x:v>
+      </x:c>
+      <x:c r="Y169" s="11" t="str">
+        <x:v>https://github.com/drkamarul/claude-skills/blob/55daeb6d8fcbfe2c96d2806d7e0838cb3c3ebd46/datamanagement/SKILL.md | https://github.com/drkamarul/claude-skills/blob/55daeb6d8fcbfe2c96d2806d7e0838cb3c3ebd46/lmer-mixed-effects/SKILL.md | https://github.com/drkamarul/claude-skills/blob/55daeb6d8fcbfe2c96d2806d7e0838cb3c3ebd46/medical-research/SKILL.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="170" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A170" s="11" t="str">
+        <x:v>RWE-0156</x:v>
+      </x:c>
+      <x:c r="B170" s="11" t="str">
+        <x:v>KFDA MCP</x:v>
+      </x:c>
+      <x:c r="C170" s="11" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D170" s="11" t="str">
+        <x:v>Regulatory &amp; Product Data</x:v>
+      </x:c>
+      <x:c r="E170" s="11" t="str">
+        <x:v>Retrieves Korean MFDS drug and related product information.</x:v>
+      </x:c>
+      <x:c r="F170" s="11" t="str">
+        <x:v>Regulatory | MCP server</x:v>
+      </x:c>
+      <x:c r="G170" s="11" t="str">
+        <x:v>Regulatory &amp; Product Data | Source inspection and research preparation</x:v>
+      </x:c>
+      <x:c r="H170" s="11" t="str">
+        <x:v>Search drug and patient-facing product information | Look up DUR information, supplements and built-in ATC mappings</x:v>
+      </x:c>
+      <x:c r="I170" s="11" t="str">
+        <x:v>Built-in mappings may be incomplete. Verify Korean source records and current restrictions; retrieval is not validated prescribing advice.</x:v>
+      </x:c>
+      <x:c r="J170" s="11" t="str">
+        <x:v>Static source and documentation reviewed</x:v>
+      </x:c>
+      <x:c r="K170" s="11" t="str">
+        <x:v>Canonical repository metadata reviewed at commit 3620ea4450217fcb9d88db6c394538da460103d3</x:v>
+      </x:c>
+      <x:c r="L170" s="11" t="str">
+        <x:v>https://github.com/pianovirus/kfda-mcp/blob/3620ea4450217fcb9d88db6c394538da460103d3/README.md | https://github.com/pianovirus/kfda-mcp/blob/3620ea4450217fcb9d88db6c394538da460103d3/pyproject.toml | https://github.com/pianovirus/kfda-mcp/blob/3620ea4450217fcb9d88db6c394538da460103d3/src/kfda_mcp/server.py</x:v>
+      </x:c>
+      <x:c r="M170" s="11" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N170" s="11" t="str">
+        <x:v>pianovirus</x:v>
+      </x:c>
+      <x:c r="O170" s="11" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P170" s="11" t="str">
+        <x:v>See pinned project manifest and setup documentation</x:v>
+      </x:c>
+      <x:c r="Q170" s="11" t="str">
+        <x:v>See pinned setup; varies by component</x:v>
+      </x:c>
+      <x:c r="R170" s="11" t="str">
+        <x:v>See capability and limitation fields; no runtime actions performed</x:v>
+      </x:c>
+      <x:c r="S170" s="11" t="str">
+        <x:v>Applicable Korean public-data API credentials; see project setup.</x:v>
+      </x:c>
+      <x:c r="T170" s="14" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+      <x:c r="U170" s="14" t="n">
+        <x:v>46203.380949074075</x:v>
+      </x:c>
+      <x:c r="V170" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W170" s="11" t="str">
+        <x:v>https://github.com/pianovirus/kfda-mcp</x:v>
+      </x:c>
+      <x:c r="X170" s="11" t="str">
+        <x:v>https://github.com/pianovirus/kfda-mcp</x:v>
+      </x:c>
+      <x:c r="Y170" s="11" t="str">
+        <x:v>https://github.com/pianovirus/kfda-mcp/blob/3620ea4450217fcb9d88db6c394538da460103d3/README.md | https://github.com/pianovirus/kfda-mcp/blob/3620ea4450217fcb9d88db6c394538da460103d3/pyproject.toml | https://github.com/pianovirus/kfda-mcp/blob/3620ea4450217fcb9d88db6c394538da460103d3/src/kfda_mcp/server.py</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="171" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A171" s="11" t="str">
+        <x:v>RWE-0142</x:v>
+      </x:c>
+      <x:c r="B171" s="11" t="str">
+        <x:v>NexVigilant Station</x:v>
+      </x:c>
+      <x:c r="C171" s="11" t="str">
+        <x:v>Hosted MCP service</x:v>
+      </x:c>
+      <x:c r="D171" s="11" t="str">
+        <x:v>Pharmacovigilance &amp; safety</x:v>
+      </x:c>
+      <x:c r="E171" s="11" t="str">
+        <x:v>Hosted service documenting pharmacovigilance source queries and signal-calculation tools.</x:v>
+      </x:c>
+      <x:c r="F171" s="11" t="str">
+        <x:v>Pharmacovigilance | Hosted MCP service</x:v>
+      </x:c>
+      <x:c r="G171" s="11" t="str">
+        <x:v>Pharmacovigilance &amp; safety | Source inspection and research preparation</x:v>
+      </x:c>
+      <x:c r="H171" s="11" t="str">
+        <x:v>Retrieve documented FAERS, labeling, trial and literature information | Expose documented disproportionality and case-assessment functions</x:v>
+      </x:c>
+      <x:c r="I171" s="11" t="str">
+        <x:v>Documentation-only review: backend implementation and live tool inventory were not inspected. Signal and causality scores need independent validation. Source-available license requires permission for organizational use.</x:v>
+      </x:c>
+      <x:c r="J171" s="11" t="str">
+        <x:v>Static documentation reviewed; hosted implementation not inspected</x:v>
+      </x:c>
+      <x:c r="K171" s="11" t="str">
+        <x:v>Canonical repository metadata reviewed at commit 28dddb074c7aa5177cac43d88d09bfefa5a2ec48</x:v>
+      </x:c>
+      <x:c r="L171" s="11" t="str">
+        <x:v>https://github.com/nexvigilant/nexvigilant-station/blob/28dddb074c7aa5177cac43d88d09bfefa5a2ec48/README.md</x:v>
+      </x:c>
+      <x:c r="M171" s="11" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N171" s="11" t="str">
+        <x:v>nexvigilant</x:v>
+      </x:c>
+      <x:c r="O171" s="11" t="str">
+        <x:v>NOASSERTION</x:v>
+      </x:c>
+      <x:c r="P171" s="11" t="str">
+        <x:v>See pinned project manifest and setup documentation</x:v>
+      </x:c>
+      <x:c r="Q171" s="11" t="str">
+        <x:v>See pinned setup; varies by component</x:v>
+      </x:c>
+      <x:c r="R171" s="11" t="str">
+        <x:v>See capability and limitation fields; no runtime actions performed</x:v>
+      </x:c>
+      <x:c r="S171" s="11" t="str">
+        <x:v>Publisher documents an unauthenticated Streamable HTTP endpoint; organizational license permission required.</x:v>
+      </x:c>
+      <x:c r="T171" s="14" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+      <x:c r="U171" s="14" t="n">
+        <x:v>46105.068194444444</x:v>
+      </x:c>
+      <x:c r="V171" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W171" s="11" t="str">
+        <x:v>https://github.com/nexvigilant/nexvigilant-station</x:v>
+      </x:c>
+      <x:c r="X171" s="11" t="str">
+        <x:v>https://github.com/nexvigilant/nexvigilant-station</x:v>
+      </x:c>
+      <x:c r="Y171" s="11" t="str">
+        <x:v>https://github.com/nexvigilant/nexvigilant-station/blob/28dddb074c7aa5177cac43d88d09bfefa5a2ec48/README.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="172" ht="198" hidden="0" customHeight="1">
+      <x:c r="A172" s="11" t="str">
+        <x:v>RWE-0127</x:v>
+      </x:c>
+      <x:c r="B172" s="11" t="str">
+        <x:v>Research KB</x:v>
+      </x:c>
+      <x:c r="C172" s="11" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D172" s="11" t="str">
+        <x:v>Literature &amp; Evidence Synthesis</x:v>
+      </x:c>
+      <x:c r="E172" s="11" t="str">
+        <x:v>Local research knowledge base with hybrid retrieval and assumption-oriented evidence inspection.</x:v>
+      </x:c>
+      <x:c r="F172" s="11" t="str">
+        <x:v>Literature | MCP server</x:v>
+      </x:c>
+      <x:c r="G172" s="11" t="str">
+        <x:v>Literature &amp; Evidence Synthesis | Source inspection and research preparation</x:v>
+      </x:c>
+      <x:c r="H172" s="11" t="str">
+        <x:v>Search a supplied corpus using lexical and embedding retrieval | Inspect citations and extracted methodological assumptions</x:v>
+      </x:c>
+      <x:c r="I172" s="11" t="str">
+        <x:v>Corpus access and licenses are separate from the code. Graph functionality is documented as disabled pending rebuild; extracted assumptions are not proof of causal identification.</x:v>
+      </x:c>
+      <x:c r="J172" s="11" t="str">
+        <x:v>Static source and documentation reviewed</x:v>
+      </x:c>
+      <x:c r="K172" s="11" t="str">
+        <x:v>Canonical repository metadata reviewed at commit bb567b9c892b40d9f2f6c576a1036ec8ac2d1e26</x:v>
+      </x:c>
+      <x:c r="L172" s="11" t="str">
+        <x:v>https://github.com/brandonmbehring-dev/research-kb/blob/bb567b9c892b40d9f2f6c576a1036ec8ac2d1e26/README.md | https://github.com/brandonmbehring-dev/research-kb/blob/bb567b9c892b40d9f2f6c576a1036ec8ac2d1e26/pyproject.toml | https://github.com/brandonmbehring-dev/research-kb/blob/bb567b9c892b40d9f2f6c576a1036ec8ac2d1e26/packages/daemon/src/research_kb_daemon/server.py | https://github.com/brandonmbehring-dev/research-kb/blob/bb567b9c892b40d9f2f6c576a1036ec8ac2d1e26/packages/mcp-server/src/research_kb_mcp/server.py | https://github.com/brandonmbehring-dev/research-kb/blob/bb567b9c892b40d9f2f6c576a1036ec8ac2d1e26/skills/assumption-tracking/SKILL.md</x:v>
+      </x:c>
+      <x:c r="M172" s="11" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N172" s="11" t="str">
+        <x:v>brandonmbehring-dev</x:v>
+      </x:c>
+      <x:c r="O172" s="11" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P172" s="11" t="str">
+        <x:v>See pinned project manifest and setup documentation</x:v>
+      </x:c>
+      <x:c r="Q172" s="11" t="str">
+        <x:v>See pinned setup; varies by component</x:v>
+      </x:c>
+      <x:c r="R172" s="11" t="str">
+        <x:v>See capability and limitation fields; no runtime actions performed</x:v>
+      </x:c>
+      <x:c r="S172" s="11" t="str">
+        <x:v>See pinned project setup; external data access may require credentials.</x:v>
+      </x:c>
+      <x:c r="T172" s="14" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+      <x:c r="U172" s="14" t="n">
+        <x:v>46265.543125</x:v>
+      </x:c>
+      <x:c r="V172" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W172" s="11" t="str">
+        <x:v>https://github.com/brandonmbehring-dev/research-kb</x:v>
+      </x:c>
+      <x:c r="X172" s="11" t="str">
+        <x:v>https://github.com/brandonmbehring-dev/research-kb</x:v>
+      </x:c>
+      <x:c r="Y172" s="11" t="str">
+        <x:v>https://github.com/brandonmbehring-dev/research-kb/blob/bb567b9c892b40d9f2f6c576a1036ec8ac2d1e26/README.md | https://github.com/brandonmbehring-dev/research-kb/blob/bb567b9c892b40d9f2f6c576a1036ec8ac2d1e26/pyproject.toml | https://github.com/brandonmbehring-dev/research-kb/blob/bb567b9c892b40d9f2f6c576a1036ec8ac2d1e26/packages/daemon/src/research_kb_daemon/server.py | https://github.com/brandonmbehring-dev/research-kb/blob/bb567b9c892b40d9f2f6c576a1036ec8ac2d1e26/packages/mcp-server/src/research_kb_mcp/server.py | https://github.com/brandonmbehring-dev/research-kb/blob/bb567b9c892b40d9f2f6c576a1036ec8ac2d1e26/skills/assumption-tracking/SKILL.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="173" ht="105.5999984741211" hidden="0" customHeight="1">
+      <x:c r="A173" s="11" t="str">
+        <x:v>RWE-0259</x:v>
+      </x:c>
+      <x:c r="B173" s="11" t="str">
+        <x:v>fhirHydrant</x:v>
+      </x:c>
+      <x:c r="C173" s="11" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D173" s="11" t="str">
+        <x:v>Clinical Data &amp; Interoperability</x:v>
+      </x:c>
+      <x:c r="E173" s="11" t="str">
+        <x:v>FHIR R4+ connector with resource inspection, terminology and optional write workflows.</x:v>
+      </x:c>
+      <x:c r="F173" s="11" t="str">
+        <x:v>Clinical Data | MCP server</x:v>
+      </x:c>
+      <x:c r="G173" s="11" t="str">
+        <x:v>Clinical Data &amp; Interoperability | Source inspection and research preparation</x:v>
+      </x:c>
+      <x:c r="H173" s="11" t="str">
+        <x:v>Read resources and history; use supported terminology operations | Expose explicitly enabled CRUD and bundle transactions</x:v>
+      </x:c>
+      <x:c r="I173" s="11" t="str">
+        <x:v>Write tools require deliberate gating. Validate FHIR profiles, authorization and patient-data governance; resource connectivity does not establish research completeness.</x:v>
+      </x:c>
+      <x:c r="J173" s="11" t="str">
+        <x:v>Static source and documentation reviewed</x:v>
+      </x:c>
+      <x:c r="K173" s="11" t="str">
+        <x:v>Canonical repository metadata reviewed at commit caba5aa0cc782c71f9ebe78bd79cfdcfee6fa221</x:v>
+      </x:c>
+      <x:c r="L173" s="11" t="str">
+        <x:v>https://github.com/faulkj/fhirHydrant/blob/caba5aa0cc782c71f9ebe78bd79cfdcfee6fa221/README.md | https://github.com/faulkj/fhirHydrant/blob/caba5aa0cc782c71f9ebe78bd79cfdcfee6fa221/package.json | https://github.com/faulkj/fhirHydrant/blob/caba5aa0cc782c71f9ebe78bd79cfdcfee6fa221/server.json | https://github.com/faulkj/fhirHydrant/blob/caba5aa0cc782c71f9ebe78bd79cfdcfee6fa221/ts/server.ts</x:v>
+      </x:c>
+      <x:c r="M173" s="11" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N173" s="11" t="str">
+        <x:v>faulkj</x:v>
+      </x:c>
+      <x:c r="O173" s="11" t="str">
+        <x:v>NOASSERTION</x:v>
+      </x:c>
+      <x:c r="P173" s="11" t="str">
+        <x:v>See pinned project manifest and setup documentation</x:v>
+      </x:c>
+      <x:c r="Q173" s="11" t="str">
+        <x:v>See pinned setup; varies by component</x:v>
+      </x:c>
+      <x:c r="R173" s="11" t="str">
+        <x:v>See capability and limitation fields; no runtime actions performed</x:v>
+      </x:c>
+      <x:c r="S173" s="11" t="str">
+        <x:v>Configured FHIR endpoint; optional SMART Backend Services JWT authentication.</x:v>
+      </x:c>
+      <x:c r="T173" s="14" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+      <x:c r="U173" s="14" t="n">
+        <x:v>46261.97315972222</x:v>
+      </x:c>
+      <x:c r="V173" s="11" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="W173" s="11" t="str">
+        <x:v>https://github.com/faulkj/fhirHydrant</x:v>
+      </x:c>
+      <x:c r="X173" s="11" t="str">
+        <x:v>https://github.com/faulkj/fhirHydrant</x:v>
+      </x:c>
+      <x:c r="Y173" s="11" t="str">
+        <x:v>https://github.com/faulkj/fhirHydrant/blob/caba5aa0cc782c71f9ebe78bd79cfdcfee6fa221/README.md | https://github.com/faulkj/fhirHydrant/blob/caba5aa0cc782c71f9ebe78bd79cfdcfee6fa221/package.json | https://github.com/faulkj/fhirHydrant/blob/caba5aa0cc782c71f9ebe78bd79cfdcfee6fa221/server.json | https://github.com/faulkj/fhirHydrant/blob/caba5aa0cc782c71f9ebe78bd79cfdcfee6fa221/ts/server.ts</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="174" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A174" s="11" t="str">
+        <x:v>RWE-0260</x:v>
+      </x:c>
+      <x:c r="B174" s="11" t="str">
+        <x:v>prismAId</x:v>
+      </x:c>
+      <x:c r="C174" s="11" t="str">
+        <x:v>Library + MCP server</x:v>
+      </x:c>
+      <x:c r="D174" s="11" t="str">
+        <x:v>Literature &amp; Evidence Synthesis</x:v>
+      </x:c>
+      <x:c r="E174" s="11" t="str">
+        <x:v>Library and MCP tools for literature-search, screening and evidence-review workflows.</x:v>
+      </x:c>
+      <x:c r="F174" s="11" t="str">
+        <x:v>Literature | Library + MCP server</x:v>
+      </x:c>
+      <x:c r="G174" s="11" t="str">
+        <x:v>Literature &amp; Evidence Synthesis | Source inspection and research preparation</x:v>
+      </x:c>
+      <x:c r="H174" s="11" t="str">
+        <x:v>Search, screen, retrieve and convert literature | Support structured review and reporting-conformance checks</x:v>
+      </x:c>
+      <x:c r="I174" s="11" t="str">
+        <x:v>LLM screening and extraction require human checking. Reporting or SHACL conformance does not establish review completeness or methodological validity.</x:v>
+      </x:c>
+      <x:c r="J174" s="11" t="str">
+        <x:v>Static source and documentation reviewed</x:v>
+      </x:c>
+      <x:c r="K174" s="11" t="str">
+        <x:v>Canonical repository metadata reviewed at commit 9457f7cfd2043f14a6d88019787692fdf2e1a985</x:v>
+      </x:c>
+      <x:c r="L174" s="11" t="str">
+        <x:v>https://github.com/open-and-sustainable/prismaid/blob/9457f7cfd2043f14a6d88019787692fdf2e1a985/README.md | https://github.com/open-and-sustainable/prismaid/blob/9457f7cfd2043f14a6d88019787692fdf2e1a985/server.json</x:v>
+      </x:c>
+      <x:c r="M174" s="11" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N174" s="11" t="str">
+        <x:v>open-and-sustainable</x:v>
+      </x:c>
+      <x:c r="O174" s="11" t="str">
+        <x:v>AGPL-3.0</x:v>
+      </x:c>
+      <x:c r="P174" s="11" t="str">
+        <x:v>See pinned project manifest and setup documentation</x:v>
+      </x:c>
+      <x:c r="Q174" s="11" t="str">
+        <x:v>See pinned setup; varies by component</x:v>
+      </x:c>
+      <x:c r="R174" s="11" t="str">
+        <x:v>See capability and limitation fields; no runtime actions performed</x:v>
+      </x:c>
+      <x:c r="S174" s="11" t="str">
+        <x:v>See pinned project setup; external data access may require credentials.</x:v>
+      </x:c>
+      <x:c r="T174" s="14" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+      <x:c r="U174" s="14" t="n">
+        <x:v>46254.44039351852</x:v>
+      </x:c>
+      <x:c r="V174" s="11" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="W174" s="11" t="str">
+        <x:v>https://github.com/open-and-sustainable/prismaid</x:v>
+      </x:c>
+      <x:c r="X174" s="11" t="str">
+        <x:v>https://github.com/open-and-sustainable/prismaid</x:v>
+      </x:c>
+      <x:c r="Y174" s="11" t="str">
+        <x:v>https://github.com/open-and-sustainable/prismaid/blob/9457f7cfd2043f14a6d88019787692fdf2e1a985/README.md | https://github.com/open-and-sustainable/prismaid/blob/9457f7cfd2043f14a6d88019787692fdf2e1a985/server.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="175" ht="105.5999984741211" hidden="0" customHeight="1">
+      <x:c r="A175" s="11" t="str">
+        <x:v>RWE-0261</x:v>
+      </x:c>
+      <x:c r="B175" s="11" t="str">
+        <x:v>Biolab MCP Server</x:v>
+      </x:c>
+      <x:c r="C175" s="11" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D175" s="11" t="str">
+        <x:v>Literature &amp; Evidence Synthesis</x:v>
+      </x:c>
+      <x:c r="E175" s="11" t="str">
+        <x:v>Literature and trial retrieval tools with source identifiers and query-audit records.</x:v>
+      </x:c>
+      <x:c r="F175" s="11" t="str">
+        <x:v>Literature | MCP server</x:v>
+      </x:c>
+      <x:c r="G175" s="11" t="str">
+        <x:v>Literature &amp; Evidence Synthesis | Source inspection and research preparation</x:v>
+      </x:c>
+      <x:c r="H175" s="11" t="str">
+        <x:v>Search PubMed, Europe PMC, ClinicalTrials.gov and preprint sources | Retrieve source records and maintain query provenance</x:v>
+      </x:c>
+      <x:c r="I175" s="11" t="str">
+        <x:v>An audit trail records actions rather than validating evidence synthesis. Check source coverage, retention and the sensitivity of externally transmitted queries.</x:v>
+      </x:c>
+      <x:c r="J175" s="11" t="str">
+        <x:v>Static source and documentation reviewed</x:v>
+      </x:c>
+      <x:c r="K175" s="11" t="str">
+        <x:v>Canonical repository metadata reviewed at commit 0bfb24074b7480c0455f5c117b274bc83e815f44</x:v>
+      </x:c>
+      <x:c r="L175" s="11" t="str">
+        <x:v>https://github.com/srikarjy/biolab-mcp-server/blob/0bfb24074b7480c0455f5c117b274bc83e815f44/README.md | https://github.com/srikarjy/biolab-mcp-server/blob/0bfb24074b7480c0455f5c117b274bc83e815f44/pyproject.toml | https://github.com/srikarjy/biolab-mcp-server/blob/0bfb24074b7480c0455f5c117b274bc83e815f44/server.json | https://github.com/srikarjy/biolab-mcp-server/blob/0bfb24074b7480c0455f5c117b274bc83e815f44/biolab/server.py</x:v>
+      </x:c>
+      <x:c r="M175" s="11" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N175" s="11" t="str">
+        <x:v>srikarjy</x:v>
+      </x:c>
+      <x:c r="O175" s="11" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P175" s="11" t="str">
+        <x:v>See pinned project manifest and setup documentation</x:v>
+      </x:c>
+      <x:c r="Q175" s="11" t="str">
+        <x:v>See pinned setup; varies by component</x:v>
+      </x:c>
+      <x:c r="R175" s="11" t="str">
+        <x:v>See capability and limitation fields; no runtime actions performed</x:v>
+      </x:c>
+      <x:c r="S175" s="11" t="str">
+        <x:v>See pinned project setup; external data access may require credentials.</x:v>
+      </x:c>
+      <x:c r="T175" s="14" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+      <x:c r="U175" s="14" t="n">
+        <x:v>46249.36493055556</x:v>
+      </x:c>
+      <x:c r="V175" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="W175" s="11" t="str">
+        <x:v>https://github.com/srikarjy/biolab-mcp-server</x:v>
+      </x:c>
+      <x:c r="X175" s="11" t="str">
+        <x:v>https://github.com/srikarjy/biolab-mcp-server</x:v>
+      </x:c>
+      <x:c r="Y175" s="11" t="str">
+        <x:v>https://github.com/srikarjy/biolab-mcp-server/blob/0bfb24074b7480c0455f5c117b274bc83e815f44/README.md | https://github.com/srikarjy/biolab-mcp-server/blob/0bfb24074b7480c0455f5c117b274bc83e815f44/pyproject.toml | https://github.com/srikarjy/biolab-mcp-server/blob/0bfb24074b7480c0455f5c117b274bc83e815f44/server.json | https://github.com/srikarjy/biolab-mcp-server/blob/0bfb24074b7480c0455f5c117b274bc83e815f44/biolab/server.py</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="176" ht="171.60000610351562" hidden="0" customHeight="1">
+      <x:c r="A176" s="11" t="str">
+        <x:v>RWE-0262</x:v>
+      </x:c>
+      <x:c r="B176" s="11" t="str">
+        <x:v>OHDSI StudyAgent</x:v>
+      </x:c>
+      <x:c r="C176" s="11" t="str">
+        <x:v>Agent harness + MCP components</x:v>
+      </x:c>
+      <x:c r="D176" s="11" t="str">
+        <x:v>Trials &amp; Study Design</x:v>
+      </x:c>
+      <x:c r="E176" s="11" t="str">
+        <x:v>Study-design agent harness with deterministic MCP components for OHDSI workflows.</x:v>
+      </x:c>
+      <x:c r="F176" s="11" t="str">
+        <x:v>Trials | Agent harness + MCP components</x:v>
+      </x:c>
+      <x:c r="G176" s="11" t="str">
+        <x:v>Trials &amp; Study Design | Source inspection and research preparation</x:v>
+      </x:c>
+      <x:c r="H176" s="11" t="str">
+        <x:v>Assist vocabulary, concept-set and phenotype work | Coordinate study-intent and validation steps through an agent workflow</x:v>
+      </x:c>
+      <x:c r="I176" s="11" t="str">
+        <x:v>Human review remains necessary for study intent and methods. Schema or tool validation does not validate identification assumptions; database execution requires governed access.</x:v>
+      </x:c>
+      <x:c r="J176" s="11" t="str">
+        <x:v>Static source and documentation reviewed</x:v>
+      </x:c>
+      <x:c r="K176" s="11" t="str">
+        <x:v>Canonical repository metadata reviewed at commit 489aabd9ab7141fa322a2d13d4212b2477c15903</x:v>
+      </x:c>
+      <x:c r="L176" s="11" t="str">
+        <x:v>https://github.com/OHDSI/StudyAgent/blob/489aabd9ab7141fa322a2d13d4212b2477c15903/README.md | https://github.com/OHDSI/StudyAgent/blob/489aabd9ab7141fa322a2d13d4212b2477c15903/pyproject.toml | https://github.com/OHDSI/StudyAgent/blob/489aabd9ab7141fa322a2d13d4212b2477c15903/acp_agent/study_agent_acp/server.py | https://github.com/OHDSI/StudyAgent/blob/489aabd9ab7141fa322a2d13d4212b2477c15903/core/study_agent_core/tools.py | https://github.com/OHDSI/StudyAgent/blob/489aabd9ab7141fa322a2d13d4212b2477c15903/mcp_server/study_agent_mcp/server.py</x:v>
+      </x:c>
+      <x:c r="M176" s="11" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N176" s="11" t="str">
+        <x:v>OHDSI</x:v>
+      </x:c>
+      <x:c r="O176" s="11" t="str">
+        <x:v>Not specified</x:v>
+      </x:c>
+      <x:c r="P176" s="11" t="str">
+        <x:v>See pinned project manifest and setup documentation</x:v>
+      </x:c>
+      <x:c r="Q176" s="11" t="str">
+        <x:v>See pinned setup; varies by component</x:v>
+      </x:c>
+      <x:c r="R176" s="11" t="str">
+        <x:v>See capability and limitation fields; no runtime actions performed</x:v>
+      </x:c>
+      <x:c r="S176" s="11" t="str">
+        <x:v>See pinned project setup; external data access may require credentials.</x:v>
+      </x:c>
+      <x:c r="T176" s="14" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+      <x:c r="U176" s="14" t="n">
+        <x:v>46270.67685185185</x:v>
+      </x:c>
+      <x:c r="V176" s="11" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="W176" s="11" t="str">
+        <x:v>https://github.com/OHDSI/StudyAgent</x:v>
+      </x:c>
+      <x:c r="X176" s="11" t="str">
+        <x:v>https://github.com/OHDSI/StudyAgent</x:v>
+      </x:c>
+      <x:c r="Y176" s="11" t="str">
+        <x:v>https://github.com/OHDSI/StudyAgent/blob/489aabd9ab7141fa322a2d13d4212b2477c15903/README.md | https://github.com/OHDSI/StudyAgent/blob/489aabd9ab7141fa322a2d13d4212b2477c15903/pyproject.toml | https://github.com/OHDSI/StudyAgent/blob/489aabd9ab7141fa322a2d13d4212b2477c15903/acp_agent/study_agent_acp/server.py | https://github.com/OHDSI/StudyAgent/blob/489aabd9ab7141fa322a2d13d4212b2477c15903/core/study_agent_core/tools.py | https://github.com/OHDSI/StudyAgent/blob/489aabd9ab7141fa322a2d13d4212b2477c15903/mcp_server/study_agent_mcp/server.py</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="177" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A177" s="11" t="str">
+        <x:v>RWE-0263</x:v>
+      </x:c>
+      <x:c r="B177" s="11" t="str">
+        <x:v>Slash OHDSI Strategus Assistant</x:v>
+      </x:c>
+      <x:c r="C177" s="11" t="str">
+        <x:v>R package + agent integration</x:v>
+      </x:c>
+      <x:c r="D177" s="11" t="str">
+        <x:v>Trials &amp; Study Design</x:v>
+      </x:c>
+      <x:c r="E177" s="11" t="str">
+        <x:v>R and agent integration for constructing and running OHDSI Strategus analyses.</x:v>
+      </x:c>
+      <x:c r="F177" s="11" t="str">
+        <x:v>Trials | R package + agent integration</x:v>
+      </x:c>
+      <x:c r="G177" s="11" t="str">
+        <x:v>Trials &amp; Study Design | Source inspection and research preparation</x:v>
+      </x:c>
+      <x:c r="H177" s="11" t="str">
+        <x:v>Guide incidence and CohortMethod analysis workflows | Support phenotype acquisition, checkpoints and resumable study execution</x:v>
+      </x:c>
+      <x:c r="I177" s="11" t="str">
+        <x:v>Not a standalone MCP server. Requires an appropriate OHDSI environment and review of cohort definitions, database permissions and statistical design.</x:v>
+      </x:c>
+      <x:c r="J177" s="11" t="str">
+        <x:v>Static source and documentation reviewed</x:v>
+      </x:c>
+      <x:c r="K177" s="11" t="str">
+        <x:v>Canonical repository metadata reviewed at commit 84d16bef6b7bb08810820ddf2da79f3022e33497</x:v>
+      </x:c>
+      <x:c r="L177" s="11" t="str">
+        <x:v>https://github.com/OHDSI/SlashOhdsiStrategusAssistant/blob/84d16bef6b7bb08810820ddf2da79f3022e33497/DESCRIPTION | https://github.com/OHDSI/SlashOhdsiStrategusAssistant/blob/84d16bef6b7bb08810820ddf2da79f3022e33497/README.md</x:v>
+      </x:c>
+      <x:c r="M177" s="11" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N177" s="11" t="str">
+        <x:v>OHDSI</x:v>
+      </x:c>
+      <x:c r="O177" s="11" t="str">
+        <x:v>Not specified</x:v>
+      </x:c>
+      <x:c r="P177" s="11" t="str">
+        <x:v>See pinned project manifest and setup documentation</x:v>
+      </x:c>
+      <x:c r="Q177" s="11" t="str">
+        <x:v>See pinned setup; varies by component</x:v>
+      </x:c>
+      <x:c r="R177" s="11" t="str">
+        <x:v>See capability and limitation fields; no runtime actions performed</x:v>
+      </x:c>
+      <x:c r="S177" s="11" t="str">
+        <x:v>See pinned project setup; external data access may require credentials.</x:v>
+      </x:c>
+      <x:c r="T177" s="14" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+      <x:c r="U177" s="14" t="n">
+        <x:v>46270.67748842593</x:v>
+      </x:c>
+      <x:c r="V177" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="W177" s="11" t="str">
+        <x:v>https://github.com/OHDSI/SlashOhdsiStrategusAssistant</x:v>
+      </x:c>
+      <x:c r="X177" s="11" t="str">
+        <x:v>https://github.com/OHDSI/SlashOhdsiStrategusAssistant</x:v>
+      </x:c>
+      <x:c r="Y177" s="11" t="str">
+        <x:v>https://github.com/OHDSI/SlashOhdsiStrategusAssistant/blob/84d16bef6b7bb08810820ddf2da79f3022e33497/DESCRIPTION | https://github.com/OHDSI/SlashOhdsiStrategusAssistant/blob/84d16bef6b7bb08810820ddf2da79f3022e33497/README.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="178" ht="118.80000305175781" hidden="0" customHeight="1">
+      <x:c r="A178" s="11" t="str">
+        <x:v>RWE-0264</x:v>
+      </x:c>
+      <x:c r="B178" s="11" t="str">
+        <x:v>Biomedical Terminology Service</x:v>
+      </x:c>
+      <x:c r="C178" s="11" t="str">
+        <x:v>Terminology service + MCP interface</x:v>
+      </x:c>
+      <x:c r="D178" s="11" t="str">
+        <x:v>OMOP &amp; terminology</x:v>
+      </x:c>
+      <x:c r="E178" s="11" t="str">
+        <x:v>Self-hosted terminology service with REST, GraphQL, FHIR and MCP interfaces.</x:v>
+      </x:c>
+      <x:c r="F178" s="11" t="str">
+        <x:v>OMOP | Terminology service + MCP interface</x:v>
+      </x:c>
+      <x:c r="G178" s="11" t="str">
+        <x:v>OMOP &amp; terminology | Source inspection and research preparation</x:v>
+      </x:c>
+      <x:c r="H178" s="11" t="str">
+        <x:v>Search terminology concepts and mappings | Expose semantic terminology access through multiple interfaces</x:v>
+      </x:c>
+      <x:c r="I178" s="11" t="str">
+        <x:v>Vocabulary datasets and licenses are separate from server code. Check versions, mapping relationships and local indexing before using concepts in phenotypes.</x:v>
+      </x:c>
+      <x:c r="J178" s="11" t="str">
+        <x:v>Static source and documentation reviewed</x:v>
+      </x:c>
+      <x:c r="K178" s="11" t="str">
+        <x:v>Canonical repository metadata reviewed at commit 951933b574cb90f745108ba8a58bc73fd9ef944f</x:v>
+      </x:c>
+      <x:c r="L178" s="11" t="str">
+        <x:v>https://github.com/Firefox2100/biomedical-terminology-service/blob/951933b574cb90f745108ba8a58bc73fd9ef944f/README.md | https://github.com/Firefox2100/biomedical-terminology-service/blob/951933b574cb90f745108ba8a58bc73fd9ef944f/pyproject.toml | https://github.com/Firefox2100/biomedical-terminology-service/blob/951933b574cb90f745108ba8a58bc73fd9ef944f/src/bioterms/mcp_api/tool.py</x:v>
+      </x:c>
+      <x:c r="M178" s="11" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N178" s="11" t="str">
+        <x:v>Firefox2100</x:v>
+      </x:c>
+      <x:c r="O178" s="11" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P178" s="11" t="str">
+        <x:v>See pinned project manifest and setup documentation</x:v>
+      </x:c>
+      <x:c r="Q178" s="11" t="str">
+        <x:v>See pinned setup; varies by component</x:v>
+      </x:c>
+      <x:c r="R178" s="11" t="str">
+        <x:v>See capability and limitation fields; no runtime actions performed</x:v>
+      </x:c>
+      <x:c r="S178" s="11" t="str">
+        <x:v>See pinned project setup; external data access may require credentials.</x:v>
+      </x:c>
+      <x:c r="T178" s="14" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+      <x:c r="U178" s="14" t="n">
+        <x:v>46262.526030092595</x:v>
+      </x:c>
+      <x:c r="V178" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W178" s="11" t="str">
+        <x:v>https://github.com/Firefox2100/biomedical-terminology-service</x:v>
+      </x:c>
+      <x:c r="X178" s="11" t="str">
+        <x:v>https://github.com/Firefox2100/biomedical-terminology-service</x:v>
+      </x:c>
+      <x:c r="Y178" s="11" t="str">
+        <x:v>https://github.com/Firefox2100/biomedical-terminology-service/blob/951933b574cb90f745108ba8a58bc73fd9ef944f/README.md | https://github.com/Firefox2100/biomedical-terminology-service/blob/951933b574cb90f745108ba8a58bc73fd9ef944f/pyproject.toml | https://github.com/Firefox2100/biomedical-terminology-service/blob/951933b574cb90f745108ba8a58bc73fd9ef944f/src/bioterms/mcp_api/tool.py</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="179" ht="198" hidden="0" customHeight="1">
+      <x:c r="A179" s="11" t="str">
+        <x:v>RWE-0265</x:v>
+      </x:c>
+      <x:c r="B179" s="11" t="str">
+        <x:v>LangCare MCP FHIR</x:v>
+      </x:c>
+      <x:c r="C179" s="11" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D179" s="11" t="str">
+        <x:v>Clinical Data &amp; Interoperability</x:v>
+      </x:c>
+      <x:c r="E179" s="11" t="str">
+        <x:v>Go MCP connector exposing generic FHIR operations across configured backends.</x:v>
+      </x:c>
+      <x:c r="F179" s="11" t="str">
+        <x:v>Clinical Data | MCP server</x:v>
+      </x:c>
+      <x:c r="G179" s="11" t="str">
+        <x:v>Clinical Data &amp; Interoperability | Source inspection and research preparation</x:v>
+      </x:c>
+      <x:c r="H179" s="11" t="str">
+        <x:v>Read and search FHIR resources | Create and update resources through supported backend adapters</x:v>
+      </x:c>
+      <x:c r="I179" s="11" t="str">
+        <x:v>Contains write operations. Endpoint compatibility, patient authorization and privacy controls must be configured and verified; no compliance certification is implied.</x:v>
+      </x:c>
+      <x:c r="J179" s="11" t="str">
+        <x:v>Static source and documentation reviewed</x:v>
+      </x:c>
+      <x:c r="K179" s="11" t="str">
+        <x:v>Canonical repository metadata reviewed at commit 430598bb5a76619ef55fa34fb1fd90c65f3d4783</x:v>
+      </x:c>
+      <x:c r="L179" s="11" t="str">
+        <x:v>https://github.com/mosaic-care/langcare-mcp-fhir/blob/430598bb5a76619ef55fa34fb1fd90c65f3d4783/README.md | https://github.com/mosaic-care/langcare-mcp-fhir/blob/430598bb5a76619ef55fa34fb1fd90c65f3d4783/package.json | https://github.com/mosaic-care/langcare-mcp-fhir/blob/430598bb5a76619ef55fa34fb1fd90c65f3d4783/server.json | https://github.com/mosaic-care/langcare-mcp-fhir/blob/430598bb5a76619ef55fa34fb1fd90c65f3d4783/cma/skills/care-coordination/care-gaps/SKILL.md | https://github.com/mosaic-care/langcare-mcp-fhir/blob/430598bb5a76619ef55fa34fb1fd90c65f3d4783/cma/skills/care-coordination/discharge-planning/SKILL.md | https://github.com/mosaic-care/langcare-mcp-fhir/blob/430598bb5a76619ef55fa34fb1fd90c65f3d4783/cma/skills/care-coordination/follow-up-tasks/SKILL.md</x:v>
+      </x:c>
+      <x:c r="M179" s="11" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N179" s="11" t="str">
+        <x:v>mosaic-care</x:v>
+      </x:c>
+      <x:c r="O179" s="11" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P179" s="11" t="str">
+        <x:v>See pinned project manifest and setup documentation</x:v>
+      </x:c>
+      <x:c r="Q179" s="11" t="str">
+        <x:v>See pinned setup; varies by component</x:v>
+      </x:c>
+      <x:c r="R179" s="11" t="str">
+        <x:v>See capability and limitation fields; no runtime actions performed</x:v>
+      </x:c>
+      <x:c r="S179" s="11" t="str">
+        <x:v>Configured GCP, Epic, Cerner or other supported FHIR backend; applicable SMART credentials.</x:v>
+      </x:c>
+      <x:c r="T179" s="14" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+      <x:c r="U179" s="14" t="n">
+        <x:v>46271.80769675926</x:v>
+      </x:c>
+      <x:c r="V179" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W179" s="11" t="str">
+        <x:v>https://github.com/mosaic-care/langcare-mcp-fhir</x:v>
+      </x:c>
+      <x:c r="X179" s="11" t="str">
+        <x:v>https://github.com/mosaic-care/langcare-mcp-fhir</x:v>
+      </x:c>
+      <x:c r="Y179" s="11" t="str">
+        <x:v>https://github.com/mosaic-care/langcare-mcp-fhir/blob/430598bb5a76619ef55fa34fb1fd90c65f3d4783/README.md | https://github.com/mosaic-care/langcare-mcp-fhir/blob/430598bb5a76619ef55fa34fb1fd90c65f3d4783/package.json | https://github.com/mosaic-care/langcare-mcp-fhir/blob/430598bb5a76619ef55fa34fb1fd90c65f3d4783/server.json | https://github.com/mosaic-care/langcare-mcp-fhir/blob/430598bb5a76619ef55fa34fb1fd90c65f3d4783/cma/skills/care-coordination/care-gaps/SKILL.md | https://github.com/mosaic-care/langcare-mcp-fhir/blob/430598bb5a76619ef55fa34fb1fd90c65f3d4783/cma/skills/care-coordination/discharge-planning/SKILL.md | https://github.com/mosaic-care/langcare-mcp-fhir/blob/430598bb5a76619ef55fa34fb1fd90c65f3d4783/cma/skills/care-coordination/follow-up-tasks/SKILL.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="180" ht="171.60000610351562" hidden="0" customHeight="1">
+      <x:c r="A180" s="11" t="str">
+        <x:v>RWE-0266</x:v>
+      </x:c>
+      <x:c r="B180" s="11" t="str">
+        <x:v>M4 Clinical Research</x:v>
+      </x:c>
+      <x:c r="C180" s="11" t="str">
+        <x:v>Research toolkit + agent/MCP integration</x:v>
+      </x:c>
+      <x:c r="D180" s="11" t="str">
+        <x:v>Clinical Data &amp; Interoperability</x:v>
+      </x:c>
+      <x:c r="E180" s="11" t="str">
+        <x:v>Clinical-research toolkit for querying structured records and notes in supported research datasets.</x:v>
+      </x:c>
+      <x:c r="F180" s="11" t="str">
+        <x:v>Clinical Data | Research toolkit + agent/MCP integration</x:v>
+      </x:c>
+      <x:c r="G180" s="11" t="str">
+        <x:v>Clinical Data &amp; Interoperability | Source inspection and research preparation</x:v>
+      </x:c>
+      <x:c r="H180" s="11" t="str">
+        <x:v>Explore MIMIC, eICU or configured custom data | Use Python and agent workflows for tabular and note-based analyses</x:v>
+      </x:c>
+      <x:c r="I180" s="11" t="str">
+        <x:v>Dataset licenses and access approvals apply separately. Review generated queries and code, note handling and cohort definitions; results are not clinically validated.</x:v>
+      </x:c>
+      <x:c r="J180" s="11" t="str">
+        <x:v>Static source and documentation reviewed</x:v>
+      </x:c>
+      <x:c r="K180" s="11" t="str">
+        <x:v>Canonical repository metadata reviewed at commit 6ed55907679157e3dff46e99da487bb969c04a9c</x:v>
+      </x:c>
+      <x:c r="L180" s="11" t="str">
+        <x:v>https://github.com/hannesill/m4/blob/6ed55907679157e3dff46e99da487bb969c04a9c/README.md | https://github.com/hannesill/m4/blob/6ed55907679157e3dff46e99da487bb969c04a9c/pyproject.toml | https://github.com/hannesill/m4/blob/6ed55907679157e3dff46e99da487bb969c04a9c/benchmark/tasks/apsiii/mimic-apsiii-24h-raw/skills-decoy/sofa-score/SKILL.md | https://github.com/hannesill/m4/blob/6ed55907679157e3dff46e99da487bb969c04a9c/benchmark/tasks/apsiii/mimic-apsiii-24h-raw/skills-rawsql/mimic-apsiii-24h-raw/SKILL.md | https://github.com/hannesill/m4/blob/6ed55907679157e3dff46e99da487bb969c04a9c/benchmark/tasks/apsiii/mimic-apsiii-24h-raw/skills/apsiii-score/SKILL.md</x:v>
+      </x:c>
+      <x:c r="M180" s="11" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N180" s="11" t="str">
+        <x:v>hannesill</x:v>
+      </x:c>
+      <x:c r="O180" s="11" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P180" s="11" t="str">
+        <x:v>See pinned project manifest and setup documentation</x:v>
+      </x:c>
+      <x:c r="Q180" s="11" t="str">
+        <x:v>See pinned setup; varies by component</x:v>
+      </x:c>
+      <x:c r="R180" s="11" t="str">
+        <x:v>See capability and limitation fields; no runtime actions performed</x:v>
+      </x:c>
+      <x:c r="S180" s="11" t="str">
+        <x:v>See pinned project setup; external data access may require credentials.</x:v>
+      </x:c>
+      <x:c r="T180" s="14" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+      <x:c r="U180" s="14" t="n">
+        <x:v>46231.72597222222</x:v>
+      </x:c>
+      <x:c r="V180" s="11" t="n">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="W180" s="11" t="str">
+        <x:v>https://github.com/hannesill/m4</x:v>
+      </x:c>
+      <x:c r="X180" s="11" t="str">
+        <x:v>https://github.com/hannesill/m4</x:v>
+      </x:c>
+      <x:c r="Y180" s="11" t="str">
+        <x:v>https://github.com/hannesill/m4/blob/6ed55907679157e3dff46e99da487bb969c04a9c/README.md | https://github.com/hannesill/m4/blob/6ed55907679157e3dff46e99da487bb969c04a9c/pyproject.toml | https://github.com/hannesill/m4/blob/6ed55907679157e3dff46e99da487bb969c04a9c/benchmark/tasks/apsiii/mimic-apsiii-24h-raw/skills-decoy/sofa-score/SKILL.md | https://github.com/hannesill/m4/blob/6ed55907679157e3dff46e99da487bb969c04a9c/benchmark/tasks/apsiii/mimic-apsiii-24h-raw/skills-rawsql/mimic-apsiii-24h-raw/SKILL.md | https://github.com/hannesill/m4/blob/6ed55907679157e3dff46e99da487bb969c04a9c/benchmark/tasks/apsiii/mimic-apsiii-24h-raw/skills/apsiii-score/SKILL.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="181" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A181" s="11" t="str">
+        <x:v>RWE-0267</x:v>
+      </x:c>
+      <x:c r="B181" s="11" t="str">
+        <x:v>Trends MCP</x:v>
+      </x:c>
+      <x:c r="C181" s="11" t="str">
+        <x:v>MCP server</x:v>
+      </x:c>
+      <x:c r="D181" s="11" t="str">
+        <x:v>Literature &amp; Evidence Synthesis</x:v>
+      </x:c>
+      <x:c r="E181" s="11" t="str">
+        <x:v>Configurable trend-source aggregator with PubMed and FDA device-source connectors.</x:v>
+      </x:c>
+      <x:c r="F181" s="11" t="str">
+        <x:v>Literature | MCP server</x:v>
+      </x:c>
+      <x:c r="G181" s="11" t="str">
+        <x:v>Literature &amp; Evidence Synthesis | Source inspection and research preparation</x:v>
+      </x:c>
+      <x:c r="H181" s="11" t="str">
+        <x:v>Retrieve PubMed abstracts and supported FDA device records | Configure source definitions for ongoing evidence discovery</x:v>
+      </x:c>
+      <x:c r="I181" s="11" t="str">
+        <x:v>Only biomedical source connectors are in scope here. Coverage is not an exhaustive review; configuration tools write local settings and may require restart.</x:v>
+      </x:c>
+      <x:c r="J181" s="11" t="str">
+        <x:v>Static source and documentation reviewed</x:v>
+      </x:c>
+      <x:c r="K181" s="11" t="str">
+        <x:v>Canonical repository metadata reviewed at commit de0d00f995e19cc3d2486870f85ca067bc5679ce</x:v>
+      </x:c>
+      <x:c r="L181" s="11" t="str">
+        <x:v>https://github.com/salwks/mcp-techTrend/blob/de0d00f995e19cc3d2486870f85ca067bc5679ce/README.md | https://github.com/salwks/mcp-techTrend/blob/de0d00f995e19cc3d2486870f85ca067bc5679ce/pyproject.toml</x:v>
+      </x:c>
+      <x:c r="M181" s="11" t="str">
+        <x:v>Not independently runtime tested by registry</x:v>
+      </x:c>
+      <x:c r="N181" s="11" t="str">
+        <x:v>salwks</x:v>
+      </x:c>
+      <x:c r="O181" s="11" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P181" s="11" t="str">
+        <x:v>See pinned project manifest and setup documentation</x:v>
+      </x:c>
+      <x:c r="Q181" s="11" t="str">
+        <x:v>See pinned setup; varies by component</x:v>
+      </x:c>
+      <x:c r="R181" s="11" t="str">
+        <x:v>See capability and limitation fields; no runtime actions performed</x:v>
+      </x:c>
+      <x:c r="S181" s="11" t="str">
+        <x:v>See pinned project setup; external data access may require credentials.</x:v>
+      </x:c>
+      <x:c r="T181" s="14" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+      <x:c r="U181" s="14" t="n">
+        <x:v>46162.95627314815</x:v>
+      </x:c>
+      <x:c r="V181" s="11" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="W181" s="11" t="str">
+        <x:v>https://github.com/salwks/mcp-techTrend</x:v>
+      </x:c>
+      <x:c r="X181" s="11" t="str">
+        <x:v>https://github.com/salwks/mcp-techTrend</x:v>
+      </x:c>
+      <x:c r="Y181" s="11" t="str">
+        <x:v>https://github.com/salwks/mcp-techTrend/blob/de0d00f995e19cc3d2486870f85ca067bc5679ce/README.md | https://github.com/salwks/mcp-techTrend/blob/de0d00f995e19cc3d2486870f85ca067bc5679ce/pyproject.toml</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:Y1"/>
@@ -10685,7 +14150,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a435f362f484d89"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5678fff3a6d94d17"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>